<commit_message>
Actualizar dashboard Oferta Zitron 2026 2026-06-13 15:49 UTC
</commit_message>
<xml_diff>
--- a/data_ofertas/Oferta Zitron 2026.xlsx
+++ b/data_ofertas/Oferta Zitron 2026.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4325" uniqueCount="575">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4370" uniqueCount="579">
   <si>
     <t>Oferta Zitron 2026</t>
   </si>
@@ -1737,6 +1737,18 @@
   </si>
   <si>
     <t>1215659696585477</t>
+  </si>
+  <si>
+    <t>1215684129710831</t>
+  </si>
+  <si>
+    <t>1092-18-PE</t>
+  </si>
+  <si>
+    <t>1215684129710848</t>
+  </si>
+  <si>
+    <t>1215689131135204</t>
   </si>
 </sst>
 </file>
@@ -2260,7 +2272,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Y267"/>
+  <dimension ref="A1:Y270"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10.4" customWidth="1"/>
@@ -3025,9 +3037,11 @@
       <c r="B13" s="11">
         <v>46146.560996562504</v>
       </c>
-      <c r="C13" s="12"/>
+      <c r="C13" s="11">
+        <v>46186.6466966088</v>
+      </c>
       <c r="D13" s="11">
-        <v>46180.57950337963</v>
+        <v>46186.64695519676</v>
       </c>
       <c r="E13" s="12" t="s">
         <v>40</v>
@@ -3076,7 +3090,9 @@
       <c r="U13" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="V13" s="12"/>
+      <c r="V13" s="11">
+        <v>46160</v>
+      </c>
       <c r="W13" s="9" t="s">
         <v>66</v>
       </c>
@@ -3092,9 +3108,11 @@
       <c r="B14" s="5">
         <v>46146.56100443287</v>
       </c>
-      <c r="C14" s="6"/>
+      <c r="C14" s="5">
+        <v>46186.64672280093</v>
+      </c>
       <c r="D14" s="5">
-        <v>46180.57952234954</v>
+        <v>46186.64719125</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>28</v>
@@ -3143,7 +3161,9 @@
       <c r="U14" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="V14" s="6"/>
+      <c r="V14" s="5">
+        <v>46160</v>
+      </c>
       <c r="W14" s="9" t="s">
         <v>66</v>
       </c>
@@ -3159,9 +3179,11 @@
       <c r="B15" s="11">
         <v>46146.56101951389</v>
       </c>
-      <c r="C15" s="12"/>
+      <c r="C15" s="11">
+        <v>46186.646759930554</v>
+      </c>
       <c r="D15" s="11">
-        <v>46162.83719186342</v>
+        <v>46186.64728831018</v>
       </c>
       <c r="E15" s="12" t="s">
         <v>33</v>
@@ -3210,7 +3232,9 @@
       <c r="U15" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="V15" s="12"/>
+      <c r="V15" s="11">
+        <v>46160</v>
+      </c>
       <c r="W15" s="9" t="s">
         <v>66</v>
       </c>
@@ -7110,7 +7134,7 @@
         <v>46146.613911712964</v>
       </c>
       <c r="D70" s="5">
-        <v>46178.89901518519</v>
+        <v>46186.64821828704</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>40</v>
@@ -7157,7 +7181,9 @@
       <c r="U70" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="V70" s="6"/>
+      <c r="V70" s="5">
+        <v>46141</v>
+      </c>
       <c r="W70" s="9" t="s">
         <v>190</v>
       </c>
@@ -7177,7 +7203,7 @@
         <v>46146.61393603009</v>
       </c>
       <c r="D71" s="11">
-        <v>46157.5672796875</v>
+        <v>46186.648291631944</v>
       </c>
       <c r="E71" s="12" t="s">
         <v>83</v>
@@ -7224,7 +7250,9 @@
       <c r="U71" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="V71" s="12"/>
+      <c r="V71" s="11">
+        <v>46141</v>
+      </c>
       <c r="W71" s="9" t="s">
         <v>190</v>
       </c>
@@ -7244,7 +7272,7 @@
         <v>46146.61397960648</v>
       </c>
       <c r="D72" s="5">
-        <v>46157.56734009259</v>
+        <v>46186.648366354166</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>153</v>
@@ -7291,7 +7319,9 @@
       <c r="U72" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="V72" s="6"/>
+      <c r="V72" s="5">
+        <v>46141</v>
+      </c>
       <c r="W72" s="9" t="s">
         <v>190</v>
       </c>
@@ -9039,7 +9069,7 @@
         <v>46164.56628622685</v>
       </c>
       <c r="D97" s="11">
-        <v>46185.894776562505</v>
+        <v>46186.64979134259</v>
       </c>
       <c r="E97" s="12" t="s">
         <v>40</v>
@@ -9055,7 +9085,7 @@
       </c>
       <c r="I97" s="12"/>
       <c r="J97" s="11">
-        <v>46162</v>
+        <v>46142</v>
       </c>
       <c r="K97" s="12" t="s">
         <v>32</v>
@@ -9090,7 +9120,9 @@
       <c r="U97" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="V97" s="12"/>
+      <c r="V97" s="11">
+        <v>46168</v>
+      </c>
       <c r="W97" s="9" t="s">
         <v>242</v>
       </c>
@@ -9110,7 +9142,7 @@
         <v>46170.78799702546</v>
       </c>
       <c r="D98" s="5">
-        <v>46185.89480037037</v>
+        <v>46186.64979221065</v>
       </c>
       <c r="E98" s="6" t="s">
         <v>83</v>
@@ -9126,7 +9158,7 @@
       </c>
       <c r="I98" s="6"/>
       <c r="J98" s="5">
-        <v>46170</v>
+        <v>46142</v>
       </c>
       <c r="K98" s="6" t="s">
         <v>32</v>
@@ -9161,7 +9193,9 @@
       <c r="U98" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="V98" s="6"/>
+      <c r="V98" s="5">
+        <v>46168</v>
+      </c>
       <c r="W98" s="9" t="s">
         <v>242</v>
       </c>
@@ -9181,7 +9215,7 @@
         <v>46182.68615517361</v>
       </c>
       <c r="D99" s="11">
-        <v>46182.6862833912</v>
+        <v>46186.64979300926</v>
       </c>
       <c r="E99" s="12" t="s">
         <v>153</v>
@@ -9195,11 +9229,9 @@
       <c r="H99" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="I99" s="11">
-        <v>46182</v>
-      </c>
+      <c r="I99" s="12"/>
       <c r="J99" s="11">
-        <v>46182</v>
+        <v>46142</v>
       </c>
       <c r="K99" s="12" t="s">
         <v>32</v>
@@ -9234,7 +9266,9 @@
       <c r="U99" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="V99" s="12"/>
+      <c r="V99" s="11">
+        <v>46168</v>
+      </c>
       <c r="W99" s="9" t="s">
         <v>242</v>
       </c>
@@ -12608,7 +12642,7 @@
         <v>46171.78756511574</v>
       </c>
       <c r="D148" s="5">
-        <v>46171.78757349537</v>
+        <v>46186.649173530095</v>
       </c>
       <c r="E148" s="6" t="s">
         <v>40</v>
@@ -12622,7 +12656,7 @@
       <c r="H148" s="6"/>
       <c r="I148" s="6"/>
       <c r="J148" s="5">
-        <v>46171</v>
+        <v>46168</v>
       </c>
       <c r="K148" s="6" t="s">
         <v>32</v>
@@ -12657,7 +12691,9 @@
       <c r="U148" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="V148" s="6"/>
+      <c r="V148" s="5">
+        <v>46168</v>
+      </c>
       <c r="W148" s="9" t="s">
         <v>346</v>
       </c>
@@ -12677,7 +12713,7 @@
         <v>46171.78756517361</v>
       </c>
       <c r="D149" s="11">
-        <v>46171.78757356481</v>
+        <v>46186.64917430555</v>
       </c>
       <c r="E149" s="12" t="s">
         <v>83</v>
@@ -12691,7 +12727,7 @@
       <c r="H149" s="12"/>
       <c r="I149" s="12"/>
       <c r="J149" s="11">
-        <v>46171</v>
+        <v>46168</v>
       </c>
       <c r="K149" s="12" t="s">
         <v>32</v>
@@ -12726,7 +12762,9 @@
       <c r="U149" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="V149" s="12"/>
+      <c r="V149" s="11">
+        <v>46168</v>
+      </c>
       <c r="W149" s="9" t="s">
         <v>346</v>
       </c>
@@ -12746,7 +12784,7 @@
         <v>46171.78756541667</v>
       </c>
       <c r="D150" s="5">
-        <v>46171.78757350694</v>
+        <v>46186.649175081024</v>
       </c>
       <c r="E150" s="6" t="s">
         <v>153</v>
@@ -12760,7 +12798,7 @@
       <c r="H150" s="6"/>
       <c r="I150" s="6"/>
       <c r="J150" s="5">
-        <v>46171</v>
+        <v>46168</v>
       </c>
       <c r="K150" s="6" t="s">
         <v>32</v>
@@ -12795,7 +12833,9 @@
       <c r="U150" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="V150" s="6"/>
+      <c r="V150" s="5">
+        <v>46168</v>
+      </c>
       <c r="W150" s="9" t="s">
         <v>346</v>
       </c>
@@ -18549,9 +18589,11 @@
       <c r="B233" s="11">
         <v>46174.78294421296</v>
       </c>
-      <c r="C233" s="12"/>
+      <c r="C233" s="11">
+        <v>46186.65179798611</v>
+      </c>
       <c r="D233" s="11">
-        <v>46185.57789545139</v>
+        <v>46186.65194880787</v>
       </c>
       <c r="E233" s="12" t="s">
         <v>83</v>
@@ -18600,12 +18642,14 @@
       <c r="U233" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="V233" s="12"/>
+      <c r="V233" s="11">
+        <v>46177</v>
+      </c>
       <c r="W233" s="9" t="s">
         <v>508</v>
       </c>
       <c r="X233" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y233" s="12"/>
     </row>
@@ -18616,9 +18660,11 @@
       <c r="B234" s="5">
         <v>46174.782957372685</v>
       </c>
-      <c r="C234" s="6"/>
+      <c r="C234" s="5">
+        <v>46186.65184641204</v>
+      </c>
       <c r="D234" s="5">
-        <v>46185.57790773148</v>
+        <v>46186.65194938658</v>
       </c>
       <c r="E234" s="6" t="s">
         <v>153</v>
@@ -18667,12 +18713,14 @@
       <c r="U234" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="V234" s="6"/>
+      <c r="V234" s="5">
+        <v>46177</v>
+      </c>
       <c r="W234" s="9" t="s">
         <v>508</v>
       </c>
       <c r="X234" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y234" s="6"/>
     </row>
@@ -18683,9 +18731,11 @@
       <c r="B235" s="11">
         <v>46175.62894534723</v>
       </c>
-      <c r="C235" s="12"/>
+      <c r="C235" s="11">
+        <v>46186.65099351852</v>
+      </c>
       <c r="D235" s="11">
-        <v>46175.63113940972</v>
+        <v>46186.65119246527</v>
       </c>
       <c r="E235" s="12" t="s">
         <v>40</v>
@@ -18734,12 +18784,14 @@
       <c r="U235" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="V235" s="12"/>
+      <c r="V235" s="11">
+        <v>46182</v>
+      </c>
       <c r="W235" s="9" t="s">
         <v>514</v>
       </c>
       <c r="X235" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y235" s="12"/>
     </row>
@@ -18821,9 +18873,11 @@
       <c r="B237" s="11">
         <v>46175.62896625</v>
       </c>
-      <c r="C237" s="12"/>
+      <c r="C237" s="11">
+        <v>46186.65103758102</v>
+      </c>
       <c r="D237" s="11">
-        <v>46185.56118189815</v>
+        <v>46186.6511930787</v>
       </c>
       <c r="E237" s="12" t="s">
         <v>153</v>
@@ -18872,12 +18926,14 @@
       <c r="U237" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="V237" s="12"/>
+      <c r="V237" s="11">
+        <v>46182</v>
+      </c>
       <c r="W237" s="9" t="s">
         <v>514</v>
       </c>
       <c r="X237" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y237" s="12"/>
     </row>
@@ -20896,6 +20952,219 @@
         <v>0</v>
       </c>
       <c r="Y267" s="12"/>
+    </row>
+    <row r="268" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A268" s="4" t="s">
+        <v>575</v>
+      </c>
+      <c r="B268" s="5">
+        <v>46186.654707650465</v>
+      </c>
+      <c r="C268" s="5">
+        <v>46186.656402152774</v>
+      </c>
+      <c r="D268" s="5">
+        <v>46186.65728032407</v>
+      </c>
+      <c r="E268" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F268" s="6" t="s">
+        <v>576</v>
+      </c>
+      <c r="G268" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H268" s="6"/>
+      <c r="I268" s="5">
+        <v>46155</v>
+      </c>
+      <c r="J268" s="5">
+        <v>46155</v>
+      </c>
+      <c r="K268" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="L268" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="M268" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N268" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="O268" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="P268" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q268" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="R268" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S268" s="6"/>
+      <c r="T268" s="6" t="s">
+        <v>576</v>
+      </c>
+      <c r="U268" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="V268" s="5">
+        <v>46157</v>
+      </c>
+      <c r="W268" s="9" t="s">
+        <v>576</v>
+      </c>
+      <c r="X268" s="6">
+        <v>1</v>
+      </c>
+      <c r="Y268" s="6"/>
+    </row>
+    <row r="269" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A269" s="10" t="s">
+        <v>577</v>
+      </c>
+      <c r="B269" s="11">
+        <v>46186.65471349537</v>
+      </c>
+      <c r="C269" s="11">
+        <v>46186.65640291666</v>
+      </c>
+      <c r="D269" s="11">
+        <v>46186.6572809375</v>
+      </c>
+      <c r="E269" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="F269" s="12" t="s">
+        <v>576</v>
+      </c>
+      <c r="G269" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="H269" s="12"/>
+      <c r="I269" s="11">
+        <v>46155</v>
+      </c>
+      <c r="J269" s="11">
+        <v>46155</v>
+      </c>
+      <c r="K269" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="L269" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="M269" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N269" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="O269" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="P269" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q269" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="R269" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S269" s="12"/>
+      <c r="T269" s="12" t="s">
+        <v>576</v>
+      </c>
+      <c r="U269" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="V269" s="11">
+        <v>46157</v>
+      </c>
+      <c r="W269" s="9" t="s">
+        <v>576</v>
+      </c>
+      <c r="X269" s="12">
+        <v>1</v>
+      </c>
+      <c r="Y269" s="12"/>
+    </row>
+    <row r="270" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A270" s="4" t="s">
+        <v>578</v>
+      </c>
+      <c r="B270" s="5">
+        <v>46186.654726875</v>
+      </c>
+      <c r="C270" s="5">
+        <v>46186.65640344907</v>
+      </c>
+      <c r="D270" s="5">
+        <v>46186.65728157407</v>
+      </c>
+      <c r="E270" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="F270" s="6" t="s">
+        <v>576</v>
+      </c>
+      <c r="G270" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H270" s="6"/>
+      <c r="I270" s="5">
+        <v>46155</v>
+      </c>
+      <c r="J270" s="5">
+        <v>46155</v>
+      </c>
+      <c r="K270" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="L270" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="M270" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N270" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="O270" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="P270" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q270" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="R270" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S270" s="6"/>
+      <c r="T270" s="6" t="s">
+        <v>576</v>
+      </c>
+      <c r="U270" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="V270" s="5">
+        <v>46157</v>
+      </c>
+      <c r="W270" s="9" t="s">
+        <v>576</v>
+      </c>
+      <c r="X270" s="6">
+        <v>1</v>
+      </c>
+      <c r="Y270" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Actualizar dashboard Oferta Zitron 2026 2026-06-13 16:15 UTC
</commit_message>
<xml_diff>
--- a/data_ofertas/Oferta Zitron 2026.xlsx
+++ b/data_ofertas/Oferta Zitron 2026.xlsx
@@ -12853,7 +12853,7 @@
       </c>
       <c r="C151" s="12"/>
       <c r="D151" s="11">
-        <v>46155.65660054398</v>
+        <v>46186.66231395833</v>
       </c>
       <c r="E151" s="12" t="s">
         <v>40</v>
@@ -12865,8 +12865,12 @@
         <v>32</v>
       </c>
       <c r="H151" s="12"/>
-      <c r="I151" s="12"/>
-      <c r="J151" s="12"/>
+      <c r="I151" s="11">
+        <v>46155</v>
+      </c>
+      <c r="J151" s="11">
+        <v>46155</v>
+      </c>
       <c r="K151" s="12" t="s">
         <v>32</v>
       </c>
@@ -12886,10 +12890,10 @@
         <v>153</v>
       </c>
       <c r="Q151" s="7" t="s">
-        <v>326</v>
+        <v>64</v>
       </c>
       <c r="R151" s="7" t="s">
-        <v>326</v>
+        <v>35</v>
       </c>
       <c r="S151" s="12" t="s">
         <v>351</v>
@@ -12918,7 +12922,7 @@
       </c>
       <c r="C152" s="6"/>
       <c r="D152" s="5">
-        <v>46155.6566144213</v>
+        <v>46186.66231451389</v>
       </c>
       <c r="E152" s="6" t="s">
         <v>83</v>
@@ -12930,8 +12934,12 @@
         <v>32</v>
       </c>
       <c r="H152" s="6"/>
-      <c r="I152" s="6"/>
-      <c r="J152" s="6"/>
+      <c r="I152" s="5">
+        <v>46155</v>
+      </c>
+      <c r="J152" s="5">
+        <v>46155</v>
+      </c>
       <c r="K152" s="6" t="s">
         <v>32</v>
       </c>
@@ -12951,10 +12959,10 @@
         <v>153</v>
       </c>
       <c r="Q152" s="7" t="s">
-        <v>326</v>
+        <v>64</v>
       </c>
       <c r="R152" s="7" t="s">
-        <v>326</v>
+        <v>35</v>
       </c>
       <c r="S152" s="6" t="s">
         <v>351</v>
@@ -12983,7 +12991,7 @@
       </c>
       <c r="C153" s="12"/>
       <c r="D153" s="11">
-        <v>46155.656629861114</v>
+        <v>46186.66231509259</v>
       </c>
       <c r="E153" s="12" t="s">
         <v>153</v>
@@ -12995,8 +13003,12 @@
         <v>32</v>
       </c>
       <c r="H153" s="12"/>
-      <c r="I153" s="12"/>
-      <c r="J153" s="12"/>
+      <c r="I153" s="11">
+        <v>46155</v>
+      </c>
+      <c r="J153" s="11">
+        <v>46155</v>
+      </c>
       <c r="K153" s="12" t="s">
         <v>32</v>
       </c>
@@ -13016,10 +13028,10 @@
         <v>32</v>
       </c>
       <c r="Q153" s="7" t="s">
-        <v>326</v>
+        <v>64</v>
       </c>
       <c r="R153" s="7" t="s">
-        <v>326</v>
+        <v>35</v>
       </c>
       <c r="S153" s="12" t="s">
         <v>351</v>

</xml_diff>

<commit_message>
Actualizar dashboard Oferta Zitron 2026 2026-06-15 20:08 UTC
</commit_message>
<xml_diff>
--- a/data_ofertas/Oferta Zitron 2026.xlsx
+++ b/data_ofertas/Oferta Zitron 2026.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4370" uniqueCount="579">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4379" uniqueCount="579">
   <si>
     <t>Oferta Zitron 2026</t>
   </si>
@@ -733,7 +733,7 @@
     <t>1214565160385301</t>
   </si>
   <si>
-    <t>25cl0054-Visita Minera Arqueros</t>
+    <t>26cl0054-Visita Minera Arqueros</t>
   </si>
   <si>
     <t>Minera Arqueros</t>
@@ -13934,9 +13934,11 @@
       <c r="B166" s="5">
         <v>46155.665985300926</v>
       </c>
-      <c r="C166" s="6"/>
+      <c r="C166" s="5">
+        <v>46188.61507181713</v>
+      </c>
       <c r="D166" s="5">
-        <v>46160.72927788194</v>
+        <v>46188.61530665509</v>
       </c>
       <c r="E166" s="6" t="s">
         <v>40</v>
@@ -13987,12 +13989,14 @@
       <c r="U166" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="V166" s="6"/>
+      <c r="V166" s="5">
+        <v>46188</v>
+      </c>
       <c r="W166" s="9" t="s">
         <v>381</v>
       </c>
       <c r="X166" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y166" s="6"/>
     </row>
@@ -14076,9 +14080,11 @@
       <c r="B168" s="5">
         <v>46155.6660016088</v>
       </c>
-      <c r="C168" s="6"/>
+      <c r="C168" s="5">
+        <v>46188.61519428241</v>
+      </c>
       <c r="D168" s="5">
-        <v>46178.7161899537</v>
+        <v>46188.61527435185</v>
       </c>
       <c r="E168" s="6" t="s">
         <v>153</v>
@@ -14129,12 +14135,14 @@
       <c r="U168" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="V168" s="6"/>
+      <c r="V168" s="5">
+        <v>46188</v>
+      </c>
       <c r="W168" s="9" t="s">
         <v>381</v>
       </c>
       <c r="X168" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y168" s="6"/>
     </row>
@@ -15188,7 +15196,7 @@
       </c>
       <c r="C184" s="6"/>
       <c r="D184" s="5">
-        <v>46166.90066099537</v>
+        <v>46188.70112761574</v>
       </c>
       <c r="E184" s="6" t="s">
         <v>40</v>
@@ -15197,9 +15205,11 @@
         <v>415</v>
       </c>
       <c r="G184" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H184" s="6"/>
+        <v>78</v>
+      </c>
+      <c r="H184" s="6" t="s">
+        <v>79</v>
+      </c>
       <c r="I184" s="6"/>
       <c r="J184" s="5">
         <v>46162</v>
@@ -15255,7 +15265,7 @@
       </c>
       <c r="C185" s="12"/>
       <c r="D185" s="11">
-        <v>46166.90069736111</v>
+        <v>46188.701169884254</v>
       </c>
       <c r="E185" s="12" t="s">
         <v>83</v>
@@ -15264,9 +15274,11 @@
         <v>415</v>
       </c>
       <c r="G185" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H185" s="12"/>
+        <v>30</v>
+      </c>
+      <c r="H185" s="12" t="s">
+        <v>31</v>
+      </c>
       <c r="I185" s="12"/>
       <c r="J185" s="11">
         <v>46162</v>
@@ -15322,7 +15334,7 @@
       </c>
       <c r="C186" s="6"/>
       <c r="D186" s="5">
-        <v>46166.90073765046</v>
+        <v>46188.70119445602</v>
       </c>
       <c r="E186" s="6" t="s">
         <v>153</v>
@@ -15331,9 +15343,11 @@
         <v>415</v>
       </c>
       <c r="G186" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H186" s="6"/>
+        <v>44</v>
+      </c>
+      <c r="H186" s="6" t="s">
+        <v>45</v>
+      </c>
       <c r="I186" s="6"/>
       <c r="J186" s="5">
         <v>46162</v>
@@ -18605,7 +18619,7 @@
         <v>46186.65179798611</v>
       </c>
       <c r="D233" s="11">
-        <v>46186.65194880787</v>
+        <v>46188.61648292824</v>
       </c>
       <c r="E233" s="12" t="s">
         <v>83</v>
@@ -18655,7 +18669,7 @@
         <v>38</v>
       </c>
       <c r="V233" s="11">
-        <v>46177</v>
+        <v>46185</v>
       </c>
       <c r="W233" s="9" t="s">
         <v>508</v>
@@ -19171,7 +19185,7 @@
       </c>
       <c r="C241" s="12"/>
       <c r="D241" s="11">
-        <v>46177.562608761575</v>
+        <v>46188.70072540509</v>
       </c>
       <c r="E241" s="12" t="s">
         <v>40</v>
@@ -19180,9 +19194,11 @@
         <v>526</v>
       </c>
       <c r="G241" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H241" s="12"/>
+        <v>78</v>
+      </c>
+      <c r="H241" s="12" t="s">
+        <v>79</v>
+      </c>
       <c r="I241" s="12"/>
       <c r="J241" s="11">
         <v>46176</v>
@@ -19240,7 +19256,7 @@
         <v>46185.59227212963</v>
       </c>
       <c r="D242" s="5">
-        <v>46185.59248471065</v>
+        <v>46188.700642615746</v>
       </c>
       <c r="E242" s="6" t="s">
         <v>83</v>
@@ -19249,9 +19265,11 @@
         <v>526</v>
       </c>
       <c r="G242" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H242" s="6"/>
+        <v>30</v>
+      </c>
+      <c r="H242" s="6" t="s">
+        <v>31</v>
+      </c>
       <c r="I242" s="6"/>
       <c r="J242" s="5">
         <v>46176</v>
@@ -19309,7 +19327,7 @@
       </c>
       <c r="C243" s="12"/>
       <c r="D243" s="11">
-        <v>46185.592278958335</v>
+        <v>46188.700669502316</v>
       </c>
       <c r="E243" s="12" t="s">
         <v>153</v>
@@ -19318,9 +19336,11 @@
         <v>526</v>
       </c>
       <c r="G243" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H243" s="12"/>
+        <v>44</v>
+      </c>
+      <c r="H243" s="12" t="s">
+        <v>45</v>
+      </c>
       <c r="I243" s="12"/>
       <c r="J243" s="11">
         <v>46176</v>
@@ -20578,7 +20598,7 @@
       </c>
       <c r="C262" s="6"/>
       <c r="D262" s="5">
-        <v>46185.56833203704</v>
+        <v>46188.70039008102</v>
       </c>
       <c r="E262" s="6" t="s">
         <v>40</v>
@@ -20587,9 +20607,11 @@
         <v>565</v>
       </c>
       <c r="G262" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H262" s="6"/>
+        <v>41</v>
+      </c>
+      <c r="H262" s="6" t="s">
+        <v>42</v>
+      </c>
       <c r="I262" s="6"/>
       <c r="J262" s="5">
         <v>46183</v>
@@ -20643,9 +20665,11 @@
       <c r="B263" s="11">
         <v>46185.56558616898</v>
       </c>
-      <c r="C263" s="12"/>
+      <c r="C263" s="11">
+        <v>46188.61555454861</v>
+      </c>
       <c r="D263" s="11">
-        <v>46185.56833222222</v>
+        <v>46188.6157578125</v>
       </c>
       <c r="E263" s="12" t="s">
         <v>83</v>
@@ -20654,9 +20678,11 @@
         <v>565</v>
       </c>
       <c r="G263" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H263" s="12"/>
+        <v>30</v>
+      </c>
+      <c r="H263" s="12" t="s">
+        <v>31</v>
+      </c>
       <c r="I263" s="12"/>
       <c r="J263" s="11">
         <v>46183</v>
@@ -20694,12 +20720,14 @@
       <c r="U263" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="V263" s="12"/>
+      <c r="V263" s="11">
+        <v>46185</v>
+      </c>
       <c r="W263" s="9" t="s">
         <v>567</v>
       </c>
       <c r="X263" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y263" s="12"/>
     </row>
@@ -20712,7 +20740,7 @@
       </c>
       <c r="C264" s="6"/>
       <c r="D264" s="5">
-        <v>46185.568332372684</v>
+        <v>46188.61571253472</v>
       </c>
       <c r="E264" s="6" t="s">
         <v>153</v>
@@ -20721,9 +20749,11 @@
         <v>565</v>
       </c>
       <c r="G264" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H264" s="6"/>
+        <v>44</v>
+      </c>
+      <c r="H264" s="6" t="s">
+        <v>45</v>
+      </c>
       <c r="I264" s="6"/>
       <c r="J264" s="5">
         <v>46183</v>

</xml_diff>

<commit_message>
Actualizar dashboard Oferta Zitron 2026 2026-06-15 21:36 UTC
</commit_message>
<xml_diff>
--- a/data_ofertas/Oferta Zitron 2026.xlsx
+++ b/data_ofertas/Oferta Zitron 2026.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4379" uniqueCount="579">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4427" uniqueCount="581">
   <si>
     <t>Oferta Zitron 2026</t>
   </si>
@@ -1497,6 +1497,12 @@
   </si>
   <si>
     <t>26VE0004 -Asistencia ventilador 34204 - 50012392</t>
+  </si>
+  <si>
+    <t>Sergio de la Fuente</t>
+  </si>
+  <si>
+    <t>sergio.delafuente@zitron.com</t>
   </si>
   <si>
     <t>Zitron España</t>
@@ -10146,7 +10152,7 @@
         <v>46150.17873741898</v>
       </c>
       <c r="D112" s="5">
-        <v>46150.179026365746</v>
+        <v>46188.849060532404</v>
       </c>
       <c r="E112" s="6" t="s">
         <v>40</v>
@@ -10155,9 +10161,11 @@
         <v>270</v>
       </c>
       <c r="G112" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H112" s="6"/>
+        <v>41</v>
+      </c>
+      <c r="H112" s="6" t="s">
+        <v>42</v>
+      </c>
       <c r="I112" s="6"/>
       <c r="J112" s="5">
         <v>46140</v>
@@ -10217,7 +10225,7 @@
         <v>46150.17874983796</v>
       </c>
       <c r="D113" s="11">
-        <v>46150.179027199076</v>
+        <v>46188.84909600695</v>
       </c>
       <c r="E113" s="12" t="s">
         <v>83</v>
@@ -10226,9 +10234,11 @@
         <v>270</v>
       </c>
       <c r="G113" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H113" s="12"/>
+        <v>30</v>
+      </c>
+      <c r="H113" s="12" t="s">
+        <v>31</v>
+      </c>
       <c r="I113" s="12"/>
       <c r="J113" s="11">
         <v>46140</v>
@@ -10288,7 +10298,7 @@
         <v>46150.17878524306</v>
       </c>
       <c r="D114" s="5">
-        <v>46150.17902804398</v>
+        <v>46188.84912655092</v>
       </c>
       <c r="E114" s="6" t="s">
         <v>153</v>
@@ -10297,9 +10307,11 @@
         <v>270</v>
       </c>
       <c r="G114" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H114" s="6"/>
+        <v>44</v>
+      </c>
+      <c r="H114" s="6" t="s">
+        <v>45</v>
+      </c>
       <c r="I114" s="6"/>
       <c r="J114" s="5">
         <v>46140</v>
@@ -12232,7 +12244,7 @@
       </c>
       <c r="C142" s="6"/>
       <c r="D142" s="5">
-        <v>46154.76732783565</v>
+        <v>46188.84494414352</v>
       </c>
       <c r="E142" s="6" t="s">
         <v>40</v>
@@ -12241,9 +12253,11 @@
         <v>331</v>
       </c>
       <c r="G142" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H142" s="6"/>
+        <v>30</v>
+      </c>
+      <c r="H142" s="6" t="s">
+        <v>31</v>
+      </c>
       <c r="I142" s="6"/>
       <c r="J142" s="5">
         <v>46150</v>
@@ -12299,7 +12313,7 @@
       </c>
       <c r="C143" s="12"/>
       <c r="D143" s="11">
-        <v>46154.767328437505</v>
+        <v>46188.84467689815</v>
       </c>
       <c r="E143" s="12" t="s">
         <v>83</v>
@@ -12308,9 +12322,11 @@
         <v>331</v>
       </c>
       <c r="G143" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H143" s="12"/>
+        <v>30</v>
+      </c>
+      <c r="H143" s="12" t="s">
+        <v>31</v>
+      </c>
       <c r="I143" s="12"/>
       <c r="J143" s="11">
         <v>46150</v>
@@ -12366,7 +12382,7 @@
       </c>
       <c r="C144" s="6"/>
       <c r="D144" s="5">
-        <v>46154.76732908565</v>
+        <v>46188.84471421296</v>
       </c>
       <c r="E144" s="6" t="s">
         <v>153</v>
@@ -12375,9 +12391,11 @@
         <v>331</v>
       </c>
       <c r="G144" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H144" s="6"/>
+        <v>44</v>
+      </c>
+      <c r="H144" s="6" t="s">
+        <v>45</v>
+      </c>
       <c r="I144" s="6"/>
       <c r="J144" s="5">
         <v>46150</v>
@@ -12853,7 +12871,7 @@
       </c>
       <c r="C151" s="12"/>
       <c r="D151" s="11">
-        <v>46186.66231395833</v>
+        <v>46188.84417585648</v>
       </c>
       <c r="E151" s="12" t="s">
         <v>40</v>
@@ -12862,9 +12880,11 @@
         <v>350</v>
       </c>
       <c r="G151" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H151" s="12"/>
+        <v>78</v>
+      </c>
+      <c r="H151" s="12" t="s">
+        <v>79</v>
+      </c>
       <c r="I151" s="11">
         <v>46155</v>
       </c>
@@ -12922,7 +12942,7 @@
       </c>
       <c r="C152" s="6"/>
       <c r="D152" s="5">
-        <v>46186.66231451389</v>
+        <v>46188.844253020834</v>
       </c>
       <c r="E152" s="6" t="s">
         <v>83</v>
@@ -12931,9 +12951,11 @@
         <v>350</v>
       </c>
       <c r="G152" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H152" s="6"/>
+        <v>30</v>
+      </c>
+      <c r="H152" s="6" t="s">
+        <v>31</v>
+      </c>
       <c r="I152" s="5">
         <v>46155</v>
       </c>
@@ -12991,7 +13013,7 @@
       </c>
       <c r="C153" s="12"/>
       <c r="D153" s="11">
-        <v>46186.66231509259</v>
+        <v>46188.844285625004</v>
       </c>
       <c r="E153" s="12" t="s">
         <v>153</v>
@@ -13000,9 +13022,11 @@
         <v>350</v>
       </c>
       <c r="G153" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H153" s="12"/>
+        <v>44</v>
+      </c>
+      <c r="H153" s="12" t="s">
+        <v>45</v>
+      </c>
       <c r="I153" s="11">
         <v>46155</v>
       </c>
@@ -14155,7 +14179,7 @@
       </c>
       <c r="C169" s="12"/>
       <c r="D169" s="11">
-        <v>46160.72499241898</v>
+        <v>46188.8468241088</v>
       </c>
       <c r="E169" s="12" t="s">
         <v>40</v>
@@ -14164,9 +14188,11 @@
         <v>385</v>
       </c>
       <c r="G169" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H169" s="12"/>
+        <v>30</v>
+      </c>
+      <c r="H169" s="12" t="s">
+        <v>31</v>
+      </c>
       <c r="I169" s="12"/>
       <c r="J169" s="11">
         <v>46129</v>
@@ -14222,7 +14248,7 @@
       </c>
       <c r="C170" s="6"/>
       <c r="D170" s="5">
-        <v>46155.84267037037</v>
+        <v>46188.84673715278</v>
       </c>
       <c r="E170" s="6" t="s">
         <v>83</v>
@@ -14231,9 +14257,11 @@
         <v>385</v>
       </c>
       <c r="G170" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H170" s="6"/>
+        <v>30</v>
+      </c>
+      <c r="H170" s="6" t="s">
+        <v>31</v>
+      </c>
       <c r="I170" s="6"/>
       <c r="J170" s="5">
         <v>46129</v>
@@ -14289,7 +14317,7 @@
       </c>
       <c r="C171" s="12"/>
       <c r="D171" s="11">
-        <v>46155.842629375</v>
+        <v>46188.84677059027</v>
       </c>
       <c r="E171" s="12" t="s">
         <v>153</v>
@@ -14298,9 +14326,11 @@
         <v>385</v>
       </c>
       <c r="G171" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H171" s="12"/>
+        <v>44</v>
+      </c>
+      <c r="H171" s="12" t="s">
+        <v>45</v>
+      </c>
       <c r="I171" s="12"/>
       <c r="J171" s="11">
         <v>46129</v>
@@ -14995,7 +15025,7 @@
       </c>
       <c r="C181" s="12"/>
       <c r="D181" s="11">
-        <v>46162.835669733795</v>
+        <v>46188.84522106481</v>
       </c>
       <c r="E181" s="12" t="s">
         <v>40</v>
@@ -15004,9 +15034,11 @@
         <v>409</v>
       </c>
       <c r="G181" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H181" s="12"/>
+        <v>41</v>
+      </c>
+      <c r="H181" s="12" t="s">
+        <v>42</v>
+      </c>
       <c r="I181" s="12"/>
       <c r="J181" s="11">
         <v>46162</v>
@@ -15062,7 +15094,7 @@
       </c>
       <c r="C182" s="6"/>
       <c r="D182" s="5">
-        <v>46162.83567032407</v>
+        <v>46188.845266296295</v>
       </c>
       <c r="E182" s="6" t="s">
         <v>83</v>
@@ -15071,9 +15103,11 @@
         <v>409</v>
       </c>
       <c r="G182" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H182" s="6"/>
+        <v>30</v>
+      </c>
+      <c r="H182" s="6" t="s">
+        <v>31</v>
+      </c>
       <c r="I182" s="6"/>
       <c r="J182" s="5">
         <v>46162</v>
@@ -15129,7 +15163,7 @@
       </c>
       <c r="C183" s="12"/>
       <c r="D183" s="11">
-        <v>46162.8356709375</v>
+        <v>46188.84529938658</v>
       </c>
       <c r="E183" s="12" t="s">
         <v>153</v>
@@ -15138,9 +15172,11 @@
         <v>409</v>
       </c>
       <c r="G183" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H183" s="12"/>
+        <v>44</v>
+      </c>
+      <c r="H183" s="12" t="s">
+        <v>45</v>
+      </c>
       <c r="I183" s="12"/>
       <c r="J183" s="11">
         <v>46162</v>
@@ -15405,7 +15441,7 @@
         <v>46164.565793182875</v>
       </c>
       <c r="D187" s="11">
-        <v>46164.56591123843</v>
+        <v>46188.84848480324</v>
       </c>
       <c r="E187" s="12" t="s">
         <v>40</v>
@@ -15414,9 +15450,11 @@
         <v>420</v>
       </c>
       <c r="G187" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H187" s="12"/>
+        <v>41</v>
+      </c>
+      <c r="H187" s="12" t="s">
+        <v>42</v>
+      </c>
       <c r="I187" s="12"/>
       <c r="J187" s="11">
         <v>46162</v>
@@ -15476,7 +15514,7 @@
         <v>46167.702879675926</v>
       </c>
       <c r="D188" s="5">
-        <v>46167.70301597222</v>
+        <v>46188.84853929398</v>
       </c>
       <c r="E188" s="6" t="s">
         <v>83</v>
@@ -15485,9 +15523,11 @@
         <v>420</v>
       </c>
       <c r="G188" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H188" s="6"/>
+        <v>30</v>
+      </c>
+      <c r="H188" s="6" t="s">
+        <v>31</v>
+      </c>
       <c r="I188" s="6"/>
       <c r="J188" s="5">
         <v>46162</v>
@@ -15547,7 +15587,7 @@
         <v>46167.702957291665</v>
       </c>
       <c r="D189" s="11">
-        <v>46167.703045497685</v>
+        <v>46188.84858297453</v>
       </c>
       <c r="E189" s="12" t="s">
         <v>153</v>
@@ -15556,9 +15596,11 @@
         <v>420</v>
       </c>
       <c r="G189" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H189" s="12"/>
+        <v>44</v>
+      </c>
+      <c r="H189" s="12" t="s">
+        <v>45</v>
+      </c>
       <c r="I189" s="12"/>
       <c r="J189" s="11">
         <v>46162</v>
@@ -16446,7 +16488,7 @@
       </c>
       <c r="C202" s="6"/>
       <c r="D202" s="5">
-        <v>46168.68063155093</v>
+        <v>46188.8457128588</v>
       </c>
       <c r="E202" s="6" t="s">
         <v>40</v>
@@ -16455,9 +16497,11 @@
         <v>447</v>
       </c>
       <c r="G202" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H202" s="6"/>
+        <v>41</v>
+      </c>
+      <c r="H202" s="6" t="s">
+        <v>42</v>
+      </c>
       <c r="I202" s="6"/>
       <c r="J202" s="5">
         <v>46164</v>
@@ -16513,7 +16557,7 @@
       </c>
       <c r="C203" s="12"/>
       <c r="D203" s="11">
-        <v>46168.68066096064</v>
+        <v>46188.845783275465</v>
       </c>
       <c r="E203" s="12" t="s">
         <v>83</v>
@@ -16522,9 +16566,11 @@
         <v>447</v>
       </c>
       <c r="G203" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H203" s="12"/>
+        <v>30</v>
+      </c>
+      <c r="H203" s="12" t="s">
+        <v>31</v>
+      </c>
       <c r="I203" s="12"/>
       <c r="J203" s="11">
         <v>46164</v>
@@ -16580,7 +16626,7 @@
       </c>
       <c r="C204" s="6"/>
       <c r="D204" s="5">
-        <v>46168.680733518515</v>
+        <v>46188.845834340274</v>
       </c>
       <c r="E204" s="6" t="s">
         <v>153</v>
@@ -16589,9 +16635,11 @@
         <v>447</v>
       </c>
       <c r="G204" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H204" s="6"/>
+        <v>44</v>
+      </c>
+      <c r="H204" s="6" t="s">
+        <v>45</v>
+      </c>
       <c r="I204" s="6"/>
       <c r="J204" s="5">
         <v>46164</v>
@@ -16649,7 +16697,7 @@
         <v>46185.58664271991</v>
       </c>
       <c r="D205" s="11">
-        <v>46185.58712146991</v>
+        <v>46188.85060873843</v>
       </c>
       <c r="E205" s="12" t="s">
         <v>40</v>
@@ -16658,9 +16706,11 @@
         <v>453</v>
       </c>
       <c r="G205" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H205" s="12"/>
+        <v>78</v>
+      </c>
+      <c r="H205" s="12" t="s">
+        <v>79</v>
+      </c>
       <c r="I205" s="12"/>
       <c r="J205" s="11">
         <v>46168</v>
@@ -16720,7 +16770,7 @@
         <v>46185.58665894676</v>
       </c>
       <c r="D206" s="5">
-        <v>46185.58708894676</v>
+        <v>46188.85074409722</v>
       </c>
       <c r="E206" s="6" t="s">
         <v>83</v>
@@ -16729,9 +16779,11 @@
         <v>453</v>
       </c>
       <c r="G206" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H206" s="6"/>
+        <v>30</v>
+      </c>
+      <c r="H206" s="6" t="s">
+        <v>31</v>
+      </c>
       <c r="I206" s="6"/>
       <c r="J206" s="5">
         <v>46168</v>
@@ -16791,7 +16843,7 @@
         <v>46185.58670597222</v>
       </c>
       <c r="D207" s="11">
-        <v>46185.586936238426</v>
+        <v>46188.8507766088</v>
       </c>
       <c r="E207" s="12" t="s">
         <v>153</v>
@@ -16800,9 +16852,11 @@
         <v>453</v>
       </c>
       <c r="G207" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H207" s="12"/>
+        <v>44</v>
+      </c>
+      <c r="H207" s="12" t="s">
+        <v>45</v>
+      </c>
       <c r="I207" s="12"/>
       <c r="J207" s="11">
         <v>46168</v>
@@ -17511,7 +17565,7 @@
       </c>
       <c r="C217" s="12"/>
       <c r="D217" s="11">
-        <v>46171.54293408565</v>
+        <v>46188.84614569445</v>
       </c>
       <c r="E217" s="12" t="s">
         <v>40</v>
@@ -17520,9 +17574,11 @@
         <v>477</v>
       </c>
       <c r="G217" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H217" s="12"/>
+        <v>41</v>
+      </c>
+      <c r="H217" s="12" t="s">
+        <v>42</v>
+      </c>
       <c r="I217" s="11">
         <v>46171</v>
       </c>
@@ -17580,7 +17636,7 @@
       </c>
       <c r="C218" s="6"/>
       <c r="D218" s="5">
-        <v>46171.54293469907</v>
+        <v>46188.8461966551</v>
       </c>
       <c r="E218" s="6" t="s">
         <v>83</v>
@@ -17589,9 +17645,11 @@
         <v>477</v>
       </c>
       <c r="G218" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H218" s="6"/>
+        <v>30</v>
+      </c>
+      <c r="H218" s="6" t="s">
+        <v>31</v>
+      </c>
       <c r="I218" s="5">
         <v>46171</v>
       </c>
@@ -17649,7 +17707,7 @@
       </c>
       <c r="C219" s="12"/>
       <c r="D219" s="11">
-        <v>46171.542935324076</v>
+        <v>46188.84623487269</v>
       </c>
       <c r="E219" s="12" t="s">
         <v>153</v>
@@ -17658,9 +17716,11 @@
         <v>477</v>
       </c>
       <c r="G219" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H219" s="12"/>
+        <v>44</v>
+      </c>
+      <c r="H219" s="12" t="s">
+        <v>45</v>
+      </c>
       <c r="I219" s="11">
         <v>46171</v>
       </c>
@@ -17921,7 +17981,7 @@
         <v>46178.59328664352</v>
       </c>
       <c r="D223" s="11">
-        <v>46178.593406087966</v>
+        <v>46188.84813209491</v>
       </c>
       <c r="E223" s="12" t="s">
         <v>40</v>
@@ -17930,9 +17990,11 @@
         <v>488</v>
       </c>
       <c r="G223" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H223" s="12"/>
+        <v>78</v>
+      </c>
+      <c r="H223" s="12" t="s">
+        <v>79</v>
+      </c>
       <c r="I223" s="12"/>
       <c r="J223" s="11">
         <v>46171</v>
@@ -17992,7 +18054,7 @@
         <v>46177.54647826389</v>
       </c>
       <c r="D224" s="5">
-        <v>46177.54651876158</v>
+        <v>46188.848162696755</v>
       </c>
       <c r="E224" s="6" t="s">
         <v>83</v>
@@ -18001,9 +18063,11 @@
         <v>488</v>
       </c>
       <c r="G224" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H224" s="6"/>
+        <v>30</v>
+      </c>
+      <c r="H224" s="6" t="s">
+        <v>31</v>
+      </c>
       <c r="I224" s="6"/>
       <c r="J224" s="5">
         <v>46171</v>
@@ -18063,7 +18127,7 @@
         <v>46178.593344699075</v>
       </c>
       <c r="D225" s="11">
-        <v>46178.59343871528</v>
+        <v>46188.84820208333</v>
       </c>
       <c r="E225" s="12" t="s">
         <v>153</v>
@@ -18072,9 +18136,11 @@
         <v>488</v>
       </c>
       <c r="G225" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H225" s="12"/>
+        <v>44</v>
+      </c>
+      <c r="H225" s="12" t="s">
+        <v>45</v>
+      </c>
       <c r="I225" s="12"/>
       <c r="J225" s="11">
         <v>46171</v>
@@ -18134,7 +18200,7 @@
         <v>46176.84111434028</v>
       </c>
       <c r="D226" s="5">
-        <v>46176.84579140046</v>
+        <v>46188.847823171294</v>
       </c>
       <c r="E226" s="6" t="s">
         <v>40</v>
@@ -18143,9 +18209,11 @@
         <v>494</v>
       </c>
       <c r="G226" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H226" s="6"/>
+        <v>495</v>
+      </c>
+      <c r="H226" s="6" t="s">
+        <v>496</v>
+      </c>
       <c r="I226" s="6"/>
       <c r="J226" s="5">
         <v>46171</v>
@@ -18175,19 +18243,19 @@
         <v>35</v>
       </c>
       <c r="S226" s="6" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="T226" s="6" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="U226" s="8" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="V226" s="5">
         <v>46175</v>
       </c>
       <c r="W226" s="9" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="X226" s="6">
         <v>1</v>
@@ -18196,7 +18264,7 @@
     </row>
     <row r="227" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A227" s="10" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="B227" s="11">
         <v>46171.55906322917</v>
@@ -18205,7 +18273,7 @@
         <v>46176.84114244213</v>
       </c>
       <c r="D227" s="11">
-        <v>46176.8457389699</v>
+        <v>46188.84785686343</v>
       </c>
       <c r="E227" s="12" t="s">
         <v>83</v>
@@ -18214,9 +18282,11 @@
         <v>494</v>
       </c>
       <c r="G227" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H227" s="12"/>
+        <v>30</v>
+      </c>
+      <c r="H227" s="12" t="s">
+        <v>31</v>
+      </c>
       <c r="I227" s="12"/>
       <c r="J227" s="11">
         <v>46171</v>
@@ -18246,19 +18316,19 @@
         <v>35</v>
       </c>
       <c r="S227" s="12" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="T227" s="12" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="U227" s="8" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="V227" s="11">
         <v>46175</v>
       </c>
       <c r="W227" s="9" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="X227" s="12">
         <v>1</v>
@@ -18267,7 +18337,7 @@
     </row>
     <row r="228" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A228" s="4" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="B228" s="5">
         <v>46171.55907711806</v>
@@ -18276,7 +18346,7 @@
         <v>46176.8412162037</v>
       </c>
       <c r="D228" s="5">
-        <v>46177.57249943287</v>
+        <v>46188.847890439814</v>
       </c>
       <c r="E228" s="6" t="s">
         <v>153</v>
@@ -18285,9 +18355,11 @@
         <v>494</v>
       </c>
       <c r="G228" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H228" s="6"/>
+        <v>44</v>
+      </c>
+      <c r="H228" s="6" t="s">
+        <v>45</v>
+      </c>
       <c r="I228" s="6"/>
       <c r="J228" s="5">
         <v>46175</v>
@@ -18317,19 +18389,19 @@
         <v>35</v>
       </c>
       <c r="S228" s="6" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="T228" s="6" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="U228" s="8" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="V228" s="5">
         <v>46175</v>
       </c>
       <c r="W228" s="9" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="X228" s="6">
         <v>1</v>
@@ -18338,7 +18410,7 @@
     </row>
     <row r="229" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A229" s="10" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="B229" s="11">
         <v>46171.56219060185</v>
@@ -18347,18 +18419,20 @@
         <v>46181.89097277778</v>
       </c>
       <c r="D229" s="11">
-        <v>46181.891124456015</v>
+        <v>46188.84747278935</v>
       </c>
       <c r="E229" s="12" t="s">
         <v>40</v>
       </c>
       <c r="F229" s="12" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="G229" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H229" s="12"/>
+        <v>78</v>
+      </c>
+      <c r="H229" s="12" t="s">
+        <v>79</v>
+      </c>
       <c r="I229" s="12"/>
       <c r="J229" s="11">
         <v>46171</v>
@@ -18389,14 +18463,14 @@
       </c>
       <c r="S229" s="12"/>
       <c r="T229" s="12" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="U229" s="12"/>
       <c r="V229" s="11">
         <v>46181</v>
       </c>
       <c r="W229" s="9" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="X229" s="12">
         <v>0</v>
@@ -18405,7 +18479,7 @@
     </row>
     <row r="230" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A230" s="4" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="B230" s="5">
         <v>46171.56219597222</v>
@@ -18414,18 +18488,20 @@
         <v>46181.89118878472</v>
       </c>
       <c r="D230" s="5">
-        <v>46181.89140920139</v>
+        <v>46188.847506562495</v>
       </c>
       <c r="E230" s="6" t="s">
         <v>83</v>
       </c>
       <c r="F230" s="6" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="G230" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H230" s="6"/>
+        <v>30</v>
+      </c>
+      <c r="H230" s="6" t="s">
+        <v>31</v>
+      </c>
       <c r="I230" s="6"/>
       <c r="J230" s="5">
         <v>46171</v>
@@ -18456,14 +18532,14 @@
       </c>
       <c r="S230" s="6"/>
       <c r="T230" s="6" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="U230" s="6"/>
       <c r="V230" s="5">
         <v>46181</v>
       </c>
       <c r="W230" s="9" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="X230" s="6">
         <v>0</v>
@@ -18472,7 +18548,7 @@
     </row>
     <row r="231" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A231" s="10" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="B231" s="11">
         <v>46171.56220810185</v>
@@ -18481,18 +18557,20 @@
         <v>46181.89122921297</v>
       </c>
       <c r="D231" s="11">
-        <v>46185.7569015162</v>
+        <v>46188.84754002315</v>
       </c>
       <c r="E231" s="12" t="s">
         <v>153</v>
       </c>
       <c r="F231" s="12" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="G231" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H231" s="12"/>
+        <v>44</v>
+      </c>
+      <c r="H231" s="12" t="s">
+        <v>45</v>
+      </c>
       <c r="I231" s="12"/>
       <c r="J231" s="11">
         <v>46171</v>
@@ -18523,14 +18601,14 @@
       </c>
       <c r="S231" s="12"/>
       <c r="T231" s="12" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="U231" s="12"/>
       <c r="V231" s="11">
         <v>46185</v>
       </c>
       <c r="W231" s="9" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="X231" s="12">
         <v>0</v>
@@ -18539,7 +18617,7 @@
     </row>
     <row r="232" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A232" s="4" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="B232" s="5">
         <v>46174.78293828704</v>
@@ -18548,18 +18626,20 @@
         <v>46178.599825983794</v>
       </c>
       <c r="D232" s="5">
-        <v>46185.57793501158</v>
+        <v>46188.8494894676</v>
       </c>
       <c r="E232" s="6" t="s">
         <v>40</v>
       </c>
       <c r="F232" s="6" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="G232" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H232" s="6"/>
+        <v>495</v>
+      </c>
+      <c r="H232" s="6" t="s">
+        <v>496</v>
+      </c>
       <c r="I232" s="6"/>
       <c r="J232" s="5">
         <v>46174</v>
@@ -18589,10 +18669,10 @@
         <v>35</v>
       </c>
       <c r="S232" s="6" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="T232" s="6" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="U232" s="8" t="s">
         <v>38</v>
@@ -18601,7 +18681,7 @@
         <v>46177</v>
       </c>
       <c r="W232" s="9" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="X232" s="6">
         <v>1</v>
@@ -18610,7 +18690,7 @@
     </row>
     <row r="233" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A233" s="10" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="B233" s="11">
         <v>46174.78294421296</v>
@@ -18619,18 +18699,20 @@
         <v>46186.65179798611</v>
       </c>
       <c r="D233" s="11">
-        <v>46188.61648292824</v>
+        <v>46188.84951959491</v>
       </c>
       <c r="E233" s="12" t="s">
         <v>83</v>
       </c>
       <c r="F233" s="12" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="G233" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H233" s="12"/>
+        <v>30</v>
+      </c>
+      <c r="H233" s="12" t="s">
+        <v>31</v>
+      </c>
       <c r="I233" s="12"/>
       <c r="J233" s="11">
         <v>46174</v>
@@ -18660,10 +18742,10 @@
         <v>35</v>
       </c>
       <c r="S233" s="12" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="T233" s="12" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="U233" s="8" t="s">
         <v>38</v>
@@ -18672,7 +18754,7 @@
         <v>46185</v>
       </c>
       <c r="W233" s="9" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="X233" s="12">
         <v>1</v>
@@ -18681,7 +18763,7 @@
     </row>
     <row r="234" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A234" s="4" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="B234" s="5">
         <v>46174.782957372685</v>
@@ -18690,18 +18772,20 @@
         <v>46186.65184641204</v>
       </c>
       <c r="D234" s="5">
-        <v>46186.65194938658</v>
+        <v>46188.84956179398</v>
       </c>
       <c r="E234" s="6" t="s">
         <v>153</v>
       </c>
       <c r="F234" s="6" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="G234" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H234" s="6"/>
+        <v>44</v>
+      </c>
+      <c r="H234" s="6" t="s">
+        <v>45</v>
+      </c>
       <c r="I234" s="6"/>
       <c r="J234" s="5">
         <v>46174</v>
@@ -18731,10 +18815,10 @@
         <v>35</v>
       </c>
       <c r="S234" s="6" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="T234" s="6" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="U234" s="8" t="s">
         <v>38</v>
@@ -18743,7 +18827,7 @@
         <v>46177</v>
       </c>
       <c r="W234" s="9" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="X234" s="6">
         <v>1</v>
@@ -18752,7 +18836,7 @@
     </row>
     <row r="235" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A235" s="10" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="B235" s="11">
         <v>46175.62894534723</v>
@@ -18761,18 +18845,20 @@
         <v>46186.65099351852</v>
       </c>
       <c r="D235" s="11">
-        <v>46186.65119246527</v>
+        <v>46188.85313337963</v>
       </c>
       <c r="E235" s="12" t="s">
         <v>40</v>
       </c>
       <c r="F235" s="12" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="G235" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H235" s="12"/>
+        <v>30</v>
+      </c>
+      <c r="H235" s="12" t="s">
+        <v>31</v>
+      </c>
       <c r="I235" s="12"/>
       <c r="J235" s="11">
         <v>46175</v>
@@ -18802,10 +18888,10 @@
         <v>35</v>
       </c>
       <c r="S235" s="12" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="T235" s="12" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="U235" s="8" t="s">
         <v>141</v>
@@ -18814,7 +18900,7 @@
         <v>46182</v>
       </c>
       <c r="W235" s="9" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="X235" s="12">
         <v>1</v>
@@ -18823,7 +18909,7 @@
     </row>
     <row r="236" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A236" s="4" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B236" s="5">
         <v>46175.628960682865</v>
@@ -18832,18 +18918,20 @@
         <v>46185.56117458333</v>
       </c>
       <c r="D236" s="5">
-        <v>46185.56194986111</v>
+        <v>46188.8531612963</v>
       </c>
       <c r="E236" s="6" t="s">
         <v>83</v>
       </c>
       <c r="F236" s="6" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="G236" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H236" s="6"/>
+        <v>30</v>
+      </c>
+      <c r="H236" s="6" t="s">
+        <v>31</v>
+      </c>
       <c r="I236" s="6"/>
       <c r="J236" s="5">
         <v>46175</v>
@@ -18873,10 +18961,10 @@
         <v>35</v>
       </c>
       <c r="S236" s="6" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="T236" s="6" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="U236" s="8" t="s">
         <v>141</v>
@@ -18885,7 +18973,7 @@
         <v>46182</v>
       </c>
       <c r="W236" s="9" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="X236" s="6">
         <v>1</v>
@@ -18894,7 +18982,7 @@
     </row>
     <row r="237" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A237" s="10" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="B237" s="11">
         <v>46175.62896625</v>
@@ -18903,18 +18991,20 @@
         <v>46186.65103758102</v>
       </c>
       <c r="D237" s="11">
-        <v>46186.6511930787</v>
+        <v>46188.853190243055</v>
       </c>
       <c r="E237" s="12" t="s">
         <v>153</v>
       </c>
       <c r="F237" s="12" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="G237" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H237" s="12"/>
+        <v>44</v>
+      </c>
+      <c r="H237" s="12" t="s">
+        <v>45</v>
+      </c>
       <c r="I237" s="12"/>
       <c r="J237" s="11">
         <v>46175</v>
@@ -18944,10 +19034,10 @@
         <v>35</v>
       </c>
       <c r="S237" s="12" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="T237" s="12" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="U237" s="8" t="s">
         <v>141</v>
@@ -18956,7 +19046,7 @@
         <v>46182</v>
       </c>
       <c r="W237" s="9" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="X237" s="12">
         <v>1</v>
@@ -18965,7 +19055,7 @@
     </row>
     <row r="238" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A238" s="4" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="B238" s="5">
         <v>46177.55207784723</v>
@@ -18974,18 +19064,20 @@
         <v>46178.71568760417</v>
       </c>
       <c r="D238" s="5">
-        <v>46178.71573163195</v>
+        <v>46188.851797511576</v>
       </c>
       <c r="E238" s="6" t="s">
         <v>40</v>
       </c>
       <c r="F238" s="6" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="G238" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H238" s="6"/>
+        <v>78</v>
+      </c>
+      <c r="H238" s="6" t="s">
+        <v>79</v>
+      </c>
       <c r="I238" s="6"/>
       <c r="J238" s="5">
         <v>46176</v>
@@ -19015,10 +19107,10 @@
         <v>35</v>
       </c>
       <c r="S238" s="6" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="T238" s="6" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="U238" s="8" t="s">
         <v>141</v>
@@ -19027,7 +19119,7 @@
         <v>46178</v>
       </c>
       <c r="W238" s="9" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="X238" s="6">
         <v>0</v>
@@ -19036,7 +19128,7 @@
     </row>
     <row r="239" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A239" s="10" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="B239" s="11">
         <v>46177.552084675925</v>
@@ -19045,18 +19137,20 @@
         <v>46178.71550456018</v>
       </c>
       <c r="D239" s="11">
-        <v>46178.71554780092</v>
+        <v>46188.85182652778</v>
       </c>
       <c r="E239" s="12" t="s">
         <v>83</v>
       </c>
       <c r="F239" s="12" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="G239" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H239" s="12"/>
+        <v>30</v>
+      </c>
+      <c r="H239" s="12" t="s">
+        <v>31</v>
+      </c>
       <c r="I239" s="12"/>
       <c r="J239" s="11">
         <v>46176</v>
@@ -19086,10 +19180,10 @@
         <v>35</v>
       </c>
       <c r="S239" s="12" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="T239" s="12" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="U239" s="8" t="s">
         <v>141</v>
@@ -19098,7 +19192,7 @@
         <v>46177</v>
       </c>
       <c r="W239" s="9" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="X239" s="12">
         <v>0</v>
@@ -19107,7 +19201,7 @@
     </row>
     <row r="240" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A240" s="4" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="B240" s="5">
         <v>46177.552097997686</v>
@@ -19116,18 +19210,20 @@
         <v>46178.71575603009</v>
       </c>
       <c r="D240" s="5">
-        <v>46178.71576918982</v>
+        <v>46188.85186135417</v>
       </c>
       <c r="E240" s="6" t="s">
         <v>153</v>
       </c>
       <c r="F240" s="6" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="G240" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H240" s="6"/>
+        <v>495</v>
+      </c>
+      <c r="H240" s="6" t="s">
+        <v>496</v>
+      </c>
       <c r="I240" s="6"/>
       <c r="J240" s="5">
         <v>46176</v>
@@ -19157,10 +19253,10 @@
         <v>35</v>
       </c>
       <c r="S240" s="6" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="T240" s="6" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="U240" s="8" t="s">
         <v>141</v>
@@ -19169,7 +19265,7 @@
         <v>46178</v>
       </c>
       <c r="W240" s="9" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="X240" s="6">
         <v>0</v>
@@ -19178,7 +19274,7 @@
     </row>
     <row r="241" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A241" s="10" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="B241" s="11">
         <v>46177.55718690972</v>
@@ -19191,7 +19287,7 @@
         <v>40</v>
       </c>
       <c r="F241" s="12" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="G241" s="12" t="s">
         <v>78</v>
@@ -19231,14 +19327,14 @@
         <v>432</v>
       </c>
       <c r="T241" s="12" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="U241" s="8" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="V241" s="12"/>
       <c r="W241" s="9" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="X241" s="12">
         <v>0</v>
@@ -19247,7 +19343,7 @@
     </row>
     <row r="242" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A242" s="4" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="B242" s="5">
         <v>46177.55719148148</v>
@@ -19262,7 +19358,7 @@
         <v>83</v>
       </c>
       <c r="F242" s="6" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="G242" s="6" t="s">
         <v>30</v>
@@ -19302,16 +19398,16 @@
         <v>432</v>
       </c>
       <c r="T242" s="6" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="U242" s="8" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="V242" s="5">
         <v>46184</v>
       </c>
       <c r="W242" s="9" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="X242" s="6">
         <v>1</v>
@@ -19320,7 +19416,7 @@
     </row>
     <row r="243" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A243" s="10" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="B243" s="11">
         <v>46177.557204282406</v>
@@ -19333,7 +19429,7 @@
         <v>153</v>
       </c>
       <c r="F243" s="12" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="G243" s="12" t="s">
         <v>44</v>
@@ -19373,14 +19469,14 @@
         <v>432</v>
       </c>
       <c r="T243" s="12" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="U243" s="8" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="V243" s="12"/>
       <c r="W243" s="9" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="X243" s="12">
         <v>0</v>
@@ -19389,7 +19485,7 @@
     </row>
     <row r="244" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A244" s="4" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="B244" s="5">
         <v>46177.58134283565</v>
@@ -19398,18 +19494,20 @@
         <v>46177.58232075231</v>
       </c>
       <c r="D244" s="5">
-        <v>46177.58265486111</v>
+        <v>46188.85124024306</v>
       </c>
       <c r="E244" s="6" t="s">
         <v>40</v>
       </c>
       <c r="F244" s="6" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="G244" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H244" s="6"/>
+        <v>41</v>
+      </c>
+      <c r="H244" s="6" t="s">
+        <v>42</v>
+      </c>
       <c r="I244" s="6"/>
       <c r="J244" s="5">
         <v>46161</v>
@@ -19439,10 +19537,10 @@
         <v>35</v>
       </c>
       <c r="S244" s="6" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="T244" s="6" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="U244" s="8" t="s">
         <v>141</v>
@@ -19451,7 +19549,7 @@
         <v>46176</v>
       </c>
       <c r="W244" s="9" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="X244" s="6">
         <v>1</v>
@@ -19460,7 +19558,7 @@
     </row>
     <row r="245" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A245" s="10" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="B245" s="11">
         <v>46177.58134928241</v>
@@ -19469,18 +19567,20 @@
         <v>46178.56063146991</v>
       </c>
       <c r="D245" s="11">
-        <v>46181.55912813658</v>
+        <v>46188.8512880787</v>
       </c>
       <c r="E245" s="12" t="s">
         <v>83</v>
       </c>
       <c r="F245" s="12" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="G245" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H245" s="12"/>
+        <v>30</v>
+      </c>
+      <c r="H245" s="12" t="s">
+        <v>31</v>
+      </c>
       <c r="I245" s="12"/>
       <c r="J245" s="11">
         <v>46161</v>
@@ -19510,10 +19610,10 @@
         <v>35</v>
       </c>
       <c r="S245" s="12" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="T245" s="12" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="U245" s="8" t="s">
         <v>141</v>
@@ -19522,7 +19622,7 @@
         <v>46176</v>
       </c>
       <c r="W245" s="9" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="X245" s="12">
         <v>1</v>
@@ -19531,7 +19631,7 @@
     </row>
     <row r="246" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A246" s="4" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="B246" s="5">
         <v>46177.58136225694</v>
@@ -19540,18 +19640,20 @@
         <v>46178.5606772801</v>
       </c>
       <c r="D246" s="5">
-        <v>46181.55914805556</v>
+        <v>46188.85133394676</v>
       </c>
       <c r="E246" s="6" t="s">
         <v>153</v>
       </c>
       <c r="F246" s="6" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="G246" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H246" s="6"/>
+        <v>44</v>
+      </c>
+      <c r="H246" s="6" t="s">
+        <v>45</v>
+      </c>
       <c r="I246" s="6"/>
       <c r="J246" s="5">
         <v>46161</v>
@@ -19581,10 +19683,10 @@
         <v>35</v>
       </c>
       <c r="S246" s="6" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="T246" s="6" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="U246" s="8" t="s">
         <v>141</v>
@@ -19593,7 +19695,7 @@
         <v>46176</v>
       </c>
       <c r="W246" s="9" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="X246" s="6">
         <v>1</v>
@@ -19602,7 +19704,7 @@
     </row>
     <row r="247" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A247" s="10" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="B247" s="11">
         <v>46181.55894307871</v>
@@ -19615,7 +19717,7 @@
         <v>40</v>
       </c>
       <c r="F247" s="12" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="G247" s="12" t="s">
         <v>56</v>
@@ -19652,17 +19754,17 @@
         <v>35</v>
       </c>
       <c r="S247" s="12" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="T247" s="12" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="U247" s="8" t="s">
         <v>95</v>
       </c>
       <c r="V247" s="12"/>
       <c r="W247" s="9" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="X247" s="12">
         <v>0</v>
@@ -19671,7 +19773,7 @@
     </row>
     <row r="248" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A248" s="4" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="B248" s="5">
         <v>46181.55895883102</v>
@@ -19686,7 +19788,7 @@
         <v>83</v>
       </c>
       <c r="F248" s="6" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="G248" s="6" t="s">
         <v>30</v>
@@ -19723,10 +19825,10 @@
         <v>35</v>
       </c>
       <c r="S248" s="6" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="T248" s="6" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="U248" s="8" t="s">
         <v>95</v>
@@ -19735,7 +19837,7 @@
         <v>46184</v>
       </c>
       <c r="W248" s="9" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="X248" s="6">
         <v>1</v>
@@ -19744,7 +19846,7 @@
     </row>
     <row r="249" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A249" s="10" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="B249" s="11">
         <v>46181.55896603009</v>
@@ -19757,7 +19859,7 @@
         <v>153</v>
       </c>
       <c r="F249" s="12" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="G249" s="12" t="s">
         <v>44</v>
@@ -19794,17 +19896,17 @@
         <v>35</v>
       </c>
       <c r="S249" s="12" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="T249" s="12" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="U249" s="8" t="s">
         <v>95</v>
       </c>
       <c r="V249" s="12"/>
       <c r="W249" s="9" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="X249" s="12">
         <v>0</v>
@@ -19813,7 +19915,7 @@
     </row>
     <row r="250" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A250" s="4" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="B250" s="5">
         <v>46181.56214887732</v>
@@ -19826,7 +19928,7 @@
         <v>40</v>
       </c>
       <c r="F250" s="6" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="G250" s="6" t="s">
         <v>32</v>
@@ -19861,7 +19963,7 @@
         <v>35</v>
       </c>
       <c r="S250" s="6" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="T250" s="6"/>
       <c r="U250" s="8" t="s">
@@ -19876,7 +19978,7 @@
     </row>
     <row r="251" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A251" s="10" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="B251" s="11">
         <v>46181.562153425926</v>
@@ -19889,7 +19991,7 @@
         <v>83</v>
       </c>
       <c r="F251" s="12" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="G251" s="12" t="s">
         <v>32</v>
@@ -19924,7 +20026,7 @@
         <v>35</v>
       </c>
       <c r="S251" s="12" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="T251" s="12"/>
       <c r="U251" s="8" t="s">
@@ -19939,7 +20041,7 @@
     </row>
     <row r="252" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A252" s="4" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="B252" s="5">
         <v>46181.562166250005</v>
@@ -19952,7 +20054,7 @@
         <v>153</v>
       </c>
       <c r="F252" s="6" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="G252" s="6" t="s">
         <v>32</v>
@@ -19987,7 +20089,7 @@
         <v>35</v>
       </c>
       <c r="S252" s="6" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="T252" s="6"/>
       <c r="U252" s="8" t="s">
@@ -20002,7 +20104,7 @@
     </row>
     <row r="253" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A253" s="10" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="B253" s="11">
         <v>46181.5643593287</v>
@@ -20015,7 +20117,7 @@
         <v>40</v>
       </c>
       <c r="F253" s="12" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="G253" s="12" t="s">
         <v>32</v>
@@ -20050,7 +20152,7 @@
         <v>35</v>
       </c>
       <c r="S253" s="12" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="T253" s="12"/>
       <c r="U253" s="12"/>
@@ -20063,7 +20165,7 @@
     </row>
     <row r="254" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A254" s="4" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="B254" s="5">
         <v>46181.56436351852</v>
@@ -20076,7 +20178,7 @@
         <v>83</v>
       </c>
       <c r="F254" s="6" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="G254" s="6" t="s">
         <v>32</v>
@@ -20111,7 +20213,7 @@
         <v>35</v>
       </c>
       <c r="S254" s="6" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="T254" s="6"/>
       <c r="U254" s="6"/>
@@ -20124,7 +20226,7 @@
     </row>
     <row r="255" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A255" s="10" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="B255" s="11">
         <v>46181.56437451389</v>
@@ -20137,7 +20239,7 @@
         <v>153</v>
       </c>
       <c r="F255" s="12" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="G255" s="12" t="s">
         <v>32</v>
@@ -20172,7 +20274,7 @@
         <v>35</v>
       </c>
       <c r="S255" s="12" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="T255" s="12"/>
       <c r="U255" s="12"/>
@@ -20185,7 +20287,7 @@
     </row>
     <row r="256" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A256" s="4" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="B256" s="5">
         <v>46185.55074734954</v>
@@ -20200,7 +20302,7 @@
         <v>40</v>
       </c>
       <c r="F256" s="6" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="G256" s="6" t="s">
         <v>32</v>
@@ -20235,10 +20337,10 @@
         <v>35</v>
       </c>
       <c r="S256" s="6" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="T256" s="6" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="U256" s="8" t="s">
         <v>95</v>
@@ -20247,7 +20349,7 @@
         <v>46184</v>
       </c>
       <c r="W256" s="9" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="X256" s="6">
         <v>1</v>
@@ -20256,7 +20358,7 @@
     </row>
     <row r="257" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A257" s="10" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="B257" s="11">
         <v>46185.5507533912</v>
@@ -20269,7 +20371,7 @@
         <v>83</v>
       </c>
       <c r="F257" s="12" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="G257" s="12" t="s">
         <v>32</v>
@@ -20304,17 +20406,17 @@
         <v>35</v>
       </c>
       <c r="S257" s="12" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="T257" s="12" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="U257" s="8" t="s">
         <v>95</v>
       </c>
       <c r="V257" s="12"/>
       <c r="W257" s="9" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="X257" s="12">
         <v>0</v>
@@ -20323,7 +20425,7 @@
     </row>
     <row r="258" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A258" s="4" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="B258" s="5">
         <v>46185.55076409722</v>
@@ -20336,7 +20438,7 @@
         <v>153</v>
       </c>
       <c r="F258" s="6" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="G258" s="6" t="s">
         <v>32</v>
@@ -20371,17 +20473,17 @@
         <v>35</v>
       </c>
       <c r="S258" s="6" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="T258" s="6" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="U258" s="8" t="s">
         <v>95</v>
       </c>
       <c r="V258" s="6"/>
       <c r="W258" s="9" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="X258" s="6">
         <v>0</v>
@@ -20390,7 +20492,7 @@
     </row>
     <row r="259" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A259" s="10" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="B259" s="11">
         <v>46185.55686909722</v>
@@ -20403,7 +20505,7 @@
         <v>40</v>
       </c>
       <c r="F259" s="12" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="G259" s="12" t="s">
         <v>32</v>
@@ -20438,17 +20540,17 @@
         <v>35</v>
       </c>
       <c r="S259" s="12" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="T259" s="12" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="U259" s="8" t="s">
         <v>291</v>
       </c>
       <c r="V259" s="12"/>
       <c r="W259" s="9" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="X259" s="12">
         <v>0</v>
@@ -20457,7 +20559,7 @@
     </row>
     <row r="260" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A260" s="4" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
       <c r="B260" s="5">
         <v>46185.55687354167</v>
@@ -20470,7 +20572,7 @@
         <v>83</v>
       </c>
       <c r="F260" s="6" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="G260" s="6" t="s">
         <v>32</v>
@@ -20505,17 +20607,17 @@
         <v>35</v>
       </c>
       <c r="S260" s="6" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="T260" s="6" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="U260" s="8" t="s">
         <v>291</v>
       </c>
       <c r="V260" s="6"/>
       <c r="W260" s="9" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="X260" s="6">
         <v>0</v>
@@ -20524,7 +20626,7 @@
     </row>
     <row r="261" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A261" s="10" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="B261" s="11">
         <v>46185.55688491898</v>
@@ -20537,7 +20639,7 @@
         <v>153</v>
       </c>
       <c r="F261" s="12" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="G261" s="12" t="s">
         <v>32</v>
@@ -20572,17 +20674,17 @@
         <v>35</v>
       </c>
       <c r="S261" s="12" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="T261" s="12" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="U261" s="8" t="s">
         <v>291</v>
       </c>
       <c r="V261" s="12"/>
       <c r="W261" s="9" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="X261" s="12">
         <v>0</v>
@@ -20591,7 +20693,7 @@
     </row>
     <row r="262" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A262" s="4" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="B262" s="5">
         <v>46185.56558032407</v>
@@ -20604,7 +20706,7 @@
         <v>40</v>
       </c>
       <c r="F262" s="6" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="G262" s="6" t="s">
         <v>41</v>
@@ -20641,17 +20743,17 @@
         <v>35</v>
       </c>
       <c r="S262" s="6" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="T262" s="6" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="U262" s="8" t="s">
         <v>141</v>
       </c>
       <c r="V262" s="6"/>
       <c r="W262" s="9" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="X262" s="6">
         <v>0</v>
@@ -20660,7 +20762,7 @@
     </row>
     <row r="263" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A263" s="10" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="B263" s="11">
         <v>46185.56558616898</v>
@@ -20675,7 +20777,7 @@
         <v>83</v>
       </c>
       <c r="F263" s="12" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="G263" s="12" t="s">
         <v>30</v>
@@ -20712,10 +20814,10 @@
         <v>35</v>
       </c>
       <c r="S263" s="12" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="T263" s="12" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="U263" s="8" t="s">
         <v>141</v>
@@ -20724,7 +20826,7 @@
         <v>46185</v>
       </c>
       <c r="W263" s="9" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="X263" s="12">
         <v>1</v>
@@ -20733,7 +20835,7 @@
     </row>
     <row r="264" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A264" s="4" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="B264" s="5">
         <v>46185.56559773148</v>
@@ -20746,7 +20848,7 @@
         <v>153</v>
       </c>
       <c r="F264" s="6" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="G264" s="6" t="s">
         <v>44</v>
@@ -20783,17 +20885,17 @@
         <v>35</v>
       </c>
       <c r="S264" s="6" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="T264" s="6" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="U264" s="8" t="s">
         <v>141</v>
       </c>
       <c r="V264" s="6"/>
       <c r="W264" s="9" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="X264" s="6">
         <v>0</v>
@@ -20802,7 +20904,7 @@
     </row>
     <row r="265" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A265" s="10" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="B265" s="11">
         <v>46185.59436649305</v>
@@ -20815,7 +20917,7 @@
         <v>40</v>
       </c>
       <c r="F265" s="12" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="G265" s="12" t="s">
         <v>32</v>
@@ -20851,14 +20953,14 @@
       </c>
       <c r="S265" s="12"/>
       <c r="T265" s="12" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="U265" s="8" t="s">
         <v>291</v>
       </c>
       <c r="V265" s="12"/>
       <c r="W265" s="9" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="X265" s="12">
         <v>0</v>
@@ -20867,7 +20969,7 @@
     </row>
     <row r="266" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A266" s="4" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
       <c r="B266" s="5">
         <v>46185.59437232639</v>
@@ -20880,7 +20982,7 @@
         <v>83</v>
       </c>
       <c r="F266" s="6" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="G266" s="6" t="s">
         <v>32</v>
@@ -20916,14 +21018,14 @@
       </c>
       <c r="S266" s="6"/>
       <c r="T266" s="6" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="U266" s="8" t="s">
         <v>291</v>
       </c>
       <c r="V266" s="6"/>
       <c r="W266" s="9" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="X266" s="6">
         <v>0</v>
@@ -20932,7 +21034,7 @@
     </row>
     <row r="267" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A267" s="10" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="B267" s="11">
         <v>46185.594386770834</v>
@@ -20945,7 +21047,7 @@
         <v>153</v>
       </c>
       <c r="F267" s="12" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="G267" s="12" t="s">
         <v>32</v>
@@ -20981,14 +21083,14 @@
       </c>
       <c r="S267" s="12"/>
       <c r="T267" s="12" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="U267" s="8" t="s">
         <v>291</v>
       </c>
       <c r="V267" s="12"/>
       <c r="W267" s="9" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="X267" s="12">
         <v>0</v>
@@ -20997,7 +21099,7 @@
     </row>
     <row r="268" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A268" s="4" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="B268" s="5">
         <v>46186.654707650465</v>
@@ -21012,7 +21114,7 @@
         <v>40</v>
       </c>
       <c r="F268" s="6" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="G268" s="6" t="s">
         <v>32</v>
@@ -21050,7 +21152,7 @@
       </c>
       <c r="S268" s="6"/>
       <c r="T268" s="6" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="U268" s="8" t="s">
         <v>38</v>
@@ -21059,7 +21161,7 @@
         <v>46157</v>
       </c>
       <c r="W268" s="9" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="X268" s="6">
         <v>1</v>
@@ -21068,7 +21170,7 @@
     </row>
     <row r="269" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A269" s="10" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B269" s="11">
         <v>46186.65471349537</v>
@@ -21083,7 +21185,7 @@
         <v>83</v>
       </c>
       <c r="F269" s="12" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="G269" s="12" t="s">
         <v>32</v>
@@ -21121,7 +21223,7 @@
       </c>
       <c r="S269" s="12"/>
       <c r="T269" s="12" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="U269" s="8" t="s">
         <v>38</v>
@@ -21130,7 +21232,7 @@
         <v>46157</v>
       </c>
       <c r="W269" s="9" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="X269" s="12">
         <v>1</v>
@@ -21139,7 +21241,7 @@
     </row>
     <row r="270" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A270" s="4" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="B270" s="5">
         <v>46186.654726875</v>
@@ -21154,7 +21256,7 @@
         <v>153</v>
       </c>
       <c r="F270" s="6" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="G270" s="6" t="s">
         <v>32</v>
@@ -21192,7 +21294,7 @@
       </c>
       <c r="S270" s="6"/>
       <c r="T270" s="6" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="U270" s="8" t="s">
         <v>38</v>
@@ -21201,7 +21303,7 @@
         <v>46157</v>
       </c>
       <c r="W270" s="9" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="X270" s="6">
         <v>1</v>

</xml_diff>

<commit_message>
Actualizar dashboard Oferta Zitron 2026 2026-06-17 21:00 UTC
</commit_message>
<xml_diff>
--- a/data_ofertas/Oferta Zitron 2026.xlsx
+++ b/data_ofertas/Oferta Zitron 2026.xlsx
@@ -19279,9 +19279,11 @@
       <c r="B241" s="11">
         <v>46177.55718690972</v>
       </c>
-      <c r="C241" s="12"/>
+      <c r="C241" s="11">
+        <v>46190.6980797338</v>
+      </c>
       <c r="D241" s="11">
-        <v>46188.70072540509</v>
+        <v>46190.698196157406</v>
       </c>
       <c r="E241" s="12" t="s">
         <v>40</v>
@@ -19332,12 +19334,14 @@
       <c r="U241" s="8" t="s">
         <v>530</v>
       </c>
-      <c r="V241" s="12"/>
+      <c r="V241" s="11">
+        <v>46189</v>
+      </c>
       <c r="W241" s="9" t="s">
         <v>529</v>
       </c>
       <c r="X241" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y241" s="12"/>
     </row>
@@ -19421,9 +19425,11 @@
       <c r="B243" s="11">
         <v>46177.557204282406</v>
       </c>
-      <c r="C243" s="12"/>
+      <c r="C243" s="11">
+        <v>46190.698173136574</v>
+      </c>
       <c r="D243" s="11">
-        <v>46188.700669502316</v>
+        <v>46190.6982653125</v>
       </c>
       <c r="E243" s="12" t="s">
         <v>153</v>
@@ -19474,12 +19480,14 @@
       <c r="U243" s="8" t="s">
         <v>530</v>
       </c>
-      <c r="V243" s="12"/>
+      <c r="V243" s="11">
+        <v>46190</v>
+      </c>
       <c r="W243" s="9" t="s">
         <v>529</v>
       </c>
       <c r="X243" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y243" s="12"/>
     </row>

</xml_diff>

<commit_message>
Actualizar dashboard Oferta Zitron 2026 2026-06-18 21:18 UTC
</commit_message>
<xml_diff>
--- a/data_ofertas/Oferta Zitron 2026.xlsx
+++ b/data_ofertas/Oferta Zitron 2026.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4427" uniqueCount="581">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4571" uniqueCount="599">
   <si>
     <t>Oferta Zitron 2026</t>
   </si>
@@ -1755,6 +1755,60 @@
   </si>
   <si>
     <t>1215689131135204</t>
+  </si>
+  <si>
+    <t>1215832622787136</t>
+  </si>
+  <si>
+    <t>26MX0057 - Solicitud de Agnico Eagle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26MX0057 </t>
+  </si>
+  <si>
+    <t>1215832471502620</t>
+  </si>
+  <si>
+    <t>1215832471502643</t>
+  </si>
+  <si>
+    <t>1215832760194125</t>
+  </si>
+  <si>
+    <t>6001084633_CH01_SUM MTTO SISTEMAS DE VENTILACION - Chuquicamata</t>
+  </si>
+  <si>
+    <t>codelco</t>
+  </si>
+  <si>
+    <t>6001084633</t>
+  </si>
+  <si>
+    <t>1215833061426162</t>
+  </si>
+  <si>
+    <t>1215832804858805</t>
+  </si>
+  <si>
+    <t>1215833256340966</t>
+  </si>
+  <si>
+    <t>25CO0018 - Actualización de trafico estudio ventilación túnel 2</t>
+  </si>
+  <si>
+    <t>julio</t>
+  </si>
+  <si>
+    <t>túnel| de Oriente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25CO0018 </t>
+  </si>
+  <si>
+    <t>1215833063487821</t>
+  </si>
+  <si>
+    <t>1215833063501310</t>
   </si>
 </sst>
 </file>
@@ -2278,7 +2332,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Y270"/>
+  <dimension ref="A1:Y279"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10.4" customWidth="1"/>
@@ -19717,9 +19771,11 @@
       <c r="B247" s="11">
         <v>46181.55894307871</v>
       </c>
-      <c r="C247" s="12"/>
+      <c r="C247" s="11">
+        <v>46191.56175753472</v>
+      </c>
       <c r="D247" s="11">
-        <v>46181.89273652778</v>
+        <v>46191.561839016205</v>
       </c>
       <c r="E247" s="12" t="s">
         <v>40</v>
@@ -19770,12 +19826,14 @@
       <c r="U247" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="V247" s="12"/>
+      <c r="V247" s="11">
+        <v>46191</v>
+      </c>
       <c r="W247" s="9" t="s">
         <v>542</v>
       </c>
       <c r="X247" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y247" s="12"/>
     </row>
@@ -19861,7 +19919,7 @@
       </c>
       <c r="C249" s="12"/>
       <c r="D249" s="11">
-        <v>46185.59164436343</v>
+        <v>46191.56176628472</v>
       </c>
       <c r="E249" s="12" t="s">
         <v>153</v>
@@ -20982,9 +21040,11 @@
       <c r="B266" s="5">
         <v>46185.59437232639</v>
       </c>
-      <c r="C266" s="6"/>
+      <c r="C266" s="5">
+        <v>46191.568297233796</v>
+      </c>
       <c r="D266" s="5">
-        <v>46185.59551452546</v>
+        <v>46191.56839601852</v>
       </c>
       <c r="E266" s="6" t="s">
         <v>83</v>
@@ -21031,12 +21091,14 @@
       <c r="U266" s="8" t="s">
         <v>291</v>
       </c>
-      <c r="V266" s="6"/>
+      <c r="V266" s="5">
+        <v>46191</v>
+      </c>
       <c r="W266" s="9" t="s">
         <v>574</v>
       </c>
       <c r="X266" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y266" s="6"/>
     </row>
@@ -21049,7 +21111,7 @@
       </c>
       <c r="C267" s="12"/>
       <c r="D267" s="11">
-        <v>46185.595515127316</v>
+        <v>46191.56830153935</v>
       </c>
       <c r="E267" s="12" t="s">
         <v>153</v>
@@ -21317,6 +21379,627 @@
         <v>1</v>
       </c>
       <c r="Y270" s="6"/>
+    </row>
+    <row r="271" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A271" s="10" t="s">
+        <v>581</v>
+      </c>
+      <c r="B271" s="11">
+        <v>46191.5563</v>
+      </c>
+      <c r="C271" s="12"/>
+      <c r="D271" s="11">
+        <v>46191.560530347226</v>
+      </c>
+      <c r="E271" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="F271" s="12" t="s">
+        <v>582</v>
+      </c>
+      <c r="G271" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="H271" s="12"/>
+      <c r="I271" s="11">
+        <v>46190</v>
+      </c>
+      <c r="J271" s="11">
+        <v>46190</v>
+      </c>
+      <c r="K271" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="L271" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="M271" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N271" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="O271" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="P271" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q271" s="7" t="s">
+        <v>431</v>
+      </c>
+      <c r="R271" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S271" s="12" t="s">
+        <v>478</v>
+      </c>
+      <c r="T271" s="12" t="s">
+        <v>583</v>
+      </c>
+      <c r="U271" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="V271" s="12"/>
+      <c r="W271" s="9" t="s">
+        <v>583</v>
+      </c>
+      <c r="X271" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y271" s="12"/>
+    </row>
+    <row r="272" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A272" s="4" t="s">
+        <v>584</v>
+      </c>
+      <c r="B272" s="5">
+        <v>46191.55632112268</v>
+      </c>
+      <c r="C272" s="6"/>
+      <c r="D272" s="5">
+        <v>46191.56054730324</v>
+      </c>
+      <c r="E272" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="F272" s="6" t="s">
+        <v>582</v>
+      </c>
+      <c r="G272" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H272" s="6"/>
+      <c r="I272" s="5">
+        <v>46190</v>
+      </c>
+      <c r="J272" s="5">
+        <v>46190</v>
+      </c>
+      <c r="K272" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="L272" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="M272" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N272" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="O272" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="P272" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q272" s="7" t="s">
+        <v>431</v>
+      </c>
+      <c r="R272" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S272" s="6" t="s">
+        <v>478</v>
+      </c>
+      <c r="T272" s="6" t="s">
+        <v>583</v>
+      </c>
+      <c r="U272" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="V272" s="6"/>
+      <c r="W272" s="9" t="s">
+        <v>583</v>
+      </c>
+      <c r="X272" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y272" s="6"/>
+    </row>
+    <row r="273" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A273" s="10" t="s">
+        <v>585</v>
+      </c>
+      <c r="B273" s="11">
+        <v>46191.55632693287</v>
+      </c>
+      <c r="C273" s="12"/>
+      <c r="D273" s="11">
+        <v>46191.56056363426</v>
+      </c>
+      <c r="E273" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="F273" s="12" t="s">
+        <v>582</v>
+      </c>
+      <c r="G273" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="H273" s="12"/>
+      <c r="I273" s="11">
+        <v>46190</v>
+      </c>
+      <c r="J273" s="11">
+        <v>46190</v>
+      </c>
+      <c r="K273" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="L273" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="M273" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N273" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="O273" s="12" t="s">
+        <v>104</v>
+      </c>
+      <c r="P273" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q273" s="7" t="s">
+        <v>431</v>
+      </c>
+      <c r="R273" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S273" s="12" t="s">
+        <v>478</v>
+      </c>
+      <c r="T273" s="12" t="s">
+        <v>583</v>
+      </c>
+      <c r="U273" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="V273" s="12"/>
+      <c r="W273" s="9" t="s">
+        <v>583</v>
+      </c>
+      <c r="X273" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y273" s="12"/>
+    </row>
+    <row r="274" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A274" s="4" t="s">
+        <v>586</v>
+      </c>
+      <c r="B274" s="5">
+        <v>46191.562819375</v>
+      </c>
+      <c r="C274" s="6"/>
+      <c r="D274" s="5">
+        <v>46191.56406366898</v>
+      </c>
+      <c r="E274" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F274" s="6" t="s">
+        <v>587</v>
+      </c>
+      <c r="G274" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H274" s="6"/>
+      <c r="I274" s="5">
+        <v>46190</v>
+      </c>
+      <c r="J274" s="5">
+        <v>46190</v>
+      </c>
+      <c r="K274" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="L274" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="M274" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N274" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="O274" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="P274" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q274" s="7" t="s">
+        <v>431</v>
+      </c>
+      <c r="R274" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S274" s="6" t="s">
+        <v>588</v>
+      </c>
+      <c r="T274" s="6" t="s">
+        <v>589</v>
+      </c>
+      <c r="U274" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="V274" s="6"/>
+      <c r="W274" s="9" t="s">
+        <v>589</v>
+      </c>
+      <c r="X274" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y274" s="6"/>
+    </row>
+    <row r="275" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A275" s="10" t="s">
+        <v>590</v>
+      </c>
+      <c r="B275" s="11">
+        <v>46191.56282547454</v>
+      </c>
+      <c r="C275" s="12"/>
+      <c r="D275" s="11">
+        <v>46191.56406429398</v>
+      </c>
+      <c r="E275" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="F275" s="12" t="s">
+        <v>587</v>
+      </c>
+      <c r="G275" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="H275" s="12"/>
+      <c r="I275" s="11">
+        <v>46190</v>
+      </c>
+      <c r="J275" s="11">
+        <v>46190</v>
+      </c>
+      <c r="K275" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="L275" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="M275" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N275" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="O275" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="P275" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q275" s="7" t="s">
+        <v>431</v>
+      </c>
+      <c r="R275" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S275" s="12" t="s">
+        <v>588</v>
+      </c>
+      <c r="T275" s="12" t="s">
+        <v>589</v>
+      </c>
+      <c r="U275" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="V275" s="12"/>
+      <c r="W275" s="9" t="s">
+        <v>589</v>
+      </c>
+      <c r="X275" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y275" s="12"/>
+    </row>
+    <row r="276" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A276" s="4" t="s">
+        <v>591</v>
+      </c>
+      <c r="B276" s="5">
+        <v>46191.56283715278</v>
+      </c>
+      <c r="C276" s="6"/>
+      <c r="D276" s="5">
+        <v>46191.56406495371</v>
+      </c>
+      <c r="E276" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="F276" s="6" t="s">
+        <v>587</v>
+      </c>
+      <c r="G276" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H276" s="6"/>
+      <c r="I276" s="5">
+        <v>46190</v>
+      </c>
+      <c r="J276" s="5">
+        <v>46190</v>
+      </c>
+      <c r="K276" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="L276" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="M276" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N276" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="O276" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="P276" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q276" s="7" t="s">
+        <v>431</v>
+      </c>
+      <c r="R276" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S276" s="6" t="s">
+        <v>588</v>
+      </c>
+      <c r="T276" s="6" t="s">
+        <v>589</v>
+      </c>
+      <c r="U276" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="V276" s="6"/>
+      <c r="W276" s="9" t="s">
+        <v>589</v>
+      </c>
+      <c r="X276" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y276" s="6"/>
+    </row>
+    <row r="277" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A277" s="10" t="s">
+        <v>592</v>
+      </c>
+      <c r="B277" s="11">
+        <v>46191.56523744213</v>
+      </c>
+      <c r="C277" s="12"/>
+      <c r="D277" s="11">
+        <v>46191.56620980324</v>
+      </c>
+      <c r="E277" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="F277" s="12" t="s">
+        <v>593</v>
+      </c>
+      <c r="G277" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="H277" s="12"/>
+      <c r="I277" s="11">
+        <v>46190</v>
+      </c>
+      <c r="J277" s="11">
+        <v>46190</v>
+      </c>
+      <c r="K277" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="L277" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="M277" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N277" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="O277" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="P277" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q277" s="7" t="s">
+        <v>594</v>
+      </c>
+      <c r="R277" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S277" s="12" t="s">
+        <v>595</v>
+      </c>
+      <c r="T277" s="12" t="s">
+        <v>596</v>
+      </c>
+      <c r="U277" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="V277" s="12"/>
+      <c r="W277" s="9" t="s">
+        <v>596</v>
+      </c>
+      <c r="X277" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y277" s="12"/>
+    </row>
+    <row r="278" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A278" s="4" t="s">
+        <v>597</v>
+      </c>
+      <c r="B278" s="5">
+        <v>46191.565243125</v>
+      </c>
+      <c r="C278" s="6"/>
+      <c r="D278" s="5">
+        <v>46191.56619353009</v>
+      </c>
+      <c r="E278" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="F278" s="6" t="s">
+        <v>593</v>
+      </c>
+      <c r="G278" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H278" s="6"/>
+      <c r="I278" s="5">
+        <v>46190</v>
+      </c>
+      <c r="J278" s="5">
+        <v>46190</v>
+      </c>
+      <c r="K278" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="L278" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="M278" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N278" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="O278" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="P278" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q278" s="7" t="s">
+        <v>594</v>
+      </c>
+      <c r="R278" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S278" s="6" t="s">
+        <v>595</v>
+      </c>
+      <c r="T278" s="6" t="s">
+        <v>596</v>
+      </c>
+      <c r="U278" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="V278" s="6"/>
+      <c r="W278" s="9" t="s">
+        <v>596</v>
+      </c>
+      <c r="X278" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y278" s="6"/>
+    </row>
+    <row r="279" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A279" s="10" t="s">
+        <v>598</v>
+      </c>
+      <c r="B279" s="11">
+        <v>46191.56525601852</v>
+      </c>
+      <c r="C279" s="12"/>
+      <c r="D279" s="11">
+        <v>46191.566233101854</v>
+      </c>
+      <c r="E279" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="F279" s="12" t="s">
+        <v>593</v>
+      </c>
+      <c r="G279" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="H279" s="12"/>
+      <c r="I279" s="11">
+        <v>46190</v>
+      </c>
+      <c r="J279" s="11">
+        <v>46190</v>
+      </c>
+      <c r="K279" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="L279" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="M279" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N279" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="O279" s="12" t="s">
+        <v>104</v>
+      </c>
+      <c r="P279" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q279" s="7" t="s">
+        <v>594</v>
+      </c>
+      <c r="R279" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S279" s="12" t="s">
+        <v>595</v>
+      </c>
+      <c r="T279" s="12" t="s">
+        <v>596</v>
+      </c>
+      <c r="U279" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="V279" s="12"/>
+      <c r="W279" s="9" t="s">
+        <v>596</v>
+      </c>
+      <c r="X279" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y279" s="12"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Actualizar dashboard Oferta Zitron 2026 2026-06-22 15:24 UTC
</commit_message>
<xml_diff>
--- a/data_ofertas/Oferta Zitron 2026.xlsx
+++ b/data_ofertas/Oferta Zitron 2026.xlsx
@@ -21456,9 +21456,11 @@
       <c r="B272" s="5">
         <v>46191.55632112268</v>
       </c>
-      <c r="C272" s="6"/>
+      <c r="C272" s="5">
+        <v>46195.629689953705</v>
+      </c>
       <c r="D272" s="5">
-        <v>46191.56054730324</v>
+        <v>46195.629756435184</v>
       </c>
       <c r="E272" s="6" t="s">
         <v>83</v>
@@ -21509,7 +21511,9 @@
       <c r="U272" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="V272" s="6"/>
+      <c r="V272" s="5">
+        <v>46195</v>
+      </c>
       <c r="W272" s="9" t="s">
         <v>583</v>
       </c>
@@ -21527,7 +21531,7 @@
       </c>
       <c r="C273" s="12"/>
       <c r="D273" s="11">
-        <v>46191.56056363426</v>
+        <v>46195.62969903935</v>
       </c>
       <c r="E273" s="12" t="s">
         <v>153</v>

</xml_diff>

<commit_message>
Actualizar dashboard Oferta Zitron 2026 2026-06-23 21:44 UTC
</commit_message>
<xml_diff>
--- a/data_ofertas/Oferta Zitron 2026.xlsx
+++ b/data_ofertas/Oferta Zitron 2026.xlsx
@@ -3600,9 +3600,11 @@
       <c r="B20" s="5">
         <v>46139.60183546296</v>
       </c>
-      <c r="C20" s="6"/>
+      <c r="C20" s="5">
+        <v>46196.89990372685</v>
+      </c>
       <c r="D20" s="5">
-        <v>46156.55999770833</v>
+        <v>46196.900087222224</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>83</v>
@@ -3653,12 +3655,14 @@
       <c r="U20" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="V20" s="6"/>
+      <c r="V20" s="5">
+        <v>46141</v>
+      </c>
       <c r="W20" s="9" t="s">
         <v>81</v>
       </c>
       <c r="X20" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y20" s="6"/>
     </row>
@@ -3671,7 +3675,7 @@
       </c>
       <c r="C21" s="12"/>
       <c r="D21" s="11">
-        <v>46156.55999826389</v>
+        <v>46196.89991287037</v>
       </c>
       <c r="E21" s="12" t="s">
         <v>33</v>
@@ -4223,9 +4227,11 @@
       <c r="B29" s="11">
         <v>46139.61063707176</v>
       </c>
-      <c r="C29" s="12"/>
+      <c r="C29" s="11">
+        <v>46196.90065589121</v>
+      </c>
       <c r="D29" s="11">
-        <v>46156.56005439815</v>
+        <v>46196.900839594906</v>
       </c>
       <c r="E29" s="12" t="s">
         <v>83</v>
@@ -4276,12 +4282,14 @@
       <c r="U29" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="V29" s="12"/>
+      <c r="V29" s="11">
+        <v>46141</v>
+      </c>
       <c r="W29" s="9" t="s">
         <v>81</v>
       </c>
       <c r="X29" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y29" s="12"/>
     </row>
@@ -4294,7 +4302,7 @@
       </c>
       <c r="C30" s="6"/>
       <c r="D30" s="5">
-        <v>46156.56007792824</v>
+        <v>46196.90066267361</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>33</v>
@@ -20975,9 +20983,11 @@
       <c r="B265" s="11">
         <v>46185.59436649305</v>
       </c>
-      <c r="C265" s="12"/>
+      <c r="C265" s="11">
+        <v>46196.894634571756</v>
+      </c>
       <c r="D265" s="11">
-        <v>46185.595513900465</v>
+        <v>46196.8947141088</v>
       </c>
       <c r="E265" s="12" t="s">
         <v>40</v>
@@ -21024,12 +21034,14 @@
       <c r="U265" s="8" t="s">
         <v>291</v>
       </c>
-      <c r="V265" s="12"/>
+      <c r="V265" s="11">
+        <v>46195</v>
+      </c>
       <c r="W265" s="9" t="s">
         <v>574</v>
       </c>
       <c r="X265" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y265" s="12"/>
     </row>
@@ -21109,9 +21121,11 @@
       <c r="B267" s="11">
         <v>46185.594386770834</v>
       </c>
-      <c r="C267" s="12"/>
+      <c r="C267" s="11">
+        <v>46196.89475716435</v>
+      </c>
       <c r="D267" s="11">
-        <v>46191.56830153935</v>
+        <v>46196.894821759255</v>
       </c>
       <c r="E267" s="12" t="s">
         <v>153</v>
@@ -21158,12 +21172,14 @@
       <c r="U267" s="8" t="s">
         <v>291</v>
       </c>
-      <c r="V267" s="12"/>
+      <c r="V267" s="11">
+        <v>46195</v>
+      </c>
       <c r="W267" s="9" t="s">
         <v>574</v>
       </c>
       <c r="X267" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y267" s="12"/>
     </row>

</xml_diff>

<commit_message>
Actualizar dashboard Oferta Zitron 2026 2026-06-24 20:26 UTC
</commit_message>
<xml_diff>
--- a/data_ofertas/Oferta Zitron 2026.xlsx
+++ b/data_ofertas/Oferta Zitron 2026.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4571" uniqueCount="599">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4619" uniqueCount="604">
   <si>
     <t>Oferta Zitron 2026</t>
   </si>
@@ -1809,6 +1809,21 @@
   </si>
   <si>
     <t>1215833063501310</t>
+  </si>
+  <si>
+    <t>1216019153661461</t>
+  </si>
+  <si>
+    <t>26CL0021</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26CL0021 </t>
+  </si>
+  <si>
+    <t>1216019372826832</t>
+  </si>
+  <si>
+    <t>1216019372826855</t>
   </si>
 </sst>
 </file>
@@ -2332,7 +2347,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Y279"/>
+  <dimension ref="A1:Y282"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10.4" customWidth="1"/>
@@ -15292,9 +15307,11 @@
       <c r="B184" s="5">
         <v>46162.838652314815</v>
       </c>
-      <c r="C184" s="6"/>
+      <c r="C184" s="5">
+        <v>46197.71481204861</v>
+      </c>
       <c r="D184" s="5">
-        <v>46188.70112761574</v>
+        <v>46197.715132233796</v>
       </c>
       <c r="E184" s="6" t="s">
         <v>40</v>
@@ -15345,12 +15362,14 @@
       <c r="U184" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="V184" s="6"/>
+      <c r="V184" s="5">
+        <v>46196</v>
+      </c>
       <c r="W184" s="9" t="s">
         <v>416</v>
       </c>
       <c r="X184" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y184" s="6"/>
     </row>
@@ -15361,9 +15380,11 @@
       <c r="B185" s="11">
         <v>46162.83865725694</v>
       </c>
-      <c r="C185" s="12"/>
+      <c r="C185" s="11">
+        <v>46197.715162106484</v>
+      </c>
       <c r="D185" s="11">
-        <v>46188.701169884254</v>
+        <v>46197.71554060185</v>
       </c>
       <c r="E185" s="12" t="s">
         <v>83</v>
@@ -15414,12 +15435,14 @@
       <c r="U185" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="V185" s="12"/>
+      <c r="V185" s="11">
+        <v>46196</v>
+      </c>
       <c r="W185" s="9" t="s">
         <v>416</v>
       </c>
       <c r="X185" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y185" s="12"/>
     </row>
@@ -15430,9 +15453,11 @@
       <c r="B186" s="5">
         <v>46162.83866952546</v>
       </c>
-      <c r="C186" s="6"/>
+      <c r="C186" s="5">
+        <v>46197.71534335648</v>
+      </c>
       <c r="D186" s="5">
-        <v>46188.70119445602</v>
+        <v>46197.7153894213</v>
       </c>
       <c r="E186" s="6" t="s">
         <v>153</v>
@@ -15483,12 +15508,14 @@
       <c r="U186" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="V186" s="6"/>
+      <c r="V186" s="5">
+        <v>46196</v>
+      </c>
       <c r="W186" s="9" t="s">
         <v>416</v>
       </c>
       <c r="X186" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y186" s="6"/>
     </row>
@@ -22020,6 +22047,201 @@
         <v>0</v>
       </c>
       <c r="Y279" s="12"/>
+    </row>
+    <row r="280" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A280" s="4" t="s">
+        <v>599</v>
+      </c>
+      <c r="B280" s="5">
+        <v>46197.84756534723</v>
+      </c>
+      <c r="C280" s="6"/>
+      <c r="D280" s="5">
+        <v>46197.84831641204</v>
+      </c>
+      <c r="E280" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F280" s="6" t="s">
+        <v>600</v>
+      </c>
+      <c r="G280" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H280" s="6"/>
+      <c r="I280" s="6"/>
+      <c r="J280" s="6"/>
+      <c r="K280" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="L280" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="M280" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N280" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="O280" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="P280" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q280" s="7" t="s">
+        <v>431</v>
+      </c>
+      <c r="R280" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S280" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="T280" s="6" t="s">
+        <v>601</v>
+      </c>
+      <c r="U280" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="V280" s="6"/>
+      <c r="W280" s="9" t="s">
+        <v>601</v>
+      </c>
+      <c r="X280" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y280" s="6"/>
+    </row>
+    <row r="281" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A281" s="10" t="s">
+        <v>602</v>
+      </c>
+      <c r="B281" s="11">
+        <v>46197.84758265046</v>
+      </c>
+      <c r="C281" s="12"/>
+      <c r="D281" s="11">
+        <v>46197.848316944444</v>
+      </c>
+      <c r="E281" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="F281" s="12" t="s">
+        <v>600</v>
+      </c>
+      <c r="G281" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="H281" s="12"/>
+      <c r="I281" s="12"/>
+      <c r="J281" s="12"/>
+      <c r="K281" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="L281" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="M281" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N281" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="O281" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="P281" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q281" s="7" t="s">
+        <v>431</v>
+      </c>
+      <c r="R281" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S281" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="T281" s="12" t="s">
+        <v>601</v>
+      </c>
+      <c r="U281" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="V281" s="12"/>
+      <c r="W281" s="9" t="s">
+        <v>601</v>
+      </c>
+      <c r="X281" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y281" s="12"/>
+    </row>
+    <row r="282" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A282" s="4" t="s">
+        <v>603</v>
+      </c>
+      <c r="B282" s="5">
+        <v>46197.84758912037</v>
+      </c>
+      <c r="C282" s="6"/>
+      <c r="D282" s="5">
+        <v>46197.84831748843</v>
+      </c>
+      <c r="E282" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="F282" s="6" t="s">
+        <v>600</v>
+      </c>
+      <c r="G282" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H282" s="6"/>
+      <c r="I282" s="6"/>
+      <c r="J282" s="6"/>
+      <c r="K282" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="L282" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="M282" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N282" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="O282" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="P282" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q282" s="7" t="s">
+        <v>431</v>
+      </c>
+      <c r="R282" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S282" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="T282" s="6" t="s">
+        <v>601</v>
+      </c>
+      <c r="U282" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="V282" s="6"/>
+      <c r="W282" s="9" t="s">
+        <v>601</v>
+      </c>
+      <c r="X282" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y282" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Actualizar dashboard Oferta Zitron 2026 2026-06-25 11:32 UTC
</commit_message>
<xml_diff>
--- a/data_ofertas/Oferta Zitron 2026.xlsx
+++ b/data_ofertas/Oferta Zitron 2026.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4712" uniqueCount="614">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4760" uniqueCount="620">
   <si>
     <t>Oferta Zitron 2026</t>
   </si>
@@ -1854,6 +1854,24 @@
   </si>
   <si>
     <t>1216020563809373</t>
+  </si>
+  <si>
+    <t>1216020821275355</t>
+  </si>
+  <si>
+    <t>AMM-ICL-0387-26-SOLICITUD DE OFERTA ARIS MINING MARMATO NIT 890.114.642</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARIS MINING MARMATO </t>
+  </si>
+  <si>
+    <t>AMM-ICL-0387-26</t>
+  </si>
+  <si>
+    <t>1216020673900356</t>
+  </si>
+  <si>
+    <t>1216020821252030</t>
   </si>
 </sst>
 </file>
@@ -2377,7 +2395,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Y288"/>
+  <dimension ref="A1:Y291"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10.4" customWidth="1"/>
@@ -22675,6 +22693,207 @@
       </c>
       <c r="Y288" s="6"/>
     </row>
+    <row r="289" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A289" s="10" t="s">
+        <v>614</v>
+      </c>
+      <c r="B289" s="11">
+        <v>46197.89618916667</v>
+      </c>
+      <c r="C289" s="12"/>
+      <c r="D289" s="11">
+        <v>46197.896865462964</v>
+      </c>
+      <c r="E289" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="F289" s="12" t="s">
+        <v>615</v>
+      </c>
+      <c r="G289" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="H289" s="12"/>
+      <c r="I289" s="12"/>
+      <c r="J289" s="11">
+        <v>46197</v>
+      </c>
+      <c r="K289" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="L289" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="M289" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N289" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="O289" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="P289" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q289" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="R289" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S289" s="12" t="s">
+        <v>616</v>
+      </c>
+      <c r="T289" s="12" t="s">
+        <v>617</v>
+      </c>
+      <c r="U289" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="V289" s="12"/>
+      <c r="W289" s="9" t="s">
+        <v>617</v>
+      </c>
+      <c r="X289" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y289" s="12"/>
+    </row>
+    <row r="290" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A290" s="4" t="s">
+        <v>618</v>
+      </c>
+      <c r="B290" s="5">
+        <v>46197.896195532405</v>
+      </c>
+      <c r="C290" s="6"/>
+      <c r="D290" s="5">
+        <v>46197.89686626157</v>
+      </c>
+      <c r="E290" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="F290" s="6" t="s">
+        <v>615</v>
+      </c>
+      <c r="G290" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H290" s="6"/>
+      <c r="I290" s="6"/>
+      <c r="J290" s="5">
+        <v>46197</v>
+      </c>
+      <c r="K290" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="L290" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="M290" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N290" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="O290" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="P290" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q290" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="R290" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S290" s="6" t="s">
+        <v>616</v>
+      </c>
+      <c r="T290" s="6" t="s">
+        <v>617</v>
+      </c>
+      <c r="U290" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="V290" s="6"/>
+      <c r="W290" s="9" t="s">
+        <v>617</v>
+      </c>
+      <c r="X290" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y290" s="6"/>
+    </row>
+    <row r="291" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A291" s="10" t="s">
+        <v>619</v>
+      </c>
+      <c r="B291" s="11">
+        <v>46197.89621086806</v>
+      </c>
+      <c r="C291" s="12"/>
+      <c r="D291" s="11">
+        <v>46197.896867083335</v>
+      </c>
+      <c r="E291" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="F291" s="12" t="s">
+        <v>615</v>
+      </c>
+      <c r="G291" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="H291" s="12"/>
+      <c r="I291" s="12"/>
+      <c r="J291" s="11">
+        <v>46197</v>
+      </c>
+      <c r="K291" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="L291" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="M291" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N291" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="O291" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="P291" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q291" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="R291" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S291" s="12" t="s">
+        <v>616</v>
+      </c>
+      <c r="T291" s="12" t="s">
+        <v>617</v>
+      </c>
+      <c r="U291" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="V291" s="12"/>
+      <c r="W291" s="9" t="s">
+        <v>617</v>
+      </c>
+      <c r="X291" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y291" s="12"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Actualizar dashboard Oferta Zitron 2026 2026-06-25 20:52 UTC
</commit_message>
<xml_diff>
--- a/data_ofertas/Oferta Zitron 2026.xlsx
+++ b/data_ofertas/Oferta Zitron 2026.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4760" uniqueCount="620">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4763" uniqueCount="620">
   <si>
     <t>Oferta Zitron 2026</t>
   </si>
@@ -22700,9 +22700,11 @@
       <c r="B289" s="11">
         <v>46197.89618916667</v>
       </c>
-      <c r="C289" s="12"/>
+      <c r="C289" s="11">
+        <v>46198.64821459491</v>
+      </c>
       <c r="D289" s="11">
-        <v>46197.896865462964</v>
+        <v>46198.77451392361</v>
       </c>
       <c r="E289" s="12" t="s">
         <v>40</v>
@@ -22711,9 +22713,11 @@
         <v>615</v>
       </c>
       <c r="G289" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H289" s="12"/>
+        <v>41</v>
+      </c>
+      <c r="H289" s="12" t="s">
+        <v>42</v>
+      </c>
       <c r="I289" s="12"/>
       <c r="J289" s="11">
         <v>46197</v>
@@ -22751,12 +22755,14 @@
       <c r="U289" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="V289" s="12"/>
+      <c r="V289" s="11">
+        <v>46198</v>
+      </c>
       <c r="W289" s="9" t="s">
         <v>617</v>
       </c>
       <c r="X289" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y289" s="12"/>
     </row>
@@ -22767,9 +22773,11 @@
       <c r="B290" s="5">
         <v>46197.896195532405</v>
       </c>
-      <c r="C290" s="6"/>
+      <c r="C290" s="5">
+        <v>46198.774273993055</v>
+      </c>
       <c r="D290" s="5">
-        <v>46197.89686626157</v>
+        <v>46198.77437046297</v>
       </c>
       <c r="E290" s="6" t="s">
         <v>83</v>
@@ -22778,9 +22786,11 @@
         <v>615</v>
       </c>
       <c r="G290" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H290" s="6"/>
+        <v>30</v>
+      </c>
+      <c r="H290" s="6" t="s">
+        <v>31</v>
+      </c>
       <c r="I290" s="6"/>
       <c r="J290" s="5">
         <v>46197</v>
@@ -22818,7 +22828,9 @@
       <c r="U290" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="V290" s="6"/>
+      <c r="V290" s="5">
+        <v>46198</v>
+      </c>
       <c r="W290" s="9" t="s">
         <v>617</v>
       </c>
@@ -22834,9 +22846,11 @@
       <c r="B291" s="11">
         <v>46197.89621086806</v>
       </c>
-      <c r="C291" s="12"/>
+      <c r="C291" s="11">
+        <v>46198.774317268515</v>
+      </c>
       <c r="D291" s="11">
-        <v>46197.896867083335</v>
+        <v>46198.77437126158</v>
       </c>
       <c r="E291" s="12" t="s">
         <v>153</v>
@@ -22845,9 +22859,11 @@
         <v>615</v>
       </c>
       <c r="G291" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H291" s="12"/>
+        <v>44</v>
+      </c>
+      <c r="H291" s="12" t="s">
+        <v>45</v>
+      </c>
       <c r="I291" s="12"/>
       <c r="J291" s="11">
         <v>46197</v>
@@ -22885,7 +22901,9 @@
       <c r="U291" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="V291" s="12"/>
+      <c r="V291" s="11">
+        <v>46198</v>
+      </c>
       <c r="W291" s="9" t="s">
         <v>617</v>
       </c>

</xml_diff>

<commit_message>
Actualizar dashboard Oferta Zitron 2026 2026-06-25 21:46 UTC
</commit_message>
<xml_diff>
--- a/data_ofertas/Oferta Zitron 2026.xlsx
+++ b/data_ofertas/Oferta Zitron 2026.xlsx
@@ -22505,9 +22505,11 @@
       <c r="B286" s="5">
         <v>46197.889788437504</v>
       </c>
-      <c r="C286" s="6"/>
+      <c r="C286" s="5">
+        <v>46198.895530497684</v>
+      </c>
       <c r="D286" s="5">
-        <v>46197.891620254624</v>
+        <v>46198.89609574074</v>
       </c>
       <c r="E286" s="6" t="s">
         <v>40</v>
@@ -22556,10 +22558,12 @@
       <c r="U286" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="V286" s="6"/>
+      <c r="V286" s="5">
+        <v>46198</v>
+      </c>
       <c r="W286" s="6"/>
       <c r="X286" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y286" s="6"/>
     </row>
@@ -22570,9 +22574,11 @@
       <c r="B287" s="11">
         <v>46197.88979412037</v>
       </c>
-      <c r="C287" s="12"/>
+      <c r="C287" s="11">
+        <v>46198.90061689814</v>
+      </c>
       <c r="D287" s="11">
-        <v>46197.89162122685</v>
+        <v>46198.90063583333</v>
       </c>
       <c r="E287" s="12" t="s">
         <v>83</v>
@@ -22621,7 +22627,9 @@
       <c r="U287" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="V287" s="12"/>
+      <c r="V287" s="11">
+        <v>46198</v>
+      </c>
       <c r="W287" s="12"/>
       <c r="X287" s="12">
         <v>0</v>
@@ -22637,7 +22645,7 @@
       </c>
       <c r="C288" s="6"/>
       <c r="D288" s="5">
-        <v>46197.89162207176</v>
+        <v>46198.90062260417</v>
       </c>
       <c r="E288" s="6" t="s">
         <v>153</v>

</xml_diff>

<commit_message>
Actualizar dashboard Oferta Zitron 2026 2026-06-26 17:42 UTC
</commit_message>
<xml_diff>
--- a/data_ofertas/Oferta Zitron 2026.xlsx
+++ b/data_ofertas/Oferta Zitron 2026.xlsx
@@ -15282,7 +15282,7 @@
         <v>46185.588656064814</v>
       </c>
       <c r="D183" s="11">
-        <v>46185.61357857639</v>
+        <v>46199.63779241898</v>
       </c>
       <c r="E183" s="12" t="s">
         <v>153</v>
@@ -15332,7 +15332,7 @@
         <v>95</v>
       </c>
       <c r="V183" s="11">
-        <v>46185</v>
+        <v>46199</v>
       </c>
       <c r="W183" s="9" t="s">
         <v>411</v>

</xml_diff>

<commit_message>
Actualizar dashboard Oferta Zitron 2026 2026-06-30 20:50 UTC
</commit_message>
<xml_diff>
--- a/data_ofertas/Oferta Zitron 2026.xlsx
+++ b/data_ofertas/Oferta Zitron 2026.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4763" uniqueCount="620">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4991" uniqueCount="648">
   <si>
     <t>Oferta Zitron 2026</t>
   </si>
@@ -1872,6 +1872,90 @@
   </si>
   <si>
     <t>1216020821252030</t>
+  </si>
+  <si>
+    <t>1216153835287402</t>
+  </si>
+  <si>
+    <t>Pedido de cotización ref. 18959 - 26AR0004.C</t>
+  </si>
+  <si>
+    <t>TEVA</t>
+  </si>
+  <si>
+    <t>26AR0004.C</t>
+  </si>
+  <si>
+    <t>1216153783207656</t>
+  </si>
+  <si>
+    <t>1216154224301517</t>
+  </si>
+  <si>
+    <t>1216158539911859</t>
+  </si>
+  <si>
+    <t>25MX0053 - Cotización Ventiladores principales</t>
+  </si>
+  <si>
+    <t>FIRST MAJESTIC ERMITAÑO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25MX0053 </t>
+  </si>
+  <si>
+    <t>1216158500910395</t>
+  </si>
+  <si>
+    <t>1216158540533988</t>
+  </si>
+  <si>
+    <t>1216158824888315</t>
+  </si>
+  <si>
+    <t>Propuesta de ventilador// Minera Sabinas</t>
+  </si>
+  <si>
+    <t>Minera Sabinas</t>
+  </si>
+  <si>
+    <t>1216158824888333</t>
+  </si>
+  <si>
+    <t>1216158793653329</t>
+  </si>
+  <si>
+    <t>1216159042290314</t>
+  </si>
+  <si>
+    <t>NP0000000115238  (RQ2040000000090 Ventilador axial 21 m3/h)</t>
+  </si>
+  <si>
+    <t>INDUSTRIA PEÑOLES</t>
+  </si>
+  <si>
+    <t>1216159042511179</t>
+  </si>
+  <si>
+    <t>1216159042508937</t>
+  </si>
+  <si>
+    <t>1216191030213996</t>
+  </si>
+  <si>
+    <t>26CL0022.C - Precio orientativo jetfans - Túnel Chile</t>
+  </si>
+  <si>
+    <t>SENER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26CL0022.C </t>
+  </si>
+  <si>
+    <t>1216191030190567</t>
+  </si>
+  <si>
+    <t>1216191030297671</t>
   </si>
 </sst>
 </file>
@@ -2395,7 +2479,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Y291"/>
+  <dimension ref="A1:Y306"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10.4" customWidth="1"/>
@@ -20847,9 +20931,11 @@
       <c r="B262" s="5">
         <v>46185.55686909722</v>
       </c>
-      <c r="C262" s="6"/>
+      <c r="C262" s="5">
+        <v>46203.545441504626</v>
+      </c>
       <c r="D262" s="5">
-        <v>46185.558165486116</v>
+        <v>46203.54575012732</v>
       </c>
       <c r="E262" s="6" t="s">
         <v>40</v>
@@ -20898,12 +20984,14 @@
       <c r="U262" s="8" t="s">
         <v>291</v>
       </c>
-      <c r="V262" s="6"/>
+      <c r="V262" s="5">
+        <v>46193</v>
+      </c>
       <c r="W262" s="9" t="s">
         <v>568</v>
       </c>
       <c r="X262" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y262" s="6"/>
     </row>
@@ -20916,7 +21004,7 @@
       </c>
       <c r="C263" s="12"/>
       <c r="D263" s="11">
-        <v>46185.5581987037</v>
+        <v>46203.54554041667</v>
       </c>
       <c r="E263" s="12" t="s">
         <v>83</v>
@@ -20983,7 +21071,7 @@
       </c>
       <c r="C264" s="6"/>
       <c r="D264" s="5">
-        <v>46185.558236666664</v>
+        <v>46203.545551435185</v>
       </c>
       <c r="E264" s="6" t="s">
         <v>153</v>
@@ -22919,6 +23007,981 @@
         <v>0</v>
       </c>
       <c r="Y291" s="12"/>
+    </row>
+    <row r="292" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A292" s="4" t="s">
+        <v>620</v>
+      </c>
+      <c r="B292" s="5">
+        <v>46203.546952488425</v>
+      </c>
+      <c r="C292" s="6"/>
+      <c r="D292" s="5">
+        <v>46203.610333379635</v>
+      </c>
+      <c r="E292" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F292" s="6" t="s">
+        <v>621</v>
+      </c>
+      <c r="G292" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H292" s="6"/>
+      <c r="I292" s="6"/>
+      <c r="J292" s="5">
+        <v>46198</v>
+      </c>
+      <c r="K292" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="L292" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="M292" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N292" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="O292" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="P292" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q292" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="R292" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S292" s="6" t="s">
+        <v>622</v>
+      </c>
+      <c r="T292" s="6" t="s">
+        <v>623</v>
+      </c>
+      <c r="U292" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="V292" s="6"/>
+      <c r="W292" s="9" t="s">
+        <v>623</v>
+      </c>
+      <c r="X292" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y292" s="6"/>
+    </row>
+    <row r="293" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A293" s="10" t="s">
+        <v>624</v>
+      </c>
+      <c r="B293" s="11">
+        <v>46203.54697321759</v>
+      </c>
+      <c r="C293" s="12"/>
+      <c r="D293" s="11">
+        <v>46203.61033358796</v>
+      </c>
+      <c r="E293" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="F293" s="12" t="s">
+        <v>621</v>
+      </c>
+      <c r="G293" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="H293" s="12"/>
+      <c r="I293" s="12"/>
+      <c r="J293" s="11">
+        <v>46198</v>
+      </c>
+      <c r="K293" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="L293" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="M293" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N293" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="O293" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="P293" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q293" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="R293" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S293" s="12" t="s">
+        <v>622</v>
+      </c>
+      <c r="T293" s="12" t="s">
+        <v>623</v>
+      </c>
+      <c r="U293" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="V293" s="12"/>
+      <c r="W293" s="9" t="s">
+        <v>623</v>
+      </c>
+      <c r="X293" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y293" s="12"/>
+    </row>
+    <row r="294" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A294" s="4" t="s">
+        <v>625</v>
+      </c>
+      <c r="B294" s="5">
+        <v>46203.54697938658</v>
+      </c>
+      <c r="C294" s="6"/>
+      <c r="D294" s="5">
+        <v>46203.61033452547</v>
+      </c>
+      <c r="E294" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="F294" s="6" t="s">
+        <v>621</v>
+      </c>
+      <c r="G294" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H294" s="6"/>
+      <c r="I294" s="6"/>
+      <c r="J294" s="5">
+        <v>46198</v>
+      </c>
+      <c r="K294" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="L294" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="M294" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N294" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="O294" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="P294" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q294" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="R294" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S294" s="6" t="s">
+        <v>622</v>
+      </c>
+      <c r="T294" s="6" t="s">
+        <v>623</v>
+      </c>
+      <c r="U294" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="V294" s="6"/>
+      <c r="W294" s="9" t="s">
+        <v>623</v>
+      </c>
+      <c r="X294" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y294" s="6"/>
+    </row>
+    <row r="295" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A295" s="10" t="s">
+        <v>626</v>
+      </c>
+      <c r="B295" s="11">
+        <v>46203.60974886574</v>
+      </c>
+      <c r="C295" s="12"/>
+      <c r="D295" s="11">
+        <v>46203.79287297453</v>
+      </c>
+      <c r="E295" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="F295" s="12" t="s">
+        <v>627</v>
+      </c>
+      <c r="G295" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="H295" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="I295" s="12"/>
+      <c r="J295" s="11">
+        <v>46203</v>
+      </c>
+      <c r="K295" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="L295" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="M295" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N295" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="O295" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="P295" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q295" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="R295" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S295" s="12" t="s">
+        <v>628</v>
+      </c>
+      <c r="T295" s="12" t="s">
+        <v>629</v>
+      </c>
+      <c r="U295" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="V295" s="12"/>
+      <c r="W295" s="9" t="s">
+        <v>629</v>
+      </c>
+      <c r="X295" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y295" s="12"/>
+    </row>
+    <row r="296" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A296" s="4" t="s">
+        <v>630</v>
+      </c>
+      <c r="B296" s="5">
+        <v>46203.60975423611</v>
+      </c>
+      <c r="C296" s="6"/>
+      <c r="D296" s="5">
+        <v>46203.79298378472</v>
+      </c>
+      <c r="E296" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="F296" s="6" t="s">
+        <v>627</v>
+      </c>
+      <c r="G296" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="H296" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="I296" s="6"/>
+      <c r="J296" s="5">
+        <v>46203</v>
+      </c>
+      <c r="K296" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="L296" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="M296" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N296" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="O296" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="P296" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q296" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="R296" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S296" s="6" t="s">
+        <v>628</v>
+      </c>
+      <c r="T296" s="6" t="s">
+        <v>629</v>
+      </c>
+      <c r="U296" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="V296" s="6"/>
+      <c r="W296" s="9" t="s">
+        <v>629</v>
+      </c>
+      <c r="X296" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y296" s="6"/>
+    </row>
+    <row r="297" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A297" s="10" t="s">
+        <v>631</v>
+      </c>
+      <c r="B297" s="11">
+        <v>46203.609769965275</v>
+      </c>
+      <c r="C297" s="12"/>
+      <c r="D297" s="11">
+        <v>46203.79292857639</v>
+      </c>
+      <c r="E297" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="F297" s="12" t="s">
+        <v>627</v>
+      </c>
+      <c r="G297" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="H297" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="I297" s="12"/>
+      <c r="J297" s="11">
+        <v>46203</v>
+      </c>
+      <c r="K297" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="L297" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="M297" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N297" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="O297" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="P297" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q297" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="R297" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S297" s="12" t="s">
+        <v>628</v>
+      </c>
+      <c r="T297" s="12" t="s">
+        <v>629</v>
+      </c>
+      <c r="U297" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="V297" s="12"/>
+      <c r="W297" s="9" t="s">
+        <v>629</v>
+      </c>
+      <c r="X297" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y297" s="12"/>
+    </row>
+    <row r="298" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A298" s="4" t="s">
+        <v>632</v>
+      </c>
+      <c r="B298" s="5">
+        <v>46203.61393550926</v>
+      </c>
+      <c r="C298" s="6"/>
+      <c r="D298" s="5">
+        <v>46203.61470467593</v>
+      </c>
+      <c r="E298" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F298" s="6" t="s">
+        <v>633</v>
+      </c>
+      <c r="G298" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H298" s="6"/>
+      <c r="I298" s="6"/>
+      <c r="J298" s="5">
+        <v>46203</v>
+      </c>
+      <c r="K298" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="L298" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="M298" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N298" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="O298" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="P298" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q298" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="R298" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S298" s="6" t="s">
+        <v>634</v>
+      </c>
+      <c r="T298" s="6"/>
+      <c r="U298" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="V298" s="6"/>
+      <c r="W298" s="6"/>
+      <c r="X298" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y298" s="6"/>
+    </row>
+    <row r="299" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A299" s="10" t="s">
+        <v>635</v>
+      </c>
+      <c r="B299" s="11">
+        <v>46203.61394043981</v>
+      </c>
+      <c r="C299" s="12"/>
+      <c r="D299" s="11">
+        <v>46203.61470534722</v>
+      </c>
+      <c r="E299" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="F299" s="12" t="s">
+        <v>633</v>
+      </c>
+      <c r="G299" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="H299" s="12"/>
+      <c r="I299" s="12"/>
+      <c r="J299" s="11">
+        <v>46203</v>
+      </c>
+      <c r="K299" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="L299" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="M299" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N299" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="O299" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="P299" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q299" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="R299" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S299" s="12" t="s">
+        <v>634</v>
+      </c>
+      <c r="T299" s="12"/>
+      <c r="U299" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="V299" s="12"/>
+      <c r="W299" s="12"/>
+      <c r="X299" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y299" s="12"/>
+    </row>
+    <row r="300" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A300" s="4" t="s">
+        <v>636</v>
+      </c>
+      <c r="B300" s="5">
+        <v>46203.61395409722</v>
+      </c>
+      <c r="C300" s="6"/>
+      <c r="D300" s="5">
+        <v>46203.6147059375</v>
+      </c>
+      <c r="E300" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="F300" s="6" t="s">
+        <v>633</v>
+      </c>
+      <c r="G300" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H300" s="6"/>
+      <c r="I300" s="6"/>
+      <c r="J300" s="5">
+        <v>46203</v>
+      </c>
+      <c r="K300" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="L300" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="M300" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N300" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="O300" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="P300" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q300" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="R300" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S300" s="6" t="s">
+        <v>634</v>
+      </c>
+      <c r="T300" s="6"/>
+      <c r="U300" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="V300" s="6"/>
+      <c r="W300" s="6"/>
+      <c r="X300" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y300" s="6"/>
+    </row>
+    <row r="301" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A301" s="10" t="s">
+        <v>637</v>
+      </c>
+      <c r="B301" s="11">
+        <v>46203.61614737268</v>
+      </c>
+      <c r="C301" s="12"/>
+      <c r="D301" s="11">
+        <v>46203.61846347222</v>
+      </c>
+      <c r="E301" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="F301" s="12" t="s">
+        <v>638</v>
+      </c>
+      <c r="G301" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="H301" s="12"/>
+      <c r="I301" s="12"/>
+      <c r="J301" s="11">
+        <v>46203</v>
+      </c>
+      <c r="K301" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="L301" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="M301" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N301" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="O301" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="P301" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q301" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="R301" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S301" s="12" t="s">
+        <v>639</v>
+      </c>
+      <c r="T301" s="12"/>
+      <c r="U301" s="12"/>
+      <c r="V301" s="12"/>
+      <c r="W301" s="12"/>
+      <c r="X301" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y301" s="12"/>
+    </row>
+    <row r="302" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A302" s="4" t="s">
+        <v>640</v>
+      </c>
+      <c r="B302" s="5">
+        <v>46203.6161543287</v>
+      </c>
+      <c r="C302" s="6"/>
+      <c r="D302" s="5">
+        <v>46203.618463680556</v>
+      </c>
+      <c r="E302" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="F302" s="6" t="s">
+        <v>638</v>
+      </c>
+      <c r="G302" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H302" s="6"/>
+      <c r="I302" s="6"/>
+      <c r="J302" s="5">
+        <v>46203</v>
+      </c>
+      <c r="K302" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="L302" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="M302" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N302" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="O302" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="P302" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q302" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="R302" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S302" s="6" t="s">
+        <v>639</v>
+      </c>
+      <c r="T302" s="6"/>
+      <c r="U302" s="6"/>
+      <c r="V302" s="6"/>
+      <c r="W302" s="6"/>
+      <c r="X302" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y302" s="6"/>
+    </row>
+    <row r="303" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A303" s="10" t="s">
+        <v>641</v>
+      </c>
+      <c r="B303" s="11">
+        <v>46203.616170381945</v>
+      </c>
+      <c r="C303" s="12"/>
+      <c r="D303" s="11">
+        <v>46203.61846380787</v>
+      </c>
+      <c r="E303" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="F303" s="12" t="s">
+        <v>638</v>
+      </c>
+      <c r="G303" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="H303" s="12"/>
+      <c r="I303" s="12"/>
+      <c r="J303" s="11">
+        <v>46203</v>
+      </c>
+      <c r="K303" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="L303" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="M303" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N303" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="O303" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="P303" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q303" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="R303" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S303" s="12" t="s">
+        <v>639</v>
+      </c>
+      <c r="T303" s="12"/>
+      <c r="U303" s="12"/>
+      <c r="V303" s="12"/>
+      <c r="W303" s="12"/>
+      <c r="X303" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y303" s="12"/>
+    </row>
+    <row r="304" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A304" s="4" t="s">
+        <v>642</v>
+      </c>
+      <c r="B304" s="5">
+        <v>46203.800516655094</v>
+      </c>
+      <c r="C304" s="6"/>
+      <c r="D304" s="5">
+        <v>46203.801443634264</v>
+      </c>
+      <c r="E304" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F304" s="6" t="s">
+        <v>643</v>
+      </c>
+      <c r="G304" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H304" s="6"/>
+      <c r="I304" s="6"/>
+      <c r="J304" s="6"/>
+      <c r="K304" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="L304" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="M304" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N304" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="O304" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="P304" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q304" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="R304" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S304" s="6" t="s">
+        <v>644</v>
+      </c>
+      <c r="T304" s="6" t="s">
+        <v>645</v>
+      </c>
+      <c r="U304" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="V304" s="6"/>
+      <c r="W304" s="9" t="s">
+        <v>645</v>
+      </c>
+      <c r="X304" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y304" s="6"/>
+    </row>
+    <row r="305" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A305" s="10" t="s">
+        <v>646</v>
+      </c>
+      <c r="B305" s="11">
+        <v>46203.80053320602</v>
+      </c>
+      <c r="C305" s="12"/>
+      <c r="D305" s="11">
+        <v>46203.80144418981</v>
+      </c>
+      <c r="E305" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="F305" s="12" t="s">
+        <v>643</v>
+      </c>
+      <c r="G305" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="H305" s="12"/>
+      <c r="I305" s="12"/>
+      <c r="J305" s="12"/>
+      <c r="K305" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="L305" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="M305" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N305" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="O305" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="P305" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q305" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="R305" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S305" s="12" t="s">
+        <v>644</v>
+      </c>
+      <c r="T305" s="12" t="s">
+        <v>645</v>
+      </c>
+      <c r="U305" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="V305" s="12"/>
+      <c r="W305" s="9" t="s">
+        <v>645</v>
+      </c>
+      <c r="X305" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y305" s="12"/>
+    </row>
+    <row r="306" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A306" s="4" t="s">
+        <v>647</v>
+      </c>
+      <c r="B306" s="5">
+        <v>46203.80053798611</v>
+      </c>
+      <c r="C306" s="6"/>
+      <c r="D306" s="5">
+        <v>46203.80144469907</v>
+      </c>
+      <c r="E306" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="F306" s="6" t="s">
+        <v>643</v>
+      </c>
+      <c r="G306" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H306" s="6"/>
+      <c r="I306" s="6"/>
+      <c r="J306" s="6"/>
+      <c r="K306" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="L306" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="M306" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N306" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="O306" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="P306" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q306" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="R306" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S306" s="6" t="s">
+        <v>644</v>
+      </c>
+      <c r="T306" s="6" t="s">
+        <v>645</v>
+      </c>
+      <c r="U306" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="V306" s="6"/>
+      <c r="W306" s="9" t="s">
+        <v>645</v>
+      </c>
+      <c r="X306" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y306" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Actualizar dashboard Oferta Zitron 2026 2026-06-30 21:41 UTC
</commit_message>
<xml_diff>
--- a/data_ofertas/Oferta Zitron 2026.xlsx
+++ b/data_ofertas/Oferta Zitron 2026.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4991" uniqueCount="648">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4997" uniqueCount="648">
   <si>
     <t>Oferta Zitron 2026</t>
   </si>
@@ -23425,7 +23425,7 @@
       </c>
       <c r="C298" s="6"/>
       <c r="D298" s="5">
-        <v>46203.61470467593</v>
+        <v>46203.8987362037</v>
       </c>
       <c r="E298" s="6" t="s">
         <v>40</v>
@@ -23434,9 +23434,11 @@
         <v>633</v>
       </c>
       <c r="G298" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H298" s="6"/>
+        <v>56</v>
+      </c>
+      <c r="H298" s="6" t="s">
+        <v>57</v>
+      </c>
       <c r="I298" s="6"/>
       <c r="J298" s="5">
         <v>46203</v>
@@ -23488,7 +23490,7 @@
       </c>
       <c r="C299" s="12"/>
       <c r="D299" s="11">
-        <v>46203.61470534722</v>
+        <v>46203.898774710644</v>
       </c>
       <c r="E299" s="12" t="s">
         <v>83</v>
@@ -23497,9 +23499,11 @@
         <v>633</v>
       </c>
       <c r="G299" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H299" s="12"/>
+        <v>30</v>
+      </c>
+      <c r="H299" s="12" t="s">
+        <v>31</v>
+      </c>
       <c r="I299" s="12"/>
       <c r="J299" s="11">
         <v>46203</v>
@@ -23551,7 +23555,7 @@
       </c>
       <c r="C300" s="6"/>
       <c r="D300" s="5">
-        <v>46203.6147059375</v>
+        <v>46203.89882076389</v>
       </c>
       <c r="E300" s="6" t="s">
         <v>153</v>
@@ -23560,9 +23564,11 @@
         <v>633</v>
       </c>
       <c r="G300" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H300" s="6"/>
+        <v>44</v>
+      </c>
+      <c r="H300" s="6" t="s">
+        <v>45</v>
+      </c>
       <c r="I300" s="6"/>
       <c r="J300" s="5">
         <v>46203</v>
@@ -23614,7 +23620,7 @@
       </c>
       <c r="C301" s="12"/>
       <c r="D301" s="11">
-        <v>46203.61846347222</v>
+        <v>46203.898326435185</v>
       </c>
       <c r="E301" s="12" t="s">
         <v>40</v>
@@ -23623,9 +23629,11 @@
         <v>638</v>
       </c>
       <c r="G301" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H301" s="12"/>
+        <v>56</v>
+      </c>
+      <c r="H301" s="12" t="s">
+        <v>57</v>
+      </c>
       <c r="I301" s="12"/>
       <c r="J301" s="11">
         <v>46203</v>
@@ -23675,7 +23683,7 @@
       </c>
       <c r="C302" s="6"/>
       <c r="D302" s="5">
-        <v>46203.618463680556</v>
+        <v>46203.898378391204</v>
       </c>
       <c r="E302" s="6" t="s">
         <v>83</v>
@@ -23684,9 +23692,11 @@
         <v>638</v>
       </c>
       <c r="G302" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H302" s="6"/>
+        <v>30</v>
+      </c>
+      <c r="H302" s="6" t="s">
+        <v>31</v>
+      </c>
       <c r="I302" s="6"/>
       <c r="J302" s="5">
         <v>46203</v>
@@ -23736,7 +23746,7 @@
       </c>
       <c r="C303" s="12"/>
       <c r="D303" s="11">
-        <v>46203.61846380787</v>
+        <v>46203.89842915509</v>
       </c>
       <c r="E303" s="12" t="s">
         <v>153</v>
@@ -23745,9 +23755,11 @@
         <v>638</v>
       </c>
       <c r="G303" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H303" s="12"/>
+        <v>44</v>
+      </c>
+      <c r="H303" s="12" t="s">
+        <v>45</v>
+      </c>
       <c r="I303" s="12"/>
       <c r="J303" s="11">
         <v>46203</v>

</xml_diff>

<commit_message>
Actualizar dashboard Oferta Zitron 2026 2026-07-02 21:11 UTC
</commit_message>
<xml_diff>
--- a/data_ofertas/Oferta Zitron 2026.xlsx
+++ b/data_ofertas/Oferta Zitron 2026.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4997" uniqueCount="648">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5053" uniqueCount="656">
   <si>
     <t>Oferta Zitron 2026</t>
   </si>
@@ -1283,6 +1283,9 @@
     <t>26CL0063</t>
   </si>
   <si>
+    <t xml:space="preserve">Se actualiza oferta a rev 01 </t>
+  </si>
+  <si>
     <t>1214984682367741</t>
   </si>
   <si>
@@ -1934,6 +1937,9 @@
     <t>INDUSTRIA PEÑOLES</t>
   </si>
   <si>
+    <t>26MX0060B</t>
+  </si>
+  <si>
     <t>1216159042511179</t>
   </si>
   <si>
@@ -1956,6 +1962,24 @@
   </si>
   <si>
     <t>1216191030297671</t>
+  </si>
+  <si>
+    <t>1216245413951120</t>
+  </si>
+  <si>
+    <t>26CO0020 - Ventilador microtúneles Colombia</t>
+  </si>
+  <si>
+    <t>ydn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26CO0020 </t>
+  </si>
+  <si>
+    <t>1216245469559473</t>
+  </si>
+  <si>
+    <t>1216245532454105</t>
   </si>
 </sst>
 </file>
@@ -2479,7 +2503,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Y306"/>
+  <dimension ref="A1:Y309"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10.4" customWidth="1"/>
@@ -3037,9 +3061,11 @@
       <c r="B10" s="5">
         <v>46146.57326584491</v>
       </c>
-      <c r="C10" s="6"/>
+      <c r="C10" s="5">
+        <v>46205.54033820602</v>
+      </c>
       <c r="D10" s="5">
-        <v>46180.57965107639</v>
+        <v>46205.54033991898</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>40</v>
@@ -3175,9 +3201,11 @@
       <c r="B12" s="5">
         <v>46146.5732847801</v>
       </c>
-      <c r="C12" s="6"/>
+      <c r="C12" s="5">
+        <v>46205.540224571756</v>
+      </c>
       <c r="D12" s="5">
-        <v>46146.65420983796</v>
+        <v>46205.54034552083</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>33</v>
@@ -8203,9 +8231,11 @@
       <c r="B82" s="5">
         <v>46141.626975983796</v>
       </c>
-      <c r="C82" s="6"/>
+      <c r="C82" s="5">
+        <v>46205.53906976852</v>
+      </c>
       <c r="D82" s="5">
-        <v>46178.90033945601</v>
+        <v>46205.539071493055</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>40</v>
@@ -8343,7 +8373,7 @@
       </c>
       <c r="C84" s="6"/>
       <c r="D84" s="5">
-        <v>46155.83295511574</v>
+        <v>46205.539076932866</v>
       </c>
       <c r="E84" s="6" t="s">
         <v>153</v>
@@ -12859,9 +12889,11 @@
       <c r="B148" s="5">
         <v>46154.766096377316</v>
       </c>
-      <c r="C148" s="6"/>
+      <c r="C148" s="5">
+        <v>46205.53888810185</v>
+      </c>
       <c r="D148" s="5">
-        <v>46155.83762229167</v>
+        <v>46205.53888976852</v>
       </c>
       <c r="E148" s="6" t="s">
         <v>40</v>
@@ -12999,7 +13031,7 @@
       </c>
       <c r="C150" s="6"/>
       <c r="D150" s="5">
-        <v>46155.83770071759</v>
+        <v>46205.53889347222</v>
       </c>
       <c r="E150" s="6" t="s">
         <v>153</v>
@@ -15644,7 +15676,7 @@
         <v>46197.71481204861</v>
       </c>
       <c r="D187" s="11">
-        <v>46197.715132233796</v>
+        <v>46205.7077784838</v>
       </c>
       <c r="E187" s="12" t="s">
         <v>40</v>
@@ -15696,7 +15728,7 @@
         <v>95</v>
       </c>
       <c r="V187" s="11">
-        <v>46196</v>
+        <v>46205</v>
       </c>
       <c r="W187" s="9" t="s">
         <v>422</v>
@@ -15704,11 +15736,13 @@
       <c r="X187" s="12">
         <v>1</v>
       </c>
-      <c r="Y187" s="12"/>
+      <c r="Y187" s="12" t="s">
+        <v>423</v>
+      </c>
     </row>
     <row r="188" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A188" s="4" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="B188" s="5">
         <v>46162.83865725694</v>
@@ -15781,7 +15815,7 @@
     </row>
     <row r="189" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A189" s="10" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="B189" s="11">
         <v>46162.83866952546</v>
@@ -15854,7 +15888,7 @@
     </row>
     <row r="190" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A190" s="4" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="B190" s="5">
         <v>46162.84063533565</v>
@@ -15869,7 +15903,7 @@
         <v>40</v>
       </c>
       <c r="F190" s="6" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="G190" s="6" t="s">
         <v>41</v>
@@ -15906,10 +15940,10 @@
         <v>35</v>
       </c>
       <c r="S190" s="6" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="T190" s="6" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="U190" s="8" t="s">
         <v>38</v>
@@ -15918,7 +15952,7 @@
         <v>46162</v>
       </c>
       <c r="W190" s="9" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="X190" s="6">
         <v>1</v>
@@ -15927,7 +15961,7 @@
     </row>
     <row r="191" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A191" s="10" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="B191" s="11">
         <v>46162.84063988426</v>
@@ -15942,7 +15976,7 @@
         <v>83</v>
       </c>
       <c r="F191" s="12" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="G191" s="12" t="s">
         <v>30</v>
@@ -15979,10 +16013,10 @@
         <v>35</v>
       </c>
       <c r="S191" s="12" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="T191" s="12" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="U191" s="8" t="s">
         <v>38</v>
@@ -15991,7 +16025,7 @@
         <v>46166</v>
       </c>
       <c r="W191" s="9" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="X191" s="12">
         <v>1</v>
@@ -16000,7 +16034,7 @@
     </row>
     <row r="192" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A192" s="4" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="B192" s="5">
         <v>46162.84065267361</v>
@@ -16015,7 +16049,7 @@
         <v>153</v>
       </c>
       <c r="F192" s="6" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="G192" s="6" t="s">
         <v>44</v>
@@ -16052,10 +16086,10 @@
         <v>35</v>
       </c>
       <c r="S192" s="6" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="T192" s="6" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="U192" s="8" t="s">
         <v>38</v>
@@ -16064,7 +16098,7 @@
         <v>46167</v>
       </c>
       <c r="W192" s="9" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="X192" s="6">
         <v>1</v>
@@ -16073,7 +16107,7 @@
     </row>
     <row r="193" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A193" s="10" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="B193" s="11">
         <v>46162.901056585644</v>
@@ -16088,7 +16122,7 @@
         <v>40</v>
       </c>
       <c r="F193" s="12" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="G193" s="12" t="s">
         <v>32</v>
@@ -16124,7 +16158,7 @@
       </c>
       <c r="S193" s="12"/>
       <c r="T193" s="12" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="U193" s="8" t="s">
         <v>95</v>
@@ -16133,18 +16167,18 @@
         <v>46176</v>
       </c>
       <c r="W193" s="9" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="X193" s="12">
         <v>1</v>
       </c>
       <c r="Y193" s="12" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
     </row>
     <row r="194" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A194" s="4" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="B194" s="5">
         <v>46162.9010628588</v>
@@ -16159,7 +16193,7 @@
         <v>83</v>
       </c>
       <c r="F194" s="6" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="G194" s="6" t="s">
         <v>32</v>
@@ -16195,7 +16229,7 @@
       </c>
       <c r="S194" s="6"/>
       <c r="T194" s="6" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="U194" s="8" t="s">
         <v>95</v>
@@ -16204,7 +16238,7 @@
         <v>46169</v>
       </c>
       <c r="W194" s="9" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="X194" s="6">
         <v>1</v>
@@ -16213,7 +16247,7 @@
     </row>
     <row r="195" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A195" s="10" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="B195" s="11">
         <v>46162.90107537037</v>
@@ -16228,7 +16262,7 @@
         <v>153</v>
       </c>
       <c r="F195" s="12" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="G195" s="12" t="s">
         <v>32</v>
@@ -16263,10 +16297,10 @@
         <v>35</v>
       </c>
       <c r="S195" s="12" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="T195" s="12" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="U195" s="8" t="s">
         <v>95</v>
@@ -16275,7 +16309,7 @@
         <v>46176</v>
       </c>
       <c r="W195" s="9" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="X195" s="12">
         <v>0</v>
@@ -16284,7 +16318,7 @@
     </row>
     <row r="196" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A196" s="4" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="B196" s="5">
         <v>46166.90447782408</v>
@@ -16297,7 +16331,7 @@
         <v>40</v>
       </c>
       <c r="F196" s="6" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="G196" s="6" t="s">
         <v>32</v>
@@ -16332,17 +16366,17 @@
         <v>35</v>
       </c>
       <c r="S196" s="6" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="T196" s="6" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="U196" s="8" t="s">
         <v>95</v>
       </c>
       <c r="V196" s="6"/>
       <c r="W196" s="9" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="X196" s="6">
         <v>0</v>
@@ -16351,7 +16385,7 @@
     </row>
     <row r="197" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A197" s="10" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="B197" s="11">
         <v>46166.904482638885</v>
@@ -16366,7 +16400,7 @@
         <v>83</v>
       </c>
       <c r="F197" s="12" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="G197" s="12" t="s">
         <v>32</v>
@@ -16401,10 +16435,10 @@
         <v>35</v>
       </c>
       <c r="S197" s="12" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="T197" s="12" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="U197" s="8" t="s">
         <v>95</v>
@@ -16413,7 +16447,7 @@
         <v>46171</v>
       </c>
       <c r="W197" s="9" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="X197" s="12">
         <v>0</v>
@@ -16422,7 +16456,7 @@
     </row>
     <row r="198" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A198" s="4" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="B198" s="5">
         <v>46166.904495173614</v>
@@ -16435,7 +16469,7 @@
         <v>153</v>
       </c>
       <c r="F198" s="6" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="G198" s="6" t="s">
         <v>32</v>
@@ -16470,17 +16504,17 @@
         <v>35</v>
       </c>
       <c r="S198" s="6" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="T198" s="6" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="U198" s="8" t="s">
         <v>95</v>
       </c>
       <c r="V198" s="6"/>
       <c r="W198" s="9" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="X198" s="6">
         <v>0</v>
@@ -16489,7 +16523,7 @@
     </row>
     <row r="199" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A199" s="10" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="B199" s="11">
         <v>46166.90582966435</v>
@@ -16502,7 +16536,7 @@
         <v>40</v>
       </c>
       <c r="F199" s="12" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="G199" s="12" t="s">
         <v>32</v>
@@ -16537,17 +16571,17 @@
         <v>35</v>
       </c>
       <c r="S199" s="12" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="T199" s="12" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="U199" s="8" t="s">
         <v>95</v>
       </c>
       <c r="V199" s="12"/>
       <c r="W199" s="9" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="X199" s="12">
         <v>0</v>
@@ -16556,7 +16590,7 @@
     </row>
     <row r="200" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A200" s="4" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="B200" s="5">
         <v>46166.90583462963</v>
@@ -16571,7 +16605,7 @@
         <v>83</v>
       </c>
       <c r="F200" s="6" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="G200" s="6" t="s">
         <v>32</v>
@@ -16606,10 +16640,10 @@
         <v>35</v>
       </c>
       <c r="S200" s="6" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="T200" s="6" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="U200" s="8" t="s">
         <v>95</v>
@@ -16618,7 +16652,7 @@
         <v>46171</v>
       </c>
       <c r="W200" s="9" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="X200" s="6">
         <v>0</v>
@@ -16627,7 +16661,7 @@
     </row>
     <row r="201" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A201" s="10" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="B201" s="11">
         <v>46166.90584622685</v>
@@ -16640,7 +16674,7 @@
         <v>153</v>
       </c>
       <c r="F201" s="12" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="G201" s="12" t="s">
         <v>32</v>
@@ -16675,17 +16709,17 @@
         <v>35</v>
       </c>
       <c r="S201" s="12" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="T201" s="12" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="U201" s="8" t="s">
         <v>95</v>
       </c>
       <c r="V201" s="12"/>
       <c r="W201" s="9" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="X201" s="12">
         <v>0</v>
@@ -16694,7 +16728,7 @@
     </row>
     <row r="202" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A202" s="4" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="B202" s="5">
         <v>46166.906513483795</v>
@@ -16707,7 +16741,7 @@
         <v>40</v>
       </c>
       <c r="F202" s="6" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="G202" s="6" t="s">
         <v>32</v>
@@ -16747,14 +16781,14 @@
         <v>179</v>
       </c>
       <c r="T202" s="6" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="U202" s="8" t="s">
         <v>95</v>
       </c>
       <c r="V202" s="6"/>
       <c r="W202" s="9" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="X202" s="6">
         <v>0</v>
@@ -16763,7 +16797,7 @@
     </row>
     <row r="203" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A203" s="10" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="B203" s="11">
         <v>46166.90651771991</v>
@@ -16778,7 +16812,7 @@
         <v>83</v>
       </c>
       <c r="F203" s="12" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="G203" s="12" t="s">
         <v>32</v>
@@ -16818,7 +16852,7 @@
         <v>179</v>
       </c>
       <c r="T203" s="12" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="U203" s="8" t="s">
         <v>95</v>
@@ -16827,7 +16861,7 @@
         <v>46171</v>
       </c>
       <c r="W203" s="9" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="X203" s="12">
         <v>0</v>
@@ -16836,7 +16870,7 @@
     </row>
     <row r="204" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A204" s="4" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="B204" s="5">
         <v>46166.90652930556</v>
@@ -16849,7 +16883,7 @@
         <v>153</v>
       </c>
       <c r="F204" s="6" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="G204" s="6" t="s">
         <v>32</v>
@@ -16887,14 +16921,14 @@
         <v>179</v>
       </c>
       <c r="T204" s="6" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="U204" s="8" t="s">
         <v>95</v>
       </c>
       <c r="V204" s="6"/>
       <c r="W204" s="9" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="X204" s="6">
         <v>0</v>
@@ -16903,7 +16937,7 @@
     </row>
     <row r="205" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A205" s="10" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="B205" s="11">
         <v>46166.90221321759</v>
@@ -16916,7 +16950,7 @@
         <v>40</v>
       </c>
       <c r="F205" s="12" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="G205" s="12" t="s">
         <v>41</v>
@@ -16953,17 +16987,17 @@
         <v>35</v>
       </c>
       <c r="S205" s="12" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="T205" s="12" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="U205" s="8" t="s">
         <v>141</v>
       </c>
       <c r="V205" s="12"/>
       <c r="W205" s="9" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="X205" s="12">
         <v>0</v>
@@ -16972,7 +17006,7 @@
     </row>
     <row r="206" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A206" s="4" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="B206" s="5">
         <v>46166.902219814816</v>
@@ -16985,7 +17019,7 @@
         <v>83</v>
       </c>
       <c r="F206" s="6" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="G206" s="6" t="s">
         <v>30</v>
@@ -17022,17 +17056,17 @@
         <v>35</v>
       </c>
       <c r="S206" s="6" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="T206" s="6" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="U206" s="8" t="s">
         <v>141</v>
       </c>
       <c r="V206" s="6"/>
       <c r="W206" s="9" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="X206" s="6">
         <v>0</v>
@@ -17041,7 +17075,7 @@
     </row>
     <row r="207" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A207" s="10" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="B207" s="11">
         <v>46166.90223270834</v>
@@ -17054,7 +17088,7 @@
         <v>153</v>
       </c>
       <c r="F207" s="12" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="G207" s="12" t="s">
         <v>44</v>
@@ -17091,17 +17125,17 @@
         <v>35</v>
       </c>
       <c r="S207" s="12" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="T207" s="12" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="U207" s="8" t="s">
         <v>141</v>
       </c>
       <c r="V207" s="12"/>
       <c r="W207" s="9" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="X207" s="12">
         <v>0</v>
@@ -17110,7 +17144,7 @@
     </row>
     <row r="208" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A208" s="4" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="B208" s="5">
         <v>46168.66132378472</v>
@@ -17125,7 +17159,7 @@
         <v>40</v>
       </c>
       <c r="F208" s="6" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="G208" s="6" t="s">
         <v>78</v>
@@ -17162,10 +17196,10 @@
         <v>35</v>
       </c>
       <c r="S208" s="6" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="T208" s="6" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="U208" s="8" t="s">
         <v>109</v>
@@ -17174,7 +17208,7 @@
         <v>46183</v>
       </c>
       <c r="W208" s="9" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="X208" s="6">
         <v>1</v>
@@ -17183,7 +17217,7 @@
     </row>
     <row r="209" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A209" s="10" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="B209" s="11">
         <v>46168.6613384375</v>
@@ -17198,7 +17232,7 @@
         <v>83</v>
       </c>
       <c r="F209" s="12" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="G209" s="12" t="s">
         <v>30</v>
@@ -17235,10 +17269,10 @@
         <v>35</v>
       </c>
       <c r="S209" s="12" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="T209" s="12" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="U209" s="8" t="s">
         <v>109</v>
@@ -17247,7 +17281,7 @@
         <v>46183</v>
       </c>
       <c r="W209" s="9" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="X209" s="12">
         <v>1</v>
@@ -17256,7 +17290,7 @@
     </row>
     <row r="210" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A210" s="4" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="B210" s="5">
         <v>46168.66134381945</v>
@@ -17271,7 +17305,7 @@
         <v>153</v>
       </c>
       <c r="F210" s="6" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="G210" s="6" t="s">
         <v>44</v>
@@ -17308,10 +17342,10 @@
         <v>35</v>
       </c>
       <c r="S210" s="6" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="T210" s="6" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="U210" s="8" t="s">
         <v>109</v>
@@ -17320,7 +17354,7 @@
         <v>46183</v>
       </c>
       <c r="W210" s="9" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="X210" s="6">
         <v>1</v>
@@ -17329,7 +17363,7 @@
     </row>
     <row r="211" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A211" s="10" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="B211" s="11">
         <v>46168.67944415509</v>
@@ -17344,7 +17378,7 @@
         <v>40</v>
       </c>
       <c r="F211" s="12" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="G211" s="12" t="s">
         <v>32</v>
@@ -17379,10 +17413,10 @@
         <v>35</v>
       </c>
       <c r="S211" s="12" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="T211" s="12" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="U211" s="8" t="s">
         <v>95</v>
@@ -17391,7 +17425,7 @@
         <v>46178</v>
       </c>
       <c r="W211" s="9" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="X211" s="12">
         <v>0</v>
@@ -17400,7 +17434,7 @@
     </row>
     <row r="212" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A212" s="4" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="B212" s="5">
         <v>46168.67944923611</v>
@@ -17415,7 +17449,7 @@
         <v>83</v>
       </c>
       <c r="F212" s="6" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="G212" s="6" t="s">
         <v>32</v>
@@ -17450,10 +17484,10 @@
         <v>35</v>
       </c>
       <c r="S212" s="6" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="T212" s="6" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="U212" s="8" t="s">
         <v>95</v>
@@ -17462,7 +17496,7 @@
         <v>46178</v>
       </c>
       <c r="W212" s="9" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="X212" s="6">
         <v>0</v>
@@ -17471,7 +17505,7 @@
     </row>
     <row r="213" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A213" s="10" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="B213" s="11">
         <v>46168.67946252315</v>
@@ -17486,7 +17520,7 @@
         <v>153</v>
       </c>
       <c r="F213" s="12" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="G213" s="12" t="s">
         <v>32</v>
@@ -17521,10 +17555,10 @@
         <v>35</v>
       </c>
       <c r="S213" s="12" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="T213" s="12" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="U213" s="8" t="s">
         <v>95</v>
@@ -17533,7 +17567,7 @@
         <v>46178</v>
       </c>
       <c r="W213" s="9" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="X213" s="12">
         <v>0</v>
@@ -17542,7 +17576,7 @@
     </row>
     <row r="214" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A214" s="4" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="B214" s="5">
         <v>46169.62462164352</v>
@@ -17557,7 +17591,7 @@
         <v>40</v>
       </c>
       <c r="F214" s="6" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="G214" s="6" t="s">
         <v>32</v>
@@ -17594,10 +17628,10 @@
         <v>35</v>
       </c>
       <c r="S214" s="6" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="T214" s="6" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="U214" s="8" t="s">
         <v>141</v>
@@ -17606,7 +17640,7 @@
         <v>46169</v>
       </c>
       <c r="W214" s="9" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="X214" s="6">
         <v>1</v>
@@ -17615,7 +17649,7 @@
     </row>
     <row r="215" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A215" s="10" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="B215" s="11">
         <v>46169.624627708334</v>
@@ -17630,7 +17664,7 @@
         <v>83</v>
       </c>
       <c r="F215" s="12" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="G215" s="12" t="s">
         <v>32</v>
@@ -17667,10 +17701,10 @@
         <v>35</v>
       </c>
       <c r="S215" s="12" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="T215" s="12" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="U215" s="8" t="s">
         <v>141</v>
@@ -17679,7 +17713,7 @@
         <v>46169</v>
       </c>
       <c r="W215" s="9" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="X215" s="12">
         <v>1</v>
@@ -17688,7 +17722,7 @@
     </row>
     <row r="216" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A216" s="4" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B216" s="5">
         <v>46169.624638611116</v>
@@ -17703,7 +17737,7 @@
         <v>153</v>
       </c>
       <c r="F216" s="6" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="G216" s="6" t="s">
         <v>32</v>
@@ -17740,10 +17774,10 @@
         <v>35</v>
       </c>
       <c r="S216" s="6" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="T216" s="6" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="U216" s="8" t="s">
         <v>141</v>
@@ -17752,7 +17786,7 @@
         <v>46169</v>
       </c>
       <c r="W216" s="9" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="X216" s="6">
         <v>1</v>
@@ -17761,7 +17795,7 @@
     </row>
     <row r="217" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A217" s="10" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="B217" s="11">
         <v>46170.78224266204</v>
@@ -17776,7 +17810,7 @@
         <v>40</v>
       </c>
       <c r="F217" s="12" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="G217" s="12" t="s">
         <v>78</v>
@@ -17813,10 +17847,10 @@
         <v>35</v>
       </c>
       <c r="S217" s="12" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="T217" s="12" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="U217" s="8" t="s">
         <v>291</v>
@@ -17825,7 +17859,7 @@
         <v>46171</v>
       </c>
       <c r="W217" s="9" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="X217" s="12">
         <v>1</v>
@@ -17834,7 +17868,7 @@
     </row>
     <row r="218" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A218" s="4" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="B218" s="5">
         <v>46170.782249386575</v>
@@ -17849,7 +17883,7 @@
         <v>83</v>
       </c>
       <c r="F218" s="6" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="G218" s="6" t="s">
         <v>30</v>
@@ -17886,10 +17920,10 @@
         <v>35</v>
       </c>
       <c r="S218" s="6" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="T218" s="6" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="U218" s="8" t="s">
         <v>291</v>
@@ -17898,7 +17932,7 @@
         <v>46171</v>
       </c>
       <c r="W218" s="9" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="X218" s="6">
         <v>1</v>
@@ -17907,7 +17941,7 @@
     </row>
     <row r="219" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A219" s="10" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="B219" s="11">
         <v>46170.78226306713</v>
@@ -17922,7 +17956,7 @@
         <v>153</v>
       </c>
       <c r="F219" s="12" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="G219" s="12" t="s">
         <v>44</v>
@@ -17959,10 +17993,10 @@
         <v>35</v>
       </c>
       <c r="S219" s="12" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="T219" s="12" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="U219" s="8" t="s">
         <v>291</v>
@@ -17971,7 +18005,7 @@
         <v>46171</v>
       </c>
       <c r="W219" s="9" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="X219" s="12">
         <v>1</v>
@@ -17980,7 +18014,7 @@
     </row>
     <row r="220" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A220" s="4" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="B220" s="5">
         <v>46171.541563032406</v>
@@ -17993,7 +18027,7 @@
         <v>40</v>
       </c>
       <c r="F220" s="6" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="G220" s="6" t="s">
         <v>41</v>
@@ -18032,17 +18066,17 @@
         <v>35</v>
       </c>
       <c r="S220" s="6" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="T220" s="6" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="U220" s="8" t="s">
         <v>141</v>
       </c>
       <c r="V220" s="6"/>
       <c r="W220" s="9" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="X220" s="6">
         <v>0</v>
@@ -18051,7 +18085,7 @@
     </row>
     <row r="221" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A221" s="10" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="B221" s="11">
         <v>46171.541569594905</v>
@@ -18064,7 +18098,7 @@
         <v>83</v>
       </c>
       <c r="F221" s="12" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="G221" s="12" t="s">
         <v>30</v>
@@ -18103,17 +18137,17 @@
         <v>35</v>
       </c>
       <c r="S221" s="12" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="T221" s="12" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="U221" s="8" t="s">
         <v>141</v>
       </c>
       <c r="V221" s="12"/>
       <c r="W221" s="9" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="X221" s="12">
         <v>0</v>
@@ -18122,7 +18156,7 @@
     </row>
     <row r="222" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A222" s="4" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="B222" s="5">
         <v>46171.54158304398</v>
@@ -18135,7 +18169,7 @@
         <v>153</v>
       </c>
       <c r="F222" s="6" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="G222" s="6" t="s">
         <v>44</v>
@@ -18174,17 +18208,17 @@
         <v>35</v>
       </c>
       <c r="S222" s="6" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="T222" s="6" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="U222" s="8" t="s">
         <v>141</v>
       </c>
       <c r="V222" s="6"/>
       <c r="W222" s="9" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="X222" s="6">
         <v>0</v>
@@ -18193,7 +18227,7 @@
     </row>
     <row r="223" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A223" s="10" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="B223" s="11">
         <v>46170.7846755787</v>
@@ -18206,7 +18240,7 @@
         <v>40</v>
       </c>
       <c r="F223" s="12" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="G223" s="12" t="s">
         <v>32</v>
@@ -18241,7 +18275,7 @@
         <v>35</v>
       </c>
       <c r="S223" s="12" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="T223" s="12" t="s">
         <v>297</v>
@@ -18260,7 +18294,7 @@
     </row>
     <row r="224" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A224" s="4" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="B224" s="5">
         <v>46170.78468033565</v>
@@ -18273,7 +18307,7 @@
         <v>83</v>
       </c>
       <c r="F224" s="6" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="G224" s="6" t="s">
         <v>32</v>
@@ -18308,7 +18342,7 @@
         <v>35</v>
       </c>
       <c r="S224" s="6" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="T224" s="6" t="s">
         <v>297</v>
@@ -18327,7 +18361,7 @@
     </row>
     <row r="225" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A225" s="10" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="B225" s="11">
         <v>46170.784693657406</v>
@@ -18340,7 +18374,7 @@
         <v>153</v>
       </c>
       <c r="F225" s="12" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="G225" s="12" t="s">
         <v>32</v>
@@ -18375,7 +18409,7 @@
         <v>35</v>
       </c>
       <c r="S225" s="12" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="T225" s="12" t="s">
         <v>297</v>
@@ -18394,7 +18428,7 @@
     </row>
     <row r="226" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A226" s="4" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="B226" s="5">
         <v>46171.55260833333</v>
@@ -18409,7 +18443,7 @@
         <v>40</v>
       </c>
       <c r="F226" s="6" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="G226" s="6" t="s">
         <v>78</v>
@@ -18446,10 +18480,10 @@
         <v>35</v>
       </c>
       <c r="S226" s="6" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="T226" s="6" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="U226" s="8" t="s">
         <v>38</v>
@@ -18458,7 +18492,7 @@
         <v>46177</v>
       </c>
       <c r="W226" s="9" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="X226" s="6">
         <v>1</v>
@@ -18467,7 +18501,7 @@
     </row>
     <row r="227" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A227" s="10" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="B227" s="11">
         <v>46171.552612685184</v>
@@ -18482,7 +18516,7 @@
         <v>83</v>
       </c>
       <c r="F227" s="12" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="G227" s="12" t="s">
         <v>30</v>
@@ -18519,10 +18553,10 @@
         <v>35</v>
       </c>
       <c r="S227" s="12" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="T227" s="12" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="U227" s="8" t="s">
         <v>38</v>
@@ -18531,7 +18565,7 @@
         <v>46176</v>
       </c>
       <c r="W227" s="9" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="X227" s="12">
         <v>1</v>
@@ -18540,7 +18574,7 @@
     </row>
     <row r="228" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A228" s="4" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="B228" s="5">
         <v>46171.55262621528</v>
@@ -18555,7 +18589,7 @@
         <v>153</v>
       </c>
       <c r="F228" s="6" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="G228" s="6" t="s">
         <v>44</v>
@@ -18592,10 +18626,10 @@
         <v>35</v>
       </c>
       <c r="S228" s="6" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="T228" s="6" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="U228" s="8" t="s">
         <v>38</v>
@@ -18604,7 +18638,7 @@
         <v>46178</v>
       </c>
       <c r="W228" s="9" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="X228" s="6">
         <v>1</v>
@@ -18613,7 +18647,7 @@
     </row>
     <row r="229" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A229" s="10" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="B229" s="11">
         <v>46171.55905822916</v>
@@ -18628,13 +18662,13 @@
         <v>40</v>
       </c>
       <c r="F229" s="12" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="G229" s="12" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="H229" s="12" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="I229" s="12"/>
       <c r="J229" s="11">
@@ -18665,19 +18699,19 @@
         <v>35</v>
       </c>
       <c r="S229" s="12" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="T229" s="12" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="U229" s="8" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="V229" s="11">
         <v>46175</v>
       </c>
       <c r="W229" s="9" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="X229" s="12">
         <v>1</v>
@@ -18686,7 +18720,7 @@
     </row>
     <row r="230" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A230" s="4" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="B230" s="5">
         <v>46171.55906322917</v>
@@ -18701,7 +18735,7 @@
         <v>83</v>
       </c>
       <c r="F230" s="6" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="G230" s="6" t="s">
         <v>30</v>
@@ -18738,19 +18772,19 @@
         <v>35</v>
       </c>
       <c r="S230" s="6" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="T230" s="6" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="U230" s="8" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="V230" s="5">
         <v>46175</v>
       </c>
       <c r="W230" s="9" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="X230" s="6">
         <v>1</v>
@@ -18759,7 +18793,7 @@
     </row>
     <row r="231" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A231" s="10" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="B231" s="11">
         <v>46171.55907711806</v>
@@ -18774,7 +18808,7 @@
         <v>153</v>
       </c>
       <c r="F231" s="12" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="G231" s="12" t="s">
         <v>44</v>
@@ -18811,19 +18845,19 @@
         <v>35</v>
       </c>
       <c r="S231" s="12" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="T231" s="12" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="U231" s="8" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="V231" s="11">
         <v>46175</v>
       </c>
       <c r="W231" s="9" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="X231" s="12">
         <v>1</v>
@@ -18832,7 +18866,7 @@
     </row>
     <row r="232" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A232" s="4" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="B232" s="5">
         <v>46171.56219060185</v>
@@ -18847,7 +18881,7 @@
         <v>40</v>
       </c>
       <c r="F232" s="6" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="G232" s="6" t="s">
         <v>78</v>
@@ -18885,14 +18919,14 @@
       </c>
       <c r="S232" s="6"/>
       <c r="T232" s="6" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="U232" s="6"/>
       <c r="V232" s="5">
         <v>46181</v>
       </c>
       <c r="W232" s="9" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="X232" s="6">
         <v>0</v>
@@ -18901,7 +18935,7 @@
     </row>
     <row r="233" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A233" s="10" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="B233" s="11">
         <v>46171.56219597222</v>
@@ -18916,7 +18950,7 @@
         <v>83</v>
       </c>
       <c r="F233" s="12" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="G233" s="12" t="s">
         <v>30</v>
@@ -18954,14 +18988,14 @@
       </c>
       <c r="S233" s="12"/>
       <c r="T233" s="12" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="U233" s="12"/>
       <c r="V233" s="11">
         <v>46181</v>
       </c>
       <c r="W233" s="9" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="X233" s="12">
         <v>0</v>
@@ -18970,7 +19004,7 @@
     </row>
     <row r="234" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A234" s="4" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="B234" s="5">
         <v>46171.56220810185</v>
@@ -18985,7 +19019,7 @@
         <v>153</v>
       </c>
       <c r="F234" s="6" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="G234" s="6" t="s">
         <v>44</v>
@@ -19023,14 +19057,14 @@
       </c>
       <c r="S234" s="6"/>
       <c r="T234" s="6" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="U234" s="6"/>
       <c r="V234" s="5">
         <v>46185</v>
       </c>
       <c r="W234" s="9" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="X234" s="6">
         <v>0</v>
@@ -19039,7 +19073,7 @@
     </row>
     <row r="235" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A235" s="10" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="B235" s="11">
         <v>46174.78293828704</v>
@@ -19054,13 +19088,13 @@
         <v>40</v>
       </c>
       <c r="F235" s="12" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="G235" s="12" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="H235" s="12" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="I235" s="12"/>
       <c r="J235" s="11">
@@ -19091,10 +19125,10 @@
         <v>35</v>
       </c>
       <c r="S235" s="12" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="T235" s="12" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="U235" s="8" t="s">
         <v>38</v>
@@ -19103,7 +19137,7 @@
         <v>46177</v>
       </c>
       <c r="W235" s="9" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="X235" s="12">
         <v>1</v>
@@ -19112,7 +19146,7 @@
     </row>
     <row r="236" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A236" s="4" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="B236" s="5">
         <v>46174.78294421296</v>
@@ -19127,7 +19161,7 @@
         <v>83</v>
       </c>
       <c r="F236" s="6" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="G236" s="6" t="s">
         <v>30</v>
@@ -19164,10 +19198,10 @@
         <v>35</v>
       </c>
       <c r="S236" s="6" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="T236" s="6" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="U236" s="8" t="s">
         <v>38</v>
@@ -19176,7 +19210,7 @@
         <v>46185</v>
       </c>
       <c r="W236" s="9" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="X236" s="6">
         <v>1</v>
@@ -19185,7 +19219,7 @@
     </row>
     <row r="237" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A237" s="10" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B237" s="11">
         <v>46174.782957372685</v>
@@ -19200,7 +19234,7 @@
         <v>153</v>
       </c>
       <c r="F237" s="12" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="G237" s="12" t="s">
         <v>44</v>
@@ -19237,10 +19271,10 @@
         <v>35</v>
       </c>
       <c r="S237" s="12" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="T237" s="12" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="U237" s="8" t="s">
         <v>38</v>
@@ -19249,7 +19283,7 @@
         <v>46177</v>
       </c>
       <c r="W237" s="9" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="X237" s="12">
         <v>1</v>
@@ -19258,7 +19292,7 @@
     </row>
     <row r="238" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A238" s="4" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="B238" s="5">
         <v>46175.62894534723</v>
@@ -19273,7 +19307,7 @@
         <v>40</v>
       </c>
       <c r="F238" s="6" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="G238" s="6" t="s">
         <v>30</v>
@@ -19310,10 +19344,10 @@
         <v>35</v>
       </c>
       <c r="S238" s="6" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="T238" s="6" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="U238" s="8" t="s">
         <v>141</v>
@@ -19322,7 +19356,7 @@
         <v>46182</v>
       </c>
       <c r="W238" s="9" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="X238" s="6">
         <v>1</v>
@@ -19331,7 +19365,7 @@
     </row>
     <row r="239" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A239" s="10" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="B239" s="11">
         <v>46175.628960682865</v>
@@ -19346,7 +19380,7 @@
         <v>83</v>
       </c>
       <c r="F239" s="12" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="G239" s="12" t="s">
         <v>30</v>
@@ -19383,10 +19417,10 @@
         <v>35</v>
       </c>
       <c r="S239" s="12" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="T239" s="12" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="U239" s="8" t="s">
         <v>141</v>
@@ -19395,7 +19429,7 @@
         <v>46182</v>
       </c>
       <c r="W239" s="9" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="X239" s="12">
         <v>1</v>
@@ -19404,7 +19438,7 @@
     </row>
     <row r="240" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A240" s="4" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="B240" s="5">
         <v>46175.62896625</v>
@@ -19419,7 +19453,7 @@
         <v>153</v>
       </c>
       <c r="F240" s="6" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="G240" s="6" t="s">
         <v>44</v>
@@ -19456,10 +19490,10 @@
         <v>35</v>
       </c>
       <c r="S240" s="6" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="T240" s="6" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="U240" s="8" t="s">
         <v>141</v>
@@ -19468,7 +19502,7 @@
         <v>46182</v>
       </c>
       <c r="W240" s="9" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="X240" s="6">
         <v>1</v>
@@ -19477,7 +19511,7 @@
     </row>
     <row r="241" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A241" s="10" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="B241" s="11">
         <v>46177.55207784723</v>
@@ -19492,7 +19526,7 @@
         <v>40</v>
       </c>
       <c r="F241" s="12" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="G241" s="12" t="s">
         <v>78</v>
@@ -19529,10 +19563,10 @@
         <v>35</v>
       </c>
       <c r="S241" s="12" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="T241" s="12" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="U241" s="8" t="s">
         <v>141</v>
@@ -19541,7 +19575,7 @@
         <v>46178</v>
       </c>
       <c r="W241" s="9" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="X241" s="12">
         <v>0</v>
@@ -19550,7 +19584,7 @@
     </row>
     <row r="242" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A242" s="4" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="B242" s="5">
         <v>46177.552084675925</v>
@@ -19565,7 +19599,7 @@
         <v>83</v>
       </c>
       <c r="F242" s="6" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="G242" s="6" t="s">
         <v>30</v>
@@ -19602,10 +19636,10 @@
         <v>35</v>
       </c>
       <c r="S242" s="6" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="T242" s="6" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="U242" s="8" t="s">
         <v>141</v>
@@ -19614,7 +19648,7 @@
         <v>46177</v>
       </c>
       <c r="W242" s="9" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="X242" s="6">
         <v>0</v>
@@ -19623,7 +19657,7 @@
     </row>
     <row r="243" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A243" s="10" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="B243" s="11">
         <v>46177.552097997686</v>
@@ -19638,13 +19672,13 @@
         <v>153</v>
       </c>
       <c r="F243" s="12" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="G243" s="12" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="H243" s="12" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="I243" s="12"/>
       <c r="J243" s="11">
@@ -19675,10 +19709,10 @@
         <v>35</v>
       </c>
       <c r="S243" s="12" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="T243" s="12" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="U243" s="8" t="s">
         <v>141</v>
@@ -19687,7 +19721,7 @@
         <v>46178</v>
       </c>
       <c r="W243" s="9" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="X243" s="12">
         <v>0</v>
@@ -19696,7 +19730,7 @@
     </row>
     <row r="244" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A244" s="4" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="B244" s="5">
         <v>46177.55718690972</v>
@@ -19711,7 +19745,7 @@
         <v>40</v>
       </c>
       <c r="F244" s="6" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="G244" s="6" t="s">
         <v>78</v>
@@ -19748,19 +19782,19 @@
         <v>35</v>
       </c>
       <c r="S244" s="6" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="T244" s="6" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="U244" s="8" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="V244" s="5">
         <v>46189</v>
       </c>
       <c r="W244" s="9" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="X244" s="6">
         <v>1</v>
@@ -19769,7 +19803,7 @@
     </row>
     <row r="245" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A245" s="10" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="B245" s="11">
         <v>46177.55719148148</v>
@@ -19784,7 +19818,7 @@
         <v>83</v>
       </c>
       <c r="F245" s="12" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="G245" s="12" t="s">
         <v>30</v>
@@ -19821,19 +19855,19 @@
         <v>35</v>
       </c>
       <c r="S245" s="12" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="T245" s="12" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="U245" s="8" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="V245" s="11">
         <v>46184</v>
       </c>
       <c r="W245" s="9" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="X245" s="12">
         <v>1</v>
@@ -19842,7 +19876,7 @@
     </row>
     <row r="246" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A246" s="4" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="B246" s="5">
         <v>46177.557204282406</v>
@@ -19857,7 +19891,7 @@
         <v>153</v>
       </c>
       <c r="F246" s="6" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="G246" s="6" t="s">
         <v>44</v>
@@ -19894,19 +19928,19 @@
         <v>35</v>
       </c>
       <c r="S246" s="6" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="T246" s="6" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="U246" s="8" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="V246" s="5">
         <v>46190</v>
       </c>
       <c r="W246" s="9" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="X246" s="6">
         <v>1</v>
@@ -19915,7 +19949,7 @@
     </row>
     <row r="247" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A247" s="10" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="B247" s="11">
         <v>46177.58134283565</v>
@@ -19930,7 +19964,7 @@
         <v>40</v>
       </c>
       <c r="F247" s="12" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="G247" s="12" t="s">
         <v>41</v>
@@ -19967,10 +20001,10 @@
         <v>35</v>
       </c>
       <c r="S247" s="12" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="T247" s="12" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="U247" s="8" t="s">
         <v>141</v>
@@ -19979,7 +20013,7 @@
         <v>46176</v>
       </c>
       <c r="W247" s="9" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="X247" s="12">
         <v>1</v>
@@ -19988,7 +20022,7 @@
     </row>
     <row r="248" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A248" s="4" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="B248" s="5">
         <v>46177.58134928241</v>
@@ -20003,7 +20037,7 @@
         <v>83</v>
       </c>
       <c r="F248" s="6" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="G248" s="6" t="s">
         <v>30</v>
@@ -20040,10 +20074,10 @@
         <v>35</v>
       </c>
       <c r="S248" s="6" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="T248" s="6" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="U248" s="8" t="s">
         <v>141</v>
@@ -20052,7 +20086,7 @@
         <v>46176</v>
       </c>
       <c r="W248" s="9" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="X248" s="6">
         <v>1</v>
@@ -20061,7 +20095,7 @@
     </row>
     <row r="249" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A249" s="10" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B249" s="11">
         <v>46177.58136225694</v>
@@ -20076,7 +20110,7 @@
         <v>153</v>
       </c>
       <c r="F249" s="12" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="G249" s="12" t="s">
         <v>44</v>
@@ -20113,10 +20147,10 @@
         <v>35</v>
       </c>
       <c r="S249" s="12" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="T249" s="12" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="U249" s="8" t="s">
         <v>141</v>
@@ -20125,7 +20159,7 @@
         <v>46176</v>
       </c>
       <c r="W249" s="9" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="X249" s="12">
         <v>1</v>
@@ -20134,7 +20168,7 @@
     </row>
     <row r="250" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A250" s="4" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="B250" s="5">
         <v>46181.55894307871</v>
@@ -20149,7 +20183,7 @@
         <v>40</v>
       </c>
       <c r="F250" s="6" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="G250" s="6" t="s">
         <v>56</v>
@@ -20186,10 +20220,10 @@
         <v>35</v>
       </c>
       <c r="S250" s="6" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="T250" s="6" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="U250" s="8" t="s">
         <v>95</v>
@@ -20198,7 +20232,7 @@
         <v>46191</v>
       </c>
       <c r="W250" s="9" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="X250" s="6">
         <v>1</v>
@@ -20207,7 +20241,7 @@
     </row>
     <row r="251" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A251" s="10" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="B251" s="11">
         <v>46181.55895883102</v>
@@ -20222,7 +20256,7 @@
         <v>83</v>
       </c>
       <c r="F251" s="12" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="G251" s="12" t="s">
         <v>30</v>
@@ -20259,10 +20293,10 @@
         <v>35</v>
       </c>
       <c r="S251" s="12" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="T251" s="12" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="U251" s="8" t="s">
         <v>95</v>
@@ -20271,7 +20305,7 @@
         <v>46184</v>
       </c>
       <c r="W251" s="9" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="X251" s="12">
         <v>1</v>
@@ -20280,7 +20314,7 @@
     </row>
     <row r="252" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A252" s="4" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="B252" s="5">
         <v>46181.55896603009</v>
@@ -20293,7 +20327,7 @@
         <v>153</v>
       </c>
       <c r="F252" s="6" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="G252" s="6" t="s">
         <v>44</v>
@@ -20330,17 +20364,17 @@
         <v>35</v>
       </c>
       <c r="S252" s="6" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="T252" s="6" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="U252" s="8" t="s">
         <v>95</v>
       </c>
       <c r="V252" s="6"/>
       <c r="W252" s="9" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="X252" s="6">
         <v>0</v>
@@ -20349,7 +20383,7 @@
     </row>
     <row r="253" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A253" s="10" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="B253" s="11">
         <v>46181.56214887732</v>
@@ -20362,7 +20396,7 @@
         <v>40</v>
       </c>
       <c r="F253" s="12" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="G253" s="12" t="s">
         <v>32</v>
@@ -20397,7 +20431,7 @@
         <v>35</v>
       </c>
       <c r="S253" s="12" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="T253" s="12"/>
       <c r="U253" s="8" t="s">
@@ -20412,7 +20446,7 @@
     </row>
     <row r="254" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A254" s="4" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="B254" s="5">
         <v>46181.562153425926</v>
@@ -20425,7 +20459,7 @@
         <v>83</v>
       </c>
       <c r="F254" s="6" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="G254" s="6" t="s">
         <v>32</v>
@@ -20460,7 +20494,7 @@
         <v>35</v>
       </c>
       <c r="S254" s="6" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="T254" s="6"/>
       <c r="U254" s="8" t="s">
@@ -20475,7 +20509,7 @@
     </row>
     <row r="255" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A255" s="10" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="B255" s="11">
         <v>46181.562166250005</v>
@@ -20488,7 +20522,7 @@
         <v>153</v>
       </c>
       <c r="F255" s="12" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="G255" s="12" t="s">
         <v>32</v>
@@ -20523,7 +20557,7 @@
         <v>35</v>
       </c>
       <c r="S255" s="12" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="T255" s="12"/>
       <c r="U255" s="8" t="s">
@@ -20538,7 +20572,7 @@
     </row>
     <row r="256" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A256" s="4" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="B256" s="5">
         <v>46181.5643593287</v>
@@ -20551,7 +20585,7 @@
         <v>40</v>
       </c>
       <c r="F256" s="6" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="G256" s="6" t="s">
         <v>32</v>
@@ -20586,7 +20620,7 @@
         <v>35</v>
       </c>
       <c r="S256" s="6" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="T256" s="6"/>
       <c r="U256" s="6"/>
@@ -20599,7 +20633,7 @@
     </row>
     <row r="257" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A257" s="10" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="B257" s="11">
         <v>46181.56436351852</v>
@@ -20612,7 +20646,7 @@
         <v>83</v>
       </c>
       <c r="F257" s="12" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="G257" s="12" t="s">
         <v>32</v>
@@ -20647,7 +20681,7 @@
         <v>35</v>
       </c>
       <c r="S257" s="12" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="T257" s="12"/>
       <c r="U257" s="12"/>
@@ -20660,7 +20694,7 @@
     </row>
     <row r="258" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A258" s="4" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="B258" s="5">
         <v>46181.56437451389</v>
@@ -20673,7 +20707,7 @@
         <v>153</v>
       </c>
       <c r="F258" s="6" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="G258" s="6" t="s">
         <v>32</v>
@@ -20708,7 +20742,7 @@
         <v>35</v>
       </c>
       <c r="S258" s="6" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="T258" s="6"/>
       <c r="U258" s="6"/>
@@ -20721,7 +20755,7 @@
     </row>
     <row r="259" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A259" s="10" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="B259" s="11">
         <v>46185.55074734954</v>
@@ -20736,7 +20770,7 @@
         <v>40</v>
       </c>
       <c r="F259" s="12" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="G259" s="12" t="s">
         <v>32</v>
@@ -20771,10 +20805,10 @@
         <v>35</v>
       </c>
       <c r="S259" s="12" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="T259" s="12" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="U259" s="8" t="s">
         <v>95</v>
@@ -20783,7 +20817,7 @@
         <v>46184</v>
       </c>
       <c r="W259" s="9" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="X259" s="12">
         <v>1</v>
@@ -20792,7 +20826,7 @@
     </row>
     <row r="260" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A260" s="4" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="B260" s="5">
         <v>46185.5507533912</v>
@@ -20805,7 +20839,7 @@
         <v>83</v>
       </c>
       <c r="F260" s="6" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="G260" s="6" t="s">
         <v>32</v>
@@ -20840,17 +20874,17 @@
         <v>35</v>
       </c>
       <c r="S260" s="6" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="T260" s="6" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="U260" s="8" t="s">
         <v>95</v>
       </c>
       <c r="V260" s="6"/>
       <c r="W260" s="9" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="X260" s="6">
         <v>0</v>
@@ -20859,7 +20893,7 @@
     </row>
     <row r="261" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A261" s="10" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="B261" s="11">
         <v>46185.55076409722</v>
@@ -20872,7 +20906,7 @@
         <v>153</v>
       </c>
       <c r="F261" s="12" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="G261" s="12" t="s">
         <v>32</v>
@@ -20907,17 +20941,17 @@
         <v>35</v>
       </c>
       <c r="S261" s="12" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="T261" s="12" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="U261" s="8" t="s">
         <v>95</v>
       </c>
       <c r="V261" s="12"/>
       <c r="W261" s="9" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="X261" s="12">
         <v>0</v>
@@ -20926,7 +20960,7 @@
     </row>
     <row r="262" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A262" s="4" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="B262" s="5">
         <v>46185.55686909722</v>
@@ -20941,7 +20975,7 @@
         <v>40</v>
       </c>
       <c r="F262" s="6" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="G262" s="6" t="s">
         <v>32</v>
@@ -20976,10 +21010,10 @@
         <v>35</v>
       </c>
       <c r="S262" s="6" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="T262" s="6" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="U262" s="8" t="s">
         <v>291</v>
@@ -20988,7 +21022,7 @@
         <v>46193</v>
       </c>
       <c r="W262" s="9" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="X262" s="6">
         <v>1</v>
@@ -20997,7 +21031,7 @@
     </row>
     <row r="263" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A263" s="10" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="B263" s="11">
         <v>46185.55687354167</v>
@@ -21010,7 +21044,7 @@
         <v>83</v>
       </c>
       <c r="F263" s="12" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="G263" s="12" t="s">
         <v>32</v>
@@ -21045,17 +21079,17 @@
         <v>35</v>
       </c>
       <c r="S263" s="12" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="T263" s="12" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="U263" s="8" t="s">
         <v>291</v>
       </c>
       <c r="V263" s="12"/>
       <c r="W263" s="9" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="X263" s="12">
         <v>0</v>
@@ -21064,7 +21098,7 @@
     </row>
     <row r="264" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A264" s="4" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="B264" s="5">
         <v>46185.55688491898</v>
@@ -21077,7 +21111,7 @@
         <v>153</v>
       </c>
       <c r="F264" s="6" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="G264" s="6" t="s">
         <v>32</v>
@@ -21112,17 +21146,17 @@
         <v>35</v>
       </c>
       <c r="S264" s="6" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="T264" s="6" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="U264" s="8" t="s">
         <v>291</v>
       </c>
       <c r="V264" s="6"/>
       <c r="W264" s="9" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="X264" s="6">
         <v>0</v>
@@ -21131,7 +21165,7 @@
     </row>
     <row r="265" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A265" s="10" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="B265" s="11">
         <v>46185.56558032407</v>
@@ -21144,7 +21178,7 @@
         <v>40</v>
       </c>
       <c r="F265" s="12" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="G265" s="12" t="s">
         <v>41</v>
@@ -21181,17 +21215,17 @@
         <v>35</v>
       </c>
       <c r="S265" s="12" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="T265" s="12" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="U265" s="8" t="s">
         <v>141</v>
       </c>
       <c r="V265" s="12"/>
       <c r="W265" s="9" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="X265" s="12">
         <v>0</v>
@@ -21200,7 +21234,7 @@
     </row>
     <row r="266" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A266" s="4" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="B266" s="5">
         <v>46185.56558616898</v>
@@ -21215,7 +21249,7 @@
         <v>83</v>
       </c>
       <c r="F266" s="6" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="G266" s="6" t="s">
         <v>30</v>
@@ -21252,10 +21286,10 @@
         <v>35</v>
       </c>
       <c r="S266" s="6" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="T266" s="6" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="U266" s="8" t="s">
         <v>141</v>
@@ -21264,7 +21298,7 @@
         <v>46185</v>
       </c>
       <c r="W266" s="9" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="X266" s="6">
         <v>1</v>
@@ -21273,7 +21307,7 @@
     </row>
     <row r="267" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A267" s="10" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="B267" s="11">
         <v>46185.56559773148</v>
@@ -21286,7 +21320,7 @@
         <v>153</v>
       </c>
       <c r="F267" s="12" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="G267" s="12" t="s">
         <v>44</v>
@@ -21323,17 +21357,17 @@
         <v>35</v>
       </c>
       <c r="S267" s="12" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="T267" s="12" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="U267" s="8" t="s">
         <v>141</v>
       </c>
       <c r="V267" s="12"/>
       <c r="W267" s="9" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="X267" s="12">
         <v>0</v>
@@ -21342,7 +21376,7 @@
     </row>
     <row r="268" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A268" s="4" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="B268" s="5">
         <v>46185.59436649305</v>
@@ -21357,7 +21391,7 @@
         <v>40</v>
       </c>
       <c r="F268" s="6" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="G268" s="6" t="s">
         <v>32</v>
@@ -21393,7 +21427,7 @@
       </c>
       <c r="S268" s="6"/>
       <c r="T268" s="6" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="U268" s="8" t="s">
         <v>291</v>
@@ -21402,7 +21436,7 @@
         <v>46195</v>
       </c>
       <c r="W268" s="9" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="X268" s="6">
         <v>1</v>
@@ -21411,7 +21445,7 @@
     </row>
     <row r="269" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A269" s="10" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="B269" s="11">
         <v>46185.59437232639</v>
@@ -21426,7 +21460,7 @@
         <v>83</v>
       </c>
       <c r="F269" s="12" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="G269" s="12" t="s">
         <v>32</v>
@@ -21462,7 +21496,7 @@
       </c>
       <c r="S269" s="12"/>
       <c r="T269" s="12" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="U269" s="8" t="s">
         <v>291</v>
@@ -21471,7 +21505,7 @@
         <v>46191</v>
       </c>
       <c r="W269" s="9" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="X269" s="12">
         <v>1</v>
@@ -21480,7 +21514,7 @@
     </row>
     <row r="270" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A270" s="4" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="B270" s="5">
         <v>46185.594386770834</v>
@@ -21495,7 +21529,7 @@
         <v>153</v>
       </c>
       <c r="F270" s="6" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="G270" s="6" t="s">
         <v>32</v>
@@ -21531,7 +21565,7 @@
       </c>
       <c r="S270" s="6"/>
       <c r="T270" s="6" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="U270" s="8" t="s">
         <v>291</v>
@@ -21540,7 +21574,7 @@
         <v>46195</v>
       </c>
       <c r="W270" s="9" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="X270" s="6">
         <v>1</v>
@@ -21549,7 +21583,7 @@
     </row>
     <row r="271" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A271" s="10" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="B271" s="11">
         <v>46186.654707650465</v>
@@ -21564,7 +21598,7 @@
         <v>40</v>
       </c>
       <c r="F271" s="12" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="G271" s="12" t="s">
         <v>32</v>
@@ -21602,7 +21636,7 @@
       </c>
       <c r="S271" s="12"/>
       <c r="T271" s="12" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="U271" s="8" t="s">
         <v>38</v>
@@ -21611,7 +21645,7 @@
         <v>46157</v>
       </c>
       <c r="W271" s="9" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="X271" s="12">
         <v>1</v>
@@ -21620,7 +21654,7 @@
     </row>
     <row r="272" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A272" s="4" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="B272" s="5">
         <v>46186.65471349537</v>
@@ -21635,7 +21669,7 @@
         <v>83</v>
       </c>
       <c r="F272" s="6" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="G272" s="6" t="s">
         <v>32</v>
@@ -21673,7 +21707,7 @@
       </c>
       <c r="S272" s="6"/>
       <c r="T272" s="6" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="U272" s="8" t="s">
         <v>38</v>
@@ -21682,7 +21716,7 @@
         <v>46157</v>
       </c>
       <c r="W272" s="9" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="X272" s="6">
         <v>1</v>
@@ -21691,7 +21725,7 @@
     </row>
     <row r="273" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A273" s="10" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="B273" s="11">
         <v>46186.654726875</v>
@@ -21706,7 +21740,7 @@
         <v>153</v>
       </c>
       <c r="F273" s="12" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="G273" s="12" t="s">
         <v>32</v>
@@ -21744,7 +21778,7 @@
       </c>
       <c r="S273" s="12"/>
       <c r="T273" s="12" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="U273" s="8" t="s">
         <v>38</v>
@@ -21753,7 +21787,7 @@
         <v>46157</v>
       </c>
       <c r="W273" s="9" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="X273" s="12">
         <v>1</v>
@@ -21762,7 +21796,7 @@
     </row>
     <row r="274" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A274" s="4" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="B274" s="5">
         <v>46191.5563</v>
@@ -21775,7 +21809,7 @@
         <v>40</v>
       </c>
       <c r="F274" s="6" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="G274" s="6" t="s">
         <v>32</v>
@@ -21812,17 +21846,17 @@
         <v>35</v>
       </c>
       <c r="S274" s="6" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="T274" s="6" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="U274" s="8" t="s">
         <v>141</v>
       </c>
       <c r="V274" s="6"/>
       <c r="W274" s="9" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="X274" s="6">
         <v>0</v>
@@ -21831,7 +21865,7 @@
     </row>
     <row r="275" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A275" s="10" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="B275" s="11">
         <v>46191.55632112268</v>
@@ -21846,7 +21880,7 @@
         <v>83</v>
       </c>
       <c r="F275" s="12" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="G275" s="12" t="s">
         <v>32</v>
@@ -21883,10 +21917,10 @@
         <v>35</v>
       </c>
       <c r="S275" s="12" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="T275" s="12" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="U275" s="8" t="s">
         <v>141</v>
@@ -21895,7 +21929,7 @@
         <v>46195</v>
       </c>
       <c r="W275" s="9" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="X275" s="12">
         <v>0</v>
@@ -21904,7 +21938,7 @@
     </row>
     <row r="276" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A276" s="4" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="B276" s="5">
         <v>46191.55632693287</v>
@@ -21917,7 +21951,7 @@
         <v>153</v>
       </c>
       <c r="F276" s="6" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="G276" s="6" t="s">
         <v>32</v>
@@ -21954,17 +21988,17 @@
         <v>35</v>
       </c>
       <c r="S276" s="6" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="T276" s="6" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="U276" s="8" t="s">
         <v>141</v>
       </c>
       <c r="V276" s="6"/>
       <c r="W276" s="9" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="X276" s="6">
         <v>0</v>
@@ -21973,7 +22007,7 @@
     </row>
     <row r="277" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A277" s="10" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="B277" s="11">
         <v>46191.562819375</v>
@@ -21986,7 +22020,7 @@
         <v>40</v>
       </c>
       <c r="F277" s="12" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="G277" s="12" t="s">
         <v>32</v>
@@ -22023,17 +22057,17 @@
         <v>35</v>
       </c>
       <c r="S277" s="12" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="T277" s="12" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="U277" s="8" t="s">
         <v>95</v>
       </c>
       <c r="V277" s="12"/>
       <c r="W277" s="9" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="X277" s="12">
         <v>0</v>
@@ -22042,7 +22076,7 @@
     </row>
     <row r="278" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A278" s="4" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="B278" s="5">
         <v>46191.56282547454</v>
@@ -22055,7 +22089,7 @@
         <v>83</v>
       </c>
       <c r="F278" s="6" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="G278" s="6" t="s">
         <v>32</v>
@@ -22092,17 +22126,17 @@
         <v>35</v>
       </c>
       <c r="S278" s="6" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="T278" s="6" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="U278" s="8" t="s">
         <v>95</v>
       </c>
       <c r="V278" s="6"/>
       <c r="W278" s="9" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="X278" s="6">
         <v>0</v>
@@ -22111,7 +22145,7 @@
     </row>
     <row r="279" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A279" s="10" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="B279" s="11">
         <v>46191.56283715278</v>
@@ -22124,7 +22158,7 @@
         <v>153</v>
       </c>
       <c r="F279" s="12" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="G279" s="12" t="s">
         <v>32</v>
@@ -22161,17 +22195,17 @@
         <v>35</v>
       </c>
       <c r="S279" s="12" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="T279" s="12" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="U279" s="8" t="s">
         <v>95</v>
       </c>
       <c r="V279" s="12"/>
       <c r="W279" s="9" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="X279" s="12">
         <v>0</v>
@@ -22180,7 +22214,7 @@
     </row>
     <row r="280" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A280" s="4" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="B280" s="5">
         <v>46191.56523744213</v>
@@ -22193,7 +22227,7 @@
         <v>40</v>
       </c>
       <c r="F280" s="6" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="G280" s="6" t="s">
         <v>32</v>
@@ -22224,23 +22258,23 @@
         <v>153</v>
       </c>
       <c r="Q280" s="7" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="R280" s="7" t="s">
         <v>35</v>
       </c>
       <c r="S280" s="6" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="T280" s="6" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="U280" s="8" t="s">
         <v>291</v>
       </c>
       <c r="V280" s="6"/>
       <c r="W280" s="9" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="X280" s="6">
         <v>0</v>
@@ -22249,7 +22283,7 @@
     </row>
     <row r="281" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A281" s="10" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="B281" s="11">
         <v>46191.565243125</v>
@@ -22262,7 +22296,7 @@
         <v>83</v>
       </c>
       <c r="F281" s="12" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="G281" s="12" t="s">
         <v>32</v>
@@ -22293,23 +22327,23 @@
         <v>153</v>
       </c>
       <c r="Q281" s="7" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="R281" s="7" t="s">
         <v>35</v>
       </c>
       <c r="S281" s="12" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="T281" s="12" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="U281" s="8" t="s">
         <v>291</v>
       </c>
       <c r="V281" s="12"/>
       <c r="W281" s="9" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="X281" s="12">
         <v>0</v>
@@ -22318,7 +22352,7 @@
     </row>
     <row r="282" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A282" s="4" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="B282" s="5">
         <v>46191.56525601852</v>
@@ -22331,7 +22365,7 @@
         <v>153</v>
       </c>
       <c r="F282" s="6" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="G282" s="6" t="s">
         <v>32</v>
@@ -22362,23 +22396,23 @@
         <v>32</v>
       </c>
       <c r="Q282" s="7" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="R282" s="7" t="s">
         <v>35</v>
       </c>
       <c r="S282" s="6" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="T282" s="6" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="U282" s="8" t="s">
         <v>291</v>
       </c>
       <c r="V282" s="6"/>
       <c r="W282" s="9" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="X282" s="6">
         <v>0</v>
@@ -22387,7 +22421,7 @@
     </row>
     <row r="283" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A283" s="10" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="B283" s="11">
         <v>46197.84756534723</v>
@@ -22400,7 +22434,7 @@
         <v>40</v>
       </c>
       <c r="F283" s="12" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="G283" s="12" t="s">
         <v>32</v>
@@ -22438,14 +22472,14 @@
         <v>80</v>
       </c>
       <c r="T283" s="12" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="U283" s="8" t="s">
         <v>95</v>
       </c>
       <c r="V283" s="12"/>
       <c r="W283" s="9" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="X283" s="12">
         <v>0</v>
@@ -22454,7 +22488,7 @@
     </row>
     <row r="284" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A284" s="4" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="B284" s="5">
         <v>46197.84758265046</v>
@@ -22467,7 +22501,7 @@
         <v>83</v>
       </c>
       <c r="F284" s="6" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="G284" s="6" t="s">
         <v>32</v>
@@ -22505,14 +22539,14 @@
         <v>80</v>
       </c>
       <c r="T284" s="6" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="U284" s="8" t="s">
         <v>95</v>
       </c>
       <c r="V284" s="6"/>
       <c r="W284" s="9" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="X284" s="6">
         <v>0</v>
@@ -22521,7 +22555,7 @@
     </row>
     <row r="285" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A285" s="10" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="B285" s="11">
         <v>46197.84758912037</v>
@@ -22534,7 +22568,7 @@
         <v>153</v>
       </c>
       <c r="F285" s="12" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="G285" s="12" t="s">
         <v>32</v>
@@ -22572,14 +22606,14 @@
         <v>80</v>
       </c>
       <c r="T285" s="12" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="U285" s="8" t="s">
         <v>95</v>
       </c>
       <c r="V285" s="12"/>
       <c r="W285" s="9" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="X285" s="12">
         <v>0</v>
@@ -22588,7 +22622,7 @@
     </row>
     <row r="286" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A286" s="4" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="B286" s="5">
         <v>46197.889788437504</v>
@@ -22603,7 +22637,7 @@
         <v>40</v>
       </c>
       <c r="F286" s="6" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="G286" s="6" t="s">
         <v>56</v>
@@ -22640,7 +22674,7 @@
         <v>35</v>
       </c>
       <c r="S286" s="6" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="T286" s="6"/>
       <c r="U286" s="8" t="s">
@@ -22657,7 +22691,7 @@
     </row>
     <row r="287" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A287" s="10" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="B287" s="11">
         <v>46197.88979412037</v>
@@ -22672,7 +22706,7 @@
         <v>83</v>
       </c>
       <c r="F287" s="12" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="G287" s="12" t="s">
         <v>30</v>
@@ -22709,7 +22743,7 @@
         <v>35</v>
       </c>
       <c r="S287" s="12" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="T287" s="12"/>
       <c r="U287" s="8" t="s">
@@ -22726,20 +22760,22 @@
     </row>
     <row r="288" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A288" s="4" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="B288" s="5">
         <v>46197.88980721065</v>
       </c>
-      <c r="C288" s="6"/>
+      <c r="C288" s="5">
+        <v>46205.53868384259</v>
+      </c>
       <c r="D288" s="5">
-        <v>46198.90062260417</v>
+        <v>46205.53868542824</v>
       </c>
       <c r="E288" s="6" t="s">
         <v>153</v>
       </c>
       <c r="F288" s="6" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="G288" s="6" t="s">
         <v>44</v>
@@ -22776,7 +22812,7 @@
         <v>35</v>
       </c>
       <c r="S288" s="6" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="T288" s="6"/>
       <c r="U288" s="8" t="s">
@@ -22791,7 +22827,7 @@
     </row>
     <row r="289" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A289" s="10" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="B289" s="11">
         <v>46197.89618916667</v>
@@ -22806,7 +22842,7 @@
         <v>40</v>
       </c>
       <c r="F289" s="12" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="G289" s="12" t="s">
         <v>41</v>
@@ -22843,10 +22879,10 @@
         <v>35</v>
       </c>
       <c r="S289" s="12" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="T289" s="12" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="U289" s="8" t="s">
         <v>95</v>
@@ -22855,7 +22891,7 @@
         <v>46198</v>
       </c>
       <c r="W289" s="9" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="X289" s="12">
         <v>1</v>
@@ -22864,7 +22900,7 @@
     </row>
     <row r="290" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A290" s="4" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="B290" s="5">
         <v>46197.896195532405</v>
@@ -22879,7 +22915,7 @@
         <v>83</v>
       </c>
       <c r="F290" s="6" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="G290" s="6" t="s">
         <v>30</v>
@@ -22916,10 +22952,10 @@
         <v>35</v>
       </c>
       <c r="S290" s="6" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="T290" s="6" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="U290" s="8" t="s">
         <v>95</v>
@@ -22928,7 +22964,7 @@
         <v>46198</v>
       </c>
       <c r="W290" s="9" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="X290" s="6">
         <v>0</v>
@@ -22937,7 +22973,7 @@
     </row>
     <row r="291" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A291" s="10" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="B291" s="11">
         <v>46197.89621086806</v>
@@ -22952,7 +22988,7 @@
         <v>153</v>
       </c>
       <c r="F291" s="12" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="G291" s="12" t="s">
         <v>44</v>
@@ -22989,10 +23025,10 @@
         <v>35</v>
       </c>
       <c r="S291" s="12" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="T291" s="12" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="U291" s="8" t="s">
         <v>95</v>
@@ -23001,7 +23037,7 @@
         <v>46198</v>
       </c>
       <c r="W291" s="9" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="X291" s="12">
         <v>0</v>
@@ -23010,7 +23046,7 @@
     </row>
     <row r="292" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A292" s="4" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="B292" s="5">
         <v>46203.546952488425</v>
@@ -23023,7 +23059,7 @@
         <v>40</v>
       </c>
       <c r="F292" s="6" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="G292" s="6" t="s">
         <v>32</v>
@@ -23058,17 +23094,17 @@
         <v>35</v>
       </c>
       <c r="S292" s="6" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="T292" s="6" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="U292" s="8" t="s">
         <v>116</v>
       </c>
       <c r="V292" s="6"/>
       <c r="W292" s="9" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="X292" s="6">
         <v>0</v>
@@ -23077,7 +23113,7 @@
     </row>
     <row r="293" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A293" s="10" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="B293" s="11">
         <v>46203.54697321759</v>
@@ -23090,7 +23126,7 @@
         <v>83</v>
       </c>
       <c r="F293" s="12" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="G293" s="12" t="s">
         <v>32</v>
@@ -23125,17 +23161,17 @@
         <v>35</v>
       </c>
       <c r="S293" s="12" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="T293" s="12" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="U293" s="8" t="s">
         <v>116</v>
       </c>
       <c r="V293" s="12"/>
       <c r="W293" s="9" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="X293" s="12">
         <v>0</v>
@@ -23144,7 +23180,7 @@
     </row>
     <row r="294" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A294" s="4" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="B294" s="5">
         <v>46203.54697938658</v>
@@ -23157,7 +23193,7 @@
         <v>153</v>
       </c>
       <c r="F294" s="6" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="G294" s="6" t="s">
         <v>32</v>
@@ -23192,17 +23228,17 @@
         <v>35</v>
       </c>
       <c r="S294" s="6" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="T294" s="6" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="U294" s="8" t="s">
         <v>116</v>
       </c>
       <c r="V294" s="6"/>
       <c r="W294" s="9" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="X294" s="6">
         <v>0</v>
@@ -23211,7 +23247,7 @@
     </row>
     <row r="295" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A295" s="10" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="B295" s="11">
         <v>46203.60974886574</v>
@@ -23224,7 +23260,7 @@
         <v>40</v>
       </c>
       <c r="F295" s="12" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="G295" s="12" t="s">
         <v>41</v>
@@ -23261,17 +23297,17 @@
         <v>35</v>
       </c>
       <c r="S295" s="12" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="T295" s="12" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="U295" s="8" t="s">
         <v>141</v>
       </c>
       <c r="V295" s="12"/>
       <c r="W295" s="9" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="X295" s="12">
         <v>0</v>
@@ -23280,7 +23316,7 @@
     </row>
     <row r="296" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A296" s="4" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="B296" s="5">
         <v>46203.60975423611</v>
@@ -23293,7 +23329,7 @@
         <v>83</v>
       </c>
       <c r="F296" s="6" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="G296" s="6" t="s">
         <v>30</v>
@@ -23330,17 +23366,17 @@
         <v>35</v>
       </c>
       <c r="S296" s="6" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="T296" s="6" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="U296" s="8" t="s">
         <v>141</v>
       </c>
       <c r="V296" s="6"/>
       <c r="W296" s="9" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="X296" s="6">
         <v>0</v>
@@ -23349,7 +23385,7 @@
     </row>
     <row r="297" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A297" s="10" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="B297" s="11">
         <v>46203.609769965275</v>
@@ -23362,7 +23398,7 @@
         <v>153</v>
       </c>
       <c r="F297" s="12" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="G297" s="12" t="s">
         <v>44</v>
@@ -23399,17 +23435,17 @@
         <v>35</v>
       </c>
       <c r="S297" s="12" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="T297" s="12" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="U297" s="8" t="s">
         <v>141</v>
       </c>
       <c r="V297" s="12"/>
       <c r="W297" s="9" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="X297" s="12">
         <v>0</v>
@@ -23418,20 +23454,22 @@
     </row>
     <row r="298" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A298" s="4" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="B298" s="5">
         <v>46203.61393550926</v>
       </c>
-      <c r="C298" s="6"/>
+      <c r="C298" s="5">
+        <v>46205.5384646412</v>
+      </c>
       <c r="D298" s="5">
-        <v>46203.8987362037</v>
+        <v>46205.69470920139</v>
       </c>
       <c r="E298" s="6" t="s">
         <v>40</v>
       </c>
       <c r="F298" s="6" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="G298" s="6" t="s">
         <v>56</v>
@@ -23468,35 +23506,37 @@
         <v>35</v>
       </c>
       <c r="S298" s="6" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="T298" s="6"/>
       <c r="U298" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="V298" s="6"/>
+      <c r="V298" s="5">
+        <v>46204</v>
+      </c>
       <c r="W298" s="6"/>
       <c r="X298" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y298" s="6"/>
     </row>
     <row r="299" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A299" s="10" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="B299" s="11">
         <v>46203.61394043981</v>
       </c>
       <c r="C299" s="12"/>
       <c r="D299" s="11">
-        <v>46203.898774710644</v>
+        <v>46205.693766944445</v>
       </c>
       <c r="E299" s="12" t="s">
         <v>83</v>
       </c>
       <c r="F299" s="12" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="G299" s="12" t="s">
         <v>30</v>
@@ -23533,7 +23573,7 @@
         <v>35</v>
       </c>
       <c r="S299" s="12" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="T299" s="12"/>
       <c r="U299" s="8" t="s">
@@ -23548,20 +23588,20 @@
     </row>
     <row r="300" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A300" s="4" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="B300" s="5">
         <v>46203.61395409722</v>
       </c>
       <c r="C300" s="6"/>
       <c r="D300" s="5">
-        <v>46203.89882076389</v>
+        <v>46205.69377196759</v>
       </c>
       <c r="E300" s="6" t="s">
         <v>153</v>
       </c>
       <c r="F300" s="6" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="G300" s="6" t="s">
         <v>44</v>
@@ -23598,7 +23638,7 @@
         <v>35</v>
       </c>
       <c r="S300" s="6" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="T300" s="6"/>
       <c r="U300" s="8" t="s">
@@ -23613,20 +23653,22 @@
     </row>
     <row r="301" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A301" s="10" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="B301" s="11">
         <v>46203.61614737268</v>
       </c>
-      <c r="C301" s="12"/>
+      <c r="C301" s="11">
+        <v>46205.538357997684</v>
+      </c>
       <c r="D301" s="11">
-        <v>46203.898326435185</v>
+        <v>46205.74700539352</v>
       </c>
       <c r="E301" s="12" t="s">
         <v>40</v>
       </c>
       <c r="F301" s="12" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="G301" s="12" t="s">
         <v>56</v>
@@ -23663,33 +23705,39 @@
         <v>35</v>
       </c>
       <c r="S301" s="12" t="s">
-        <v>639</v>
-      </c>
-      <c r="T301" s="12"/>
+        <v>640</v>
+      </c>
+      <c r="T301" s="12" t="s">
+        <v>641</v>
+      </c>
       <c r="U301" s="12"/>
-      <c r="V301" s="12"/>
-      <c r="W301" s="12"/>
+      <c r="V301" s="11">
+        <v>46204</v>
+      </c>
+      <c r="W301" s="9" t="s">
+        <v>641</v>
+      </c>
       <c r="X301" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y301" s="12"/>
     </row>
     <row r="302" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A302" s="4" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="B302" s="5">
         <v>46203.6161543287</v>
       </c>
       <c r="C302" s="6"/>
       <c r="D302" s="5">
-        <v>46203.898378391204</v>
+        <v>46205.747005937505</v>
       </c>
       <c r="E302" s="6" t="s">
         <v>83</v>
       </c>
       <c r="F302" s="6" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="G302" s="6" t="s">
         <v>30</v>
@@ -23726,12 +23774,16 @@
         <v>35</v>
       </c>
       <c r="S302" s="6" t="s">
-        <v>639</v>
-      </c>
-      <c r="T302" s="6"/>
+        <v>640</v>
+      </c>
+      <c r="T302" s="6" t="s">
+        <v>641</v>
+      </c>
       <c r="U302" s="6"/>
       <c r="V302" s="6"/>
-      <c r="W302" s="6"/>
+      <c r="W302" s="9" t="s">
+        <v>641</v>
+      </c>
       <c r="X302" s="6">
         <v>0</v>
       </c>
@@ -23739,20 +23791,20 @@
     </row>
     <row r="303" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A303" s="10" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="B303" s="11">
         <v>46203.616170381945</v>
       </c>
       <c r="C303" s="12"/>
       <c r="D303" s="11">
-        <v>46203.89842915509</v>
+        <v>46205.74700643518</v>
       </c>
       <c r="E303" s="12" t="s">
         <v>153</v>
       </c>
       <c r="F303" s="12" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="G303" s="12" t="s">
         <v>44</v>
@@ -23789,12 +23841,16 @@
         <v>35</v>
       </c>
       <c r="S303" s="12" t="s">
-        <v>639</v>
-      </c>
-      <c r="T303" s="12"/>
+        <v>640</v>
+      </c>
+      <c r="T303" s="12" t="s">
+        <v>641</v>
+      </c>
       <c r="U303" s="12"/>
       <c r="V303" s="12"/>
-      <c r="W303" s="12"/>
+      <c r="W303" s="9" t="s">
+        <v>641</v>
+      </c>
       <c r="X303" s="12">
         <v>0</v>
       </c>
@@ -23802,7 +23858,7 @@
     </row>
     <row r="304" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A304" s="4" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
       <c r="B304" s="5">
         <v>46203.800516655094</v>
@@ -23815,7 +23871,7 @@
         <v>40</v>
       </c>
       <c r="F304" s="6" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="G304" s="6" t="s">
         <v>32</v>
@@ -23848,17 +23904,17 @@
         <v>35</v>
       </c>
       <c r="S304" s="6" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
       <c r="T304" s="6" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
       <c r="U304" s="8" t="s">
         <v>95</v>
       </c>
       <c r="V304" s="6"/>
       <c r="W304" s="9" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
       <c r="X304" s="6">
         <v>0</v>
@@ -23867,7 +23923,7 @@
     </row>
     <row r="305" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A305" s="10" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="B305" s="11">
         <v>46203.80053320602</v>
@@ -23880,7 +23936,7 @@
         <v>83</v>
       </c>
       <c r="F305" s="12" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="G305" s="12" t="s">
         <v>32</v>
@@ -23913,17 +23969,17 @@
         <v>35</v>
       </c>
       <c r="S305" s="12" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
       <c r="T305" s="12" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
       <c r="U305" s="8" t="s">
         <v>95</v>
       </c>
       <c r="V305" s="12"/>
       <c r="W305" s="9" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
       <c r="X305" s="12">
         <v>0</v>
@@ -23932,7 +23988,7 @@
     </row>
     <row r="306" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A306" s="4" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
       <c r="B306" s="5">
         <v>46203.80053798611</v>
@@ -23945,7 +24001,7 @@
         <v>153</v>
       </c>
       <c r="F306" s="6" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="G306" s="6" t="s">
         <v>32</v>
@@ -23978,22 +24034,229 @@
         <v>35</v>
       </c>
       <c r="S306" s="6" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
       <c r="T306" s="6" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
       <c r="U306" s="8" t="s">
         <v>95</v>
       </c>
       <c r="V306" s="6"/>
       <c r="W306" s="9" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
       <c r="X306" s="6">
         <v>0</v>
       </c>
       <c r="Y306" s="6"/>
+    </row>
+    <row r="307" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A307" s="10" t="s">
+        <v>650</v>
+      </c>
+      <c r="B307" s="11">
+        <v>46205.69645481481</v>
+      </c>
+      <c r="C307" s="11">
+        <v>46205.745780694444</v>
+      </c>
+      <c r="D307" s="11">
+        <v>46205.74591362268</v>
+      </c>
+      <c r="E307" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="F307" s="12" t="s">
+        <v>651</v>
+      </c>
+      <c r="G307" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="H307" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="I307" s="12"/>
+      <c r="J307" s="11">
+        <v>46204</v>
+      </c>
+      <c r="K307" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="L307" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="M307" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N307" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="O307" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="P307" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q307" s="7" t="s">
+        <v>600</v>
+      </c>
+      <c r="R307" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S307" s="12" t="s">
+        <v>652</v>
+      </c>
+      <c r="T307" s="12" t="s">
+        <v>653</v>
+      </c>
+      <c r="U307" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="V307" s="11">
+        <v>46204</v>
+      </c>
+      <c r="W307" s="9" t="s">
+        <v>653</v>
+      </c>
+      <c r="X307" s="12">
+        <v>0.1</v>
+      </c>
+      <c r="Y307" s="12"/>
+    </row>
+    <row r="308" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A308" s="4" t="s">
+        <v>654</v>
+      </c>
+      <c r="B308" s="5">
+        <v>46205.69646774305</v>
+      </c>
+      <c r="C308" s="6"/>
+      <c r="D308" s="5">
+        <v>46205.69730648148</v>
+      </c>
+      <c r="E308" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="F308" s="6" t="s">
+        <v>651</v>
+      </c>
+      <c r="G308" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H308" s="6"/>
+      <c r="I308" s="6"/>
+      <c r="J308" s="5">
+        <v>46204</v>
+      </c>
+      <c r="K308" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="L308" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="M308" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N308" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="O308" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="P308" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q308" s="7" t="s">
+        <v>600</v>
+      </c>
+      <c r="R308" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S308" s="6" t="s">
+        <v>652</v>
+      </c>
+      <c r="T308" s="6" t="s">
+        <v>653</v>
+      </c>
+      <c r="U308" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="V308" s="6"/>
+      <c r="W308" s="9" t="s">
+        <v>653</v>
+      </c>
+      <c r="X308" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y308" s="6"/>
+    </row>
+    <row r="309" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A309" s="10" t="s">
+        <v>655</v>
+      </c>
+      <c r="B309" s="11">
+        <v>46205.696475439814</v>
+      </c>
+      <c r="C309" s="12"/>
+      <c r="D309" s="11">
+        <v>46205.74578806713</v>
+      </c>
+      <c r="E309" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="F309" s="12" t="s">
+        <v>651</v>
+      </c>
+      <c r="G309" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="H309" s="12"/>
+      <c r="I309" s="12"/>
+      <c r="J309" s="11">
+        <v>46204</v>
+      </c>
+      <c r="K309" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="L309" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="M309" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N309" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="O309" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="P309" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q309" s="7" t="s">
+        <v>600</v>
+      </c>
+      <c r="R309" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S309" s="12" t="s">
+        <v>652</v>
+      </c>
+      <c r="T309" s="12" t="s">
+        <v>653</v>
+      </c>
+      <c r="U309" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="V309" s="12"/>
+      <c r="W309" s="9" t="s">
+        <v>653</v>
+      </c>
+      <c r="X309" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y309" s="12"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Actualizar dashboard Oferta Zitron 2026 2026-07-06 16:50 UTC
</commit_message>
<xml_diff>
--- a/data_ofertas/Oferta Zitron 2026.xlsx
+++ b/data_ofertas/Oferta Zitron 2026.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5053" uniqueCount="656">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5332" uniqueCount="689">
   <si>
     <t>Oferta Zitron 2026</t>
   </si>
@@ -1946,6 +1946,24 @@
     <t>1216159042508937</t>
   </si>
   <si>
+    <t>1216309131400281</t>
+  </si>
+  <si>
+    <t>26MX0060A - Minera Tizapa (peñoles)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minera Tizapa </t>
+  </si>
+  <si>
+    <t>26MX0060A</t>
+  </si>
+  <si>
+    <t>1216308892649162</t>
+  </si>
+  <si>
+    <t>1216309039007177</t>
+  </si>
+  <si>
     <t>1216191030213996</t>
   </si>
   <si>
@@ -1980,6 +1998,87 @@
   </si>
   <si>
     <t>1216245532454105</t>
+  </si>
+  <si>
+    <t>1216302054264585</t>
+  </si>
+  <si>
+    <t>Capex 2027 Fresnillo PLC. Mina Fresnillo</t>
+  </si>
+  <si>
+    <t>Fresnillo</t>
+  </si>
+  <si>
+    <t>1216302176593404</t>
+  </si>
+  <si>
+    <t>1216302176276751</t>
+  </si>
+  <si>
+    <t>1216307636821847</t>
+  </si>
+  <si>
+    <t>25PE0024 - Condestable</t>
+  </si>
+  <si>
+    <t>Condestable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25PE0024 </t>
+  </si>
+  <si>
+    <t>1216307956141200</t>
+  </si>
+  <si>
+    <t>1216307691889645</t>
+  </si>
+  <si>
+    <t>1216307694294073</t>
+  </si>
+  <si>
+    <t>26CL0001 - CRTG Reparacion</t>
+  </si>
+  <si>
+    <t>1216307694294092</t>
+  </si>
+  <si>
+    <t>1216307958592302</t>
+  </si>
+  <si>
+    <t>1216308605988824</t>
+  </si>
+  <si>
+    <t>26CO0019 - Aris Mining Compra en colombia.Dejar comision del 3% para el cliente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aris Mining </t>
+  </si>
+  <si>
+    <t xml:space="preserve">26CO0019 </t>
+  </si>
+  <si>
+    <t>1216308605988843</t>
+  </si>
+  <si>
+    <t>1216308605975590</t>
+  </si>
+  <si>
+    <t>1216309031807087</t>
+  </si>
+  <si>
+    <t>26PE0025 - LINCUNA</t>
+  </si>
+  <si>
+    <t>LINCUNA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26PE0025 </t>
+  </si>
+  <si>
+    <t>1216309135895502</t>
+  </si>
+  <si>
+    <t>1216309407658435</t>
   </si>
 </sst>
 </file>
@@ -2503,7 +2602,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Y309"/>
+  <dimension ref="A1:Y327"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10.4" customWidth="1"/>
@@ -2773,7 +2872,7 @@
         <v>46160.87336363426</v>
       </c>
       <c r="D6" s="5">
-        <v>46169.129010868055</v>
+        <v>46209.698053935186</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>33</v>
@@ -2789,7 +2888,7 @@
       </c>
       <c r="I6" s="6"/>
       <c r="J6" s="5">
-        <v>46076</v>
+        <v>46166</v>
       </c>
       <c r="K6" s="6" t="s">
         <v>32</v>
@@ -5201,9 +5300,11 @@
       <c r="B40" s="5">
         <v>46139.626861956014</v>
       </c>
-      <c r="C40" s="6"/>
+      <c r="C40" s="5">
+        <v>46209.677002627315</v>
+      </c>
       <c r="D40" s="5">
-        <v>46146.65524590277</v>
+        <v>46209.67770237269</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>40</v>
@@ -5256,7 +5357,9 @@
       <c r="U40" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="V40" s="6"/>
+      <c r="V40" s="5">
+        <v>46206</v>
+      </c>
       <c r="W40" s="9" t="s">
         <v>129</v>
       </c>
@@ -5272,9 +5375,11 @@
       <c r="B41" s="11">
         <v>46139.626905219906</v>
       </c>
-      <c r="C41" s="12"/>
+      <c r="C41" s="11">
+        <v>46209.67695857639</v>
+      </c>
       <c r="D41" s="11">
-        <v>46155.721906597224</v>
+        <v>46209.67770303241</v>
       </c>
       <c r="E41" s="12" t="s">
         <v>83</v>
@@ -5327,7 +5432,9 @@
       <c r="U41" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="V41" s="12"/>
+      <c r="V41" s="11">
+        <v>46206</v>
+      </c>
       <c r="W41" s="9" t="s">
         <v>129</v>
       </c>
@@ -5343,9 +5450,11 @@
       <c r="B42" s="5">
         <v>46139.752653993055</v>
       </c>
-      <c r="C42" s="6"/>
+      <c r="C42" s="5">
+        <v>46209.67704334491</v>
+      </c>
       <c r="D42" s="5">
-        <v>46146.65526381944</v>
+        <v>46209.67770355324</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>33</v>
@@ -5398,7 +5507,9 @@
       <c r="U42" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="V42" s="6"/>
+      <c r="V42" s="5">
+        <v>46206</v>
+      </c>
       <c r="W42" s="9" t="s">
         <v>129</v>
       </c>
@@ -5414,9 +5525,11 @@
       <c r="B43" s="11">
         <v>46146.59164503472</v>
       </c>
-      <c r="C43" s="12"/>
+      <c r="C43" s="11">
+        <v>46209.67705643519</v>
+      </c>
       <c r="D43" s="11">
-        <v>46180.600272800926</v>
+        <v>46209.677860254626</v>
       </c>
       <c r="E43" s="12" t="s">
         <v>40</v>
@@ -5467,7 +5580,9 @@
       <c r="U43" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="V43" s="12"/>
+      <c r="V43" s="11">
+        <v>46206</v>
+      </c>
       <c r="W43" s="9" t="s">
         <v>129</v>
       </c>
@@ -5483,9 +5598,11 @@
       <c r="B44" s="5">
         <v>46146.59165107639</v>
       </c>
-      <c r="C44" s="6"/>
+      <c r="C44" s="5">
+        <v>46209.67706408565</v>
+      </c>
       <c r="D44" s="5">
-        <v>46155.839989224536</v>
+        <v>46209.67786081019</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>83</v>
@@ -5536,7 +5653,9 @@
       <c r="U44" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="V44" s="6"/>
+      <c r="V44" s="5">
+        <v>46206</v>
+      </c>
       <c r="W44" s="9" t="s">
         <v>129</v>
       </c>
@@ -5552,9 +5671,11 @@
       <c r="B45" s="11">
         <v>46146.59166475694</v>
       </c>
-      <c r="C45" s="12"/>
+      <c r="C45" s="11">
+        <v>46209.67710688658</v>
+      </c>
       <c r="D45" s="11">
-        <v>46155.840025</v>
+        <v>46209.67786138889</v>
       </c>
       <c r="E45" s="12" t="s">
         <v>33</v>
@@ -5605,7 +5726,9 @@
       <c r="U45" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="V45" s="12"/>
+      <c r="V45" s="11">
+        <v>46206</v>
+      </c>
       <c r="W45" s="9" t="s">
         <v>129</v>
       </c>
@@ -6432,7 +6555,7 @@
         <v>46141.591915833334</v>
       </c>
       <c r="D57" s="11">
-        <v>46160.592815763885</v>
+        <v>46209.68118792824</v>
       </c>
       <c r="E57" s="12" t="s">
         <v>153</v>
@@ -6486,7 +6609,7 @@
         <v>95</v>
       </c>
       <c r="V57" s="11">
-        <v>46129</v>
+        <v>46160</v>
       </c>
       <c r="W57" s="9" t="s">
         <v>162</v>
@@ -13311,9 +13434,11 @@
       <c r="B154" s="5">
         <v>46155.65621130787</v>
       </c>
-      <c r="C154" s="6"/>
+      <c r="C154" s="5">
+        <v>46209.690346828706</v>
+      </c>
       <c r="D154" s="5">
-        <v>46188.84417585648</v>
+        <v>46209.69048982639</v>
       </c>
       <c r="E154" s="6" t="s">
         <v>40</v>
@@ -13366,7 +13491,9 @@
       <c r="U154" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="V154" s="6"/>
+      <c r="V154" s="5">
+        <v>46203</v>
+      </c>
       <c r="W154" s="9" t="s">
         <v>358</v>
       </c>
@@ -13382,9 +13509,11 @@
       <c r="B155" s="11">
         <v>46155.65621641204</v>
       </c>
-      <c r="C155" s="12"/>
+      <c r="C155" s="11">
+        <v>46209.690368125</v>
+      </c>
       <c r="D155" s="11">
-        <v>46188.844253020834</v>
+        <v>46209.69049034722</v>
       </c>
       <c r="E155" s="12" t="s">
         <v>83</v>
@@ -13437,7 +13566,9 @@
       <c r="U155" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="V155" s="12"/>
+      <c r="V155" s="11">
+        <v>46203</v>
+      </c>
       <c r="W155" s="9" t="s">
         <v>358</v>
       </c>
@@ -13453,9 +13584,11 @@
       <c r="B156" s="5">
         <v>46155.65622783564</v>
       </c>
-      <c r="C156" s="6"/>
+      <c r="C156" s="5">
+        <v>46209.69041228009</v>
+      </c>
       <c r="D156" s="5">
-        <v>46188.844285625004</v>
+        <v>46209.69049086806</v>
       </c>
       <c r="E156" s="6" t="s">
         <v>153</v>
@@ -13508,7 +13641,9 @@
       <c r="U156" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="V156" s="6"/>
+      <c r="V156" s="5">
+        <v>46203</v>
+      </c>
       <c r="W156" s="9" t="s">
         <v>358</v>
       </c>
@@ -13674,7 +13809,7 @@
         <v>46168.89510594908</v>
       </c>
       <c r="D159" s="11">
-        <v>46169.131401226856</v>
+        <v>46209.69123590278</v>
       </c>
       <c r="E159" s="12" t="s">
         <v>153</v>
@@ -13726,7 +13861,7 @@
         <v>141</v>
       </c>
       <c r="V159" s="11">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="W159" s="9" t="s">
         <v>364</v>
@@ -15185,7 +15320,7 @@
         <v>46185.58422899306</v>
       </c>
       <c r="D180" s="5">
-        <v>46185.584230416665</v>
+        <v>46209.689411168976</v>
       </c>
       <c r="E180" s="6" t="s">
         <v>153</v>
@@ -15235,7 +15370,7 @@
         <v>405</v>
       </c>
       <c r="V180" s="5">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="W180" s="9" t="s">
         <v>404</v>
@@ -15465,9 +15600,11 @@
       <c r="B184" s="5">
         <v>46162.834460949074</v>
       </c>
-      <c r="C184" s="6"/>
+      <c r="C184" s="5">
+        <v>46209.595849537036</v>
+      </c>
       <c r="D184" s="5">
-        <v>46188.84522106481</v>
+        <v>46209.59606409722</v>
       </c>
       <c r="E184" s="6" t="s">
         <v>40</v>
@@ -15518,12 +15655,14 @@
       <c r="U184" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="V184" s="6"/>
+      <c r="V184" s="5">
+        <v>46206</v>
+      </c>
       <c r="W184" s="9" t="s">
         <v>417</v>
       </c>
       <c r="X184" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y184" s="6"/>
     </row>
@@ -15534,9 +15673,11 @@
       <c r="B185" s="11">
         <v>46162.83446643519</v>
       </c>
-      <c r="C185" s="12"/>
+      <c r="C185" s="11">
+        <v>46209.59587217592</v>
+      </c>
       <c r="D185" s="11">
-        <v>46188.845266296295</v>
+        <v>46209.596110451384</v>
       </c>
       <c r="E185" s="12" t="s">
         <v>83</v>
@@ -15587,12 +15728,14 @@
       <c r="U185" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="V185" s="12"/>
+      <c r="V185" s="11">
+        <v>46206</v>
+      </c>
       <c r="W185" s="9" t="s">
         <v>417</v>
       </c>
       <c r="X185" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y185" s="12"/>
     </row>
@@ -15603,9 +15746,11 @@
       <c r="B186" s="5">
         <v>46162.83447847222</v>
       </c>
-      <c r="C186" s="6"/>
+      <c r="C186" s="5">
+        <v>46209.692366863426</v>
+      </c>
       <c r="D186" s="5">
-        <v>46188.84529938658</v>
+        <v>46209.69248355324</v>
       </c>
       <c r="E186" s="6" t="s">
         <v>153</v>
@@ -15656,12 +15801,14 @@
       <c r="U186" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="V186" s="6"/>
+      <c r="V186" s="5">
+        <v>46206</v>
+      </c>
       <c r="W186" s="9" t="s">
         <v>417</v>
       </c>
       <c r="X186" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y186" s="6"/>
     </row>
@@ -16256,7 +16403,7 @@
         <v>46177.55503821759</v>
       </c>
       <c r="D195" s="11">
-        <v>46177.558142141206</v>
+        <v>46209.68604188657</v>
       </c>
       <c r="E195" s="12" t="s">
         <v>153</v>
@@ -16306,7 +16453,7 @@
         <v>95</v>
       </c>
       <c r="V195" s="11">
-        <v>46176</v>
+        <v>46175</v>
       </c>
       <c r="W195" s="9" t="s">
         <v>434</v>
@@ -18019,9 +18166,11 @@
       <c r="B220" s="5">
         <v>46171.541563032406</v>
       </c>
-      <c r="C220" s="6"/>
+      <c r="C220" s="5">
+        <v>46209.69275125</v>
+      </c>
       <c r="D220" s="5">
-        <v>46188.84614569445</v>
+        <v>46209.692897141205</v>
       </c>
       <c r="E220" s="6" t="s">
         <v>40</v>
@@ -18074,12 +18223,14 @@
       <c r="U220" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="V220" s="6"/>
+      <c r="V220" s="5">
+        <v>46206</v>
+      </c>
       <c r="W220" s="9" t="s">
         <v>485</v>
       </c>
       <c r="X220" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y220" s="6"/>
     </row>
@@ -18090,9 +18241,11 @@
       <c r="B221" s="11">
         <v>46171.541569594905</v>
       </c>
-      <c r="C221" s="12"/>
+      <c r="C221" s="11">
+        <v>46209.69275806713</v>
+      </c>
       <c r="D221" s="11">
-        <v>46188.8461966551</v>
+        <v>46209.69289769676</v>
       </c>
       <c r="E221" s="12" t="s">
         <v>83</v>
@@ -18145,12 +18298,14 @@
       <c r="U221" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="V221" s="12"/>
+      <c r="V221" s="11">
+        <v>46206</v>
+      </c>
       <c r="W221" s="9" t="s">
         <v>485</v>
       </c>
       <c r="X221" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y221" s="12"/>
     </row>
@@ -18161,9 +18316,11 @@
       <c r="B222" s="5">
         <v>46171.54158304398</v>
       </c>
-      <c r="C222" s="6"/>
+      <c r="C222" s="5">
+        <v>46209.69280556713</v>
+      </c>
       <c r="D222" s="5">
-        <v>46188.84623487269</v>
+        <v>46209.69289822917</v>
       </c>
       <c r="E222" s="6" t="s">
         <v>153</v>
@@ -18216,12 +18373,14 @@
       <c r="U222" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="V222" s="6"/>
+      <c r="V222" s="5">
+        <v>46206</v>
+      </c>
       <c r="W222" s="9" t="s">
         <v>485</v>
       </c>
       <c r="X222" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y222" s="6"/>
     </row>
@@ -19520,7 +19679,7 @@
         <v>46178.71568760417</v>
       </c>
       <c r="D241" s="11">
-        <v>46188.851797511576</v>
+        <v>46209.69178057871</v>
       </c>
       <c r="E241" s="12" t="s">
         <v>40</v>
@@ -19578,7 +19737,7 @@
         <v>530</v>
       </c>
       <c r="X241" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y241" s="12"/>
     </row>
@@ -19593,7 +19752,7 @@
         <v>46178.71550456018</v>
       </c>
       <c r="D242" s="5">
-        <v>46188.85182652778</v>
+        <v>46209.69178112269</v>
       </c>
       <c r="E242" s="6" t="s">
         <v>83</v>
@@ -19651,7 +19810,7 @@
         <v>530</v>
       </c>
       <c r="X242" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y242" s="6"/>
     </row>
@@ -19666,7 +19825,7 @@
         <v>46178.71575603009</v>
       </c>
       <c r="D243" s="11">
-        <v>46188.85186135417</v>
+        <v>46209.69178159723</v>
       </c>
       <c r="E243" s="12" t="s">
         <v>153</v>
@@ -19724,7 +19883,7 @@
         <v>530</v>
       </c>
       <c r="X243" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y243" s="12"/>
     </row>
@@ -23252,9 +23411,11 @@
       <c r="B295" s="11">
         <v>46203.60974886574</v>
       </c>
-      <c r="C295" s="12"/>
+      <c r="C295" s="11">
+        <v>46209.595248541664</v>
+      </c>
       <c r="D295" s="11">
-        <v>46203.79287297453</v>
+        <v>46209.59552325231</v>
       </c>
       <c r="E295" s="12" t="s">
         <v>40</v>
@@ -23305,12 +23466,14 @@
       <c r="U295" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="V295" s="12"/>
+      <c r="V295" s="11">
+        <v>46203</v>
+      </c>
       <c r="W295" s="9" t="s">
         <v>630</v>
       </c>
       <c r="X295" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y295" s="12"/>
     </row>
@@ -23321,9 +23484,11 @@
       <c r="B296" s="5">
         <v>46203.60975423611</v>
       </c>
-      <c r="C296" s="6"/>
+      <c r="C296" s="5">
+        <v>46209.595320520835</v>
+      </c>
       <c r="D296" s="5">
-        <v>46203.79298378472</v>
+        <v>46209.595523854165</v>
       </c>
       <c r="E296" s="6" t="s">
         <v>83</v>
@@ -23374,12 +23539,14 @@
       <c r="U296" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="V296" s="6"/>
+      <c r="V296" s="5">
+        <v>46203</v>
+      </c>
       <c r="W296" s="9" t="s">
         <v>630</v>
       </c>
       <c r="X296" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y296" s="6"/>
     </row>
@@ -23390,9 +23557,11 @@
       <c r="B297" s="11">
         <v>46203.609769965275</v>
       </c>
-      <c r="C297" s="12"/>
+      <c r="C297" s="11">
+        <v>46209.595356342594</v>
+      </c>
       <c r="D297" s="11">
-        <v>46203.79292857639</v>
+        <v>46209.59552444445</v>
       </c>
       <c r="E297" s="12" t="s">
         <v>153</v>
@@ -23443,12 +23612,14 @@
       <c r="U297" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="V297" s="12"/>
+      <c r="V297" s="11">
+        <v>46203</v>
+      </c>
       <c r="W297" s="9" t="s">
         <v>630</v>
       </c>
       <c r="X297" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y297" s="12"/>
     </row>
@@ -23729,9 +23900,11 @@
       <c r="B302" s="5">
         <v>46203.6161543287</v>
       </c>
-      <c r="C302" s="6"/>
+      <c r="C302" s="5">
+        <v>46209.693145833335</v>
+      </c>
       <c r="D302" s="5">
-        <v>46205.747005937505</v>
+        <v>46209.693251770834</v>
       </c>
       <c r="E302" s="6" t="s">
         <v>83</v>
@@ -23780,12 +23953,14 @@
         <v>641</v>
       </c>
       <c r="U302" s="6"/>
-      <c r="V302" s="6"/>
+      <c r="V302" s="5">
+        <v>46206</v>
+      </c>
       <c r="W302" s="9" t="s">
         <v>641</v>
       </c>
       <c r="X302" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y302" s="6"/>
     </row>
@@ -23796,9 +23971,11 @@
       <c r="B303" s="11">
         <v>46203.616170381945</v>
       </c>
-      <c r="C303" s="12"/>
+      <c r="C303" s="11">
+        <v>46209.693188958336</v>
+      </c>
       <c r="D303" s="11">
-        <v>46205.74700643518</v>
+        <v>46209.693252303245</v>
       </c>
       <c r="E303" s="12" t="s">
         <v>153</v>
@@ -23847,12 +24024,14 @@
         <v>641</v>
       </c>
       <c r="U303" s="12"/>
-      <c r="V303" s="12"/>
+      <c r="V303" s="11">
+        <v>46206</v>
+      </c>
       <c r="W303" s="9" t="s">
         <v>641</v>
       </c>
       <c r="X303" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y303" s="12"/>
     </row>
@@ -23861,11 +24040,13 @@
         <v>644</v>
       </c>
       <c r="B304" s="5">
-        <v>46203.800516655094</v>
-      </c>
-      <c r="C304" s="6"/>
+        <v>46209.69556905093</v>
+      </c>
+      <c r="C304" s="5">
+        <v>46209.69556883102</v>
+      </c>
       <c r="D304" s="5">
-        <v>46203.801443634264</v>
+        <v>46209.69710803241</v>
       </c>
       <c r="E304" s="6" t="s">
         <v>40</v>
@@ -23874,11 +24055,15 @@
         <v>645</v>
       </c>
       <c r="G304" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H304" s="6"/>
+        <v>56</v>
+      </c>
+      <c r="H304" s="6" t="s">
+        <v>57</v>
+      </c>
       <c r="I304" s="6"/>
-      <c r="J304" s="6"/>
+      <c r="J304" s="5">
+        <v>46203</v>
+      </c>
       <c r="K304" s="6" t="s">
         <v>32</v>
       </c>
@@ -23909,15 +24094,15 @@
       <c r="T304" s="6" t="s">
         <v>647</v>
       </c>
-      <c r="U304" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="V304" s="6"/>
+      <c r="U304" s="6"/>
+      <c r="V304" s="5">
+        <v>46204</v>
+      </c>
       <c r="W304" s="9" t="s">
         <v>647</v>
       </c>
       <c r="X304" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y304" s="6"/>
     </row>
@@ -23926,11 +24111,13 @@
         <v>648</v>
       </c>
       <c r="B305" s="11">
-        <v>46203.80053320602</v>
-      </c>
-      <c r="C305" s="12"/>
+        <v>46209.695574259254</v>
+      </c>
+      <c r="C305" s="11">
+        <v>46209.695574247686</v>
+      </c>
       <c r="D305" s="11">
-        <v>46203.80144418981</v>
+        <v>46209.69710858796</v>
       </c>
       <c r="E305" s="12" t="s">
         <v>83</v>
@@ -23939,11 +24126,15 @@
         <v>645</v>
       </c>
       <c r="G305" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H305" s="12"/>
+        <v>30</v>
+      </c>
+      <c r="H305" s="12" t="s">
+        <v>31</v>
+      </c>
       <c r="I305" s="12"/>
-      <c r="J305" s="12"/>
+      <c r="J305" s="11">
+        <v>46203</v>
+      </c>
       <c r="K305" s="12" t="s">
         <v>32</v>
       </c>
@@ -23974,15 +24165,15 @@
       <c r="T305" s="12" t="s">
         <v>647</v>
       </c>
-      <c r="U305" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="V305" s="12"/>
+      <c r="U305" s="12"/>
+      <c r="V305" s="11">
+        <v>46206</v>
+      </c>
       <c r="W305" s="9" t="s">
         <v>647</v>
       </c>
       <c r="X305" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y305" s="12"/>
     </row>
@@ -23991,11 +24182,13 @@
         <v>649</v>
       </c>
       <c r="B306" s="5">
-        <v>46203.80053798611</v>
-      </c>
-      <c r="C306" s="6"/>
+        <v>46209.69558688658</v>
+      </c>
+      <c r="C306" s="5">
+        <v>46209.69558664352</v>
+      </c>
       <c r="D306" s="5">
-        <v>46203.80144469907</v>
+        <v>46209.69710913194</v>
       </c>
       <c r="E306" s="6" t="s">
         <v>153</v>
@@ -24004,11 +24197,15 @@
         <v>645</v>
       </c>
       <c r="G306" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H306" s="6"/>
+        <v>44</v>
+      </c>
+      <c r="H306" s="6" t="s">
+        <v>45</v>
+      </c>
       <c r="I306" s="6"/>
-      <c r="J306" s="6"/>
+      <c r="J306" s="5">
+        <v>46203</v>
+      </c>
       <c r="K306" s="6" t="s">
         <v>32</v>
       </c>
@@ -24039,15 +24236,15 @@
       <c r="T306" s="6" t="s">
         <v>647</v>
       </c>
-      <c r="U306" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="V306" s="6"/>
+      <c r="U306" s="6"/>
+      <c r="V306" s="5">
+        <v>46206</v>
+      </c>
       <c r="W306" s="9" t="s">
         <v>647</v>
       </c>
       <c r="X306" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y306" s="6"/>
     </row>
@@ -24056,13 +24253,13 @@
         <v>650</v>
       </c>
       <c r="B307" s="11">
-        <v>46205.69645481481</v>
+        <v>46203.800516655094</v>
       </c>
       <c r="C307" s="11">
-        <v>46205.745780694444</v>
+        <v>46209.679211979164</v>
       </c>
       <c r="D307" s="11">
-        <v>46205.74591362268</v>
+        <v>46209.68072039352</v>
       </c>
       <c r="E307" s="12" t="s">
         <v>40</v>
@@ -24071,15 +24268,11 @@
         <v>651</v>
       </c>
       <c r="G307" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="H307" s="12" t="s">
-        <v>57</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="H307" s="12"/>
       <c r="I307" s="12"/>
-      <c r="J307" s="11">
-        <v>46204</v>
-      </c>
+      <c r="J307" s="12"/>
       <c r="K307" s="12" t="s">
         <v>32</v>
       </c>
@@ -24099,7 +24292,7 @@
         <v>153</v>
       </c>
       <c r="Q307" s="7" t="s">
-        <v>600</v>
+        <v>320</v>
       </c>
       <c r="R307" s="7" t="s">
         <v>35</v>
@@ -24111,16 +24304,16 @@
         <v>653</v>
       </c>
       <c r="U307" s="8" t="s">
-        <v>291</v>
+        <v>95</v>
       </c>
       <c r="V307" s="11">
-        <v>46204</v>
+        <v>46206</v>
       </c>
       <c r="W307" s="9" t="s">
         <v>653</v>
       </c>
       <c r="X307" s="12">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="Y307" s="12"/>
     </row>
@@ -24129,11 +24322,13 @@
         <v>654</v>
       </c>
       <c r="B308" s="5">
-        <v>46205.69646774305</v>
-      </c>
-      <c r="C308" s="6"/>
+        <v>46203.80053320602</v>
+      </c>
+      <c r="C308" s="5">
+        <v>46209.679220543985</v>
+      </c>
       <c r="D308" s="5">
-        <v>46205.69730648148</v>
+        <v>46209.680721006946</v>
       </c>
       <c r="E308" s="6" t="s">
         <v>83</v>
@@ -24146,9 +24341,7 @@
       </c>
       <c r="H308" s="6"/>
       <c r="I308" s="6"/>
-      <c r="J308" s="5">
-        <v>46204</v>
-      </c>
+      <c r="J308" s="6"/>
       <c r="K308" s="6" t="s">
         <v>32</v>
       </c>
@@ -24168,7 +24361,7 @@
         <v>153</v>
       </c>
       <c r="Q308" s="7" t="s">
-        <v>600</v>
+        <v>320</v>
       </c>
       <c r="R308" s="7" t="s">
         <v>35</v>
@@ -24180,14 +24373,16 @@
         <v>653</v>
       </c>
       <c r="U308" s="8" t="s">
-        <v>291</v>
-      </c>
-      <c r="V308" s="6"/>
+        <v>95</v>
+      </c>
+      <c r="V308" s="5">
+        <v>46206</v>
+      </c>
       <c r="W308" s="9" t="s">
         <v>653</v>
       </c>
       <c r="X308" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y308" s="6"/>
     </row>
@@ -24196,11 +24391,13 @@
         <v>655</v>
       </c>
       <c r="B309" s="11">
-        <v>46205.696475439814</v>
-      </c>
-      <c r="C309" s="12"/>
+        <v>46203.80053798611</v>
+      </c>
+      <c r="C309" s="11">
+        <v>46209.67928012731</v>
+      </c>
       <c r="D309" s="11">
-        <v>46205.74578806713</v>
+        <v>46209.68072159722</v>
       </c>
       <c r="E309" s="12" t="s">
         <v>153</v>
@@ -24213,9 +24410,7 @@
       </c>
       <c r="H309" s="12"/>
       <c r="I309" s="12"/>
-      <c r="J309" s="11">
-        <v>46204</v>
-      </c>
+      <c r="J309" s="12"/>
       <c r="K309" s="12" t="s">
         <v>32</v>
       </c>
@@ -24235,7 +24430,7 @@
         <v>32</v>
       </c>
       <c r="Q309" s="7" t="s">
-        <v>600</v>
+        <v>320</v>
       </c>
       <c r="R309" s="7" t="s">
         <v>35</v>
@@ -24247,16 +24442,1256 @@
         <v>653</v>
       </c>
       <c r="U309" s="8" t="s">
-        <v>291</v>
-      </c>
-      <c r="V309" s="12"/>
+        <v>95</v>
+      </c>
+      <c r="V309" s="11">
+        <v>46206</v>
+      </c>
       <c r="W309" s="9" t="s">
         <v>653</v>
       </c>
       <c r="X309" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y309" s="12"/>
+    </row>
+    <row r="310" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A310" s="4" t="s">
+        <v>656</v>
+      </c>
+      <c r="B310" s="5">
+        <v>46205.69645481481</v>
+      </c>
+      <c r="C310" s="5">
+        <v>46205.745780694444</v>
+      </c>
+      <c r="D310" s="5">
+        <v>46209.59670633102</v>
+      </c>
+      <c r="E310" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F310" s="6" t="s">
+        <v>657</v>
+      </c>
+      <c r="G310" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H310" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="I310" s="6"/>
+      <c r="J310" s="5">
+        <v>46204</v>
+      </c>
+      <c r="K310" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="L310" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="M310" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N310" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="O310" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="P310" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q310" s="7" t="s">
+        <v>600</v>
+      </c>
+      <c r="R310" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S310" s="6" t="s">
+        <v>658</v>
+      </c>
+      <c r="T310" s="6" t="s">
+        <v>659</v>
+      </c>
+      <c r="U310" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="V310" s="5">
+        <v>46204</v>
+      </c>
+      <c r="W310" s="9" t="s">
+        <v>659</v>
+      </c>
+      <c r="X310" s="6">
+        <v>1</v>
+      </c>
+      <c r="Y310" s="6"/>
+    </row>
+    <row r="311" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A311" s="10" t="s">
+        <v>660</v>
+      </c>
+      <c r="B311" s="11">
+        <v>46205.69646774305</v>
+      </c>
+      <c r="C311" s="11">
+        <v>46209.68901288194</v>
+      </c>
+      <c r="D311" s="11">
+        <v>46209.68908002315</v>
+      </c>
+      <c r="E311" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="F311" s="12" t="s">
+        <v>657</v>
+      </c>
+      <c r="G311" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="H311" s="12"/>
+      <c r="I311" s="12"/>
+      <c r="J311" s="11">
+        <v>46204</v>
+      </c>
+      <c r="K311" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="L311" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="M311" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N311" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="O311" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="P311" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q311" s="7" t="s">
+        <v>600</v>
+      </c>
+      <c r="R311" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S311" s="12" t="s">
+        <v>658</v>
+      </c>
+      <c r="T311" s="12" t="s">
+        <v>659</v>
+      </c>
+      <c r="U311" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="V311" s="11">
+        <v>46204</v>
+      </c>
+      <c r="W311" s="9" t="s">
+        <v>659</v>
+      </c>
+      <c r="X311" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y311" s="12"/>
+    </row>
+    <row r="312" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A312" s="4" t="s">
+        <v>661</v>
+      </c>
+      <c r="B312" s="5">
+        <v>46205.696475439814</v>
+      </c>
+      <c r="C312" s="5">
+        <v>46209.68904957176</v>
+      </c>
+      <c r="D312" s="5">
+        <v>46209.68911980324</v>
+      </c>
+      <c r="E312" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="F312" s="6" t="s">
+        <v>657</v>
+      </c>
+      <c r="G312" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H312" s="6"/>
+      <c r="I312" s="6"/>
+      <c r="J312" s="5">
+        <v>46204</v>
+      </c>
+      <c r="K312" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="L312" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="M312" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N312" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="O312" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="P312" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q312" s="7" t="s">
+        <v>600</v>
+      </c>
+      <c r="R312" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S312" s="6" t="s">
+        <v>658</v>
+      </c>
+      <c r="T312" s="6" t="s">
+        <v>659</v>
+      </c>
+      <c r="U312" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="V312" s="5">
+        <v>46204</v>
+      </c>
+      <c r="W312" s="9" t="s">
+        <v>659</v>
+      </c>
+      <c r="X312" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y312" s="6"/>
+    </row>
+    <row r="313" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A313" s="10" t="s">
+        <v>662</v>
+      </c>
+      <c r="B313" s="11">
+        <v>46209.59653997685</v>
+      </c>
+      <c r="C313" s="12"/>
+      <c r="D313" s="11">
+        <v>46209.59723758102</v>
+      </c>
+      <c r="E313" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="F313" s="12" t="s">
+        <v>663</v>
+      </c>
+      <c r="G313" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="H313" s="12"/>
+      <c r="I313" s="12"/>
+      <c r="J313" s="11">
+        <v>46209</v>
+      </c>
+      <c r="K313" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="L313" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="M313" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N313" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="O313" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="P313" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q313" s="7" t="s">
+        <v>600</v>
+      </c>
+      <c r="R313" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S313" s="12" t="s">
+        <v>664</v>
+      </c>
+      <c r="T313" s="12"/>
+      <c r="U313" s="12"/>
+      <c r="V313" s="12"/>
+      <c r="W313" s="12"/>
+      <c r="X313" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y313" s="12"/>
+    </row>
+    <row r="314" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A314" s="4" t="s">
+        <v>665</v>
+      </c>
+      <c r="B314" s="5">
+        <v>46209.596545925924</v>
+      </c>
+      <c r="C314" s="6"/>
+      <c r="D314" s="5">
+        <v>46209.59723829861</v>
+      </c>
+      <c r="E314" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="F314" s="6" t="s">
+        <v>663</v>
+      </c>
+      <c r="G314" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H314" s="6"/>
+      <c r="I314" s="6"/>
+      <c r="J314" s="5">
+        <v>46209</v>
+      </c>
+      <c r="K314" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="L314" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="M314" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N314" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="O314" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="P314" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q314" s="7" t="s">
+        <v>600</v>
+      </c>
+      <c r="R314" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S314" s="6" t="s">
+        <v>664</v>
+      </c>
+      <c r="T314" s="6"/>
+      <c r="U314" s="6"/>
+      <c r="V314" s="6"/>
+      <c r="W314" s="6"/>
+      <c r="X314" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y314" s="6"/>
+    </row>
+    <row r="315" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A315" s="10" t="s">
+        <v>666</v>
+      </c>
+      <c r="B315" s="11">
+        <v>46209.59655829861</v>
+      </c>
+      <c r="C315" s="12"/>
+      <c r="D315" s="11">
+        <v>46209.59723881945</v>
+      </c>
+      <c r="E315" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="F315" s="12" t="s">
+        <v>663</v>
+      </c>
+      <c r="G315" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="H315" s="12"/>
+      <c r="I315" s="12"/>
+      <c r="J315" s="11">
+        <v>46209</v>
+      </c>
+      <c r="K315" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="L315" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="M315" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N315" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="O315" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="P315" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q315" s="7" t="s">
+        <v>600</v>
+      </c>
+      <c r="R315" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S315" s="12" t="s">
+        <v>664</v>
+      </c>
+      <c r="T315" s="12"/>
+      <c r="U315" s="12"/>
+      <c r="V315" s="12"/>
+      <c r="W315" s="12"/>
+      <c r="X315" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y315" s="12"/>
+    </row>
+    <row r="316" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A316" s="4" t="s">
+        <v>667</v>
+      </c>
+      <c r="B316" s="5">
+        <v>46209.67231148148</v>
+      </c>
+      <c r="C316" s="5">
+        <v>46209.67251287037</v>
+      </c>
+      <c r="D316" s="5">
+        <v>46209.67377996528</v>
+      </c>
+      <c r="E316" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F316" s="6" t="s">
+        <v>668</v>
+      </c>
+      <c r="G316" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H316" s="6"/>
+      <c r="I316" s="6"/>
+      <c r="J316" s="6"/>
+      <c r="K316" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="L316" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="M316" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N316" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="O316" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="P316" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q316" s="7" t="s">
+        <v>600</v>
+      </c>
+      <c r="R316" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S316" s="6" t="s">
+        <v>669</v>
+      </c>
+      <c r="T316" s="6" t="s">
+        <v>670</v>
+      </c>
+      <c r="U316" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="V316" s="5">
+        <v>46205</v>
+      </c>
+      <c r="W316" s="9" t="s">
+        <v>670</v>
+      </c>
+      <c r="X316" s="6">
+        <v>1</v>
+      </c>
+      <c r="Y316" s="6"/>
+    </row>
+    <row r="317" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A317" s="10" t="s">
+        <v>671</v>
+      </c>
+      <c r="B317" s="11">
+        <v>46209.6723166088</v>
+      </c>
+      <c r="C317" s="11">
+        <v>46209.67251912037</v>
+      </c>
+      <c r="D317" s="11">
+        <v>46209.673780937504</v>
+      </c>
+      <c r="E317" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="F317" s="12" t="s">
+        <v>668</v>
+      </c>
+      <c r="G317" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="H317" s="12"/>
+      <c r="I317" s="12"/>
+      <c r="J317" s="12"/>
+      <c r="K317" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="L317" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="M317" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N317" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="O317" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="P317" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q317" s="7" t="s">
+        <v>600</v>
+      </c>
+      <c r="R317" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S317" s="12" t="s">
+        <v>669</v>
+      </c>
+      <c r="T317" s="12" t="s">
+        <v>670</v>
+      </c>
+      <c r="U317" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="V317" s="11">
+        <v>46205</v>
+      </c>
+      <c r="W317" s="9" t="s">
+        <v>670</v>
+      </c>
+      <c r="X317" s="12">
+        <v>1</v>
+      </c>
+      <c r="Y317" s="12"/>
+    </row>
+    <row r="318" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A318" s="4" t="s">
+        <v>672</v>
+      </c>
+      <c r="B318" s="5">
+        <v>46209.67233206019</v>
+      </c>
+      <c r="C318" s="5">
+        <v>46209.67256756945</v>
+      </c>
+      <c r="D318" s="5">
+        <v>46209.67378166667</v>
+      </c>
+      <c r="E318" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="F318" s="6" t="s">
+        <v>668</v>
+      </c>
+      <c r="G318" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H318" s="6"/>
+      <c r="I318" s="6"/>
+      <c r="J318" s="6"/>
+      <c r="K318" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="L318" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="M318" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N318" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="O318" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="P318" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q318" s="7" t="s">
+        <v>600</v>
+      </c>
+      <c r="R318" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S318" s="6" t="s">
+        <v>669</v>
+      </c>
+      <c r="T318" s="6" t="s">
+        <v>670</v>
+      </c>
+      <c r="U318" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="V318" s="5">
+        <v>46205</v>
+      </c>
+      <c r="W318" s="9" t="s">
+        <v>670</v>
+      </c>
+      <c r="X318" s="6">
+        <v>1</v>
+      </c>
+      <c r="Y318" s="6"/>
+    </row>
+    <row r="319" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A319" s="10" t="s">
+        <v>673</v>
+      </c>
+      <c r="B319" s="11">
+        <v>46209.67536922454</v>
+      </c>
+      <c r="C319" s="11">
+        <v>46209.67579587963</v>
+      </c>
+      <c r="D319" s="11">
+        <v>46209.675797523145</v>
+      </c>
+      <c r="E319" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="F319" s="12" t="s">
+        <v>674</v>
+      </c>
+      <c r="G319" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="H319" s="12"/>
+      <c r="I319" s="12"/>
+      <c r="J319" s="12"/>
+      <c r="K319" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="L319" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="M319" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N319" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="O319" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="P319" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q319" s="7" t="s">
+        <v>332</v>
+      </c>
+      <c r="R319" s="7" t="s">
+        <v>332</v>
+      </c>
+      <c r="S319" s="12" t="s">
+        <v>669</v>
+      </c>
+      <c r="T319" s="12" t="s">
+        <v>670</v>
+      </c>
+      <c r="U319" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="V319" s="11">
+        <v>46196</v>
+      </c>
+      <c r="W319" s="9" t="s">
+        <v>670</v>
+      </c>
+      <c r="X319" s="12">
+        <v>1</v>
+      </c>
+      <c r="Y319" s="12"/>
+    </row>
+    <row r="320" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A320" s="4" t="s">
+        <v>675</v>
+      </c>
+      <c r="B320" s="5">
+        <v>46209.675375023144</v>
+      </c>
+      <c r="C320" s="5">
+        <v>46209.67580091435</v>
+      </c>
+      <c r="D320" s="5">
+        <v>46209.675802453705</v>
+      </c>
+      <c r="E320" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="F320" s="6" t="s">
+        <v>674</v>
+      </c>
+      <c r="G320" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H320" s="6"/>
+      <c r="I320" s="6"/>
+      <c r="J320" s="6"/>
+      <c r="K320" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="L320" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="M320" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N320" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="O320" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="P320" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q320" s="7" t="s">
+        <v>332</v>
+      </c>
+      <c r="R320" s="7" t="s">
+        <v>332</v>
+      </c>
+      <c r="S320" s="6" t="s">
+        <v>669</v>
+      </c>
+      <c r="T320" s="6" t="s">
+        <v>670</v>
+      </c>
+      <c r="U320" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="V320" s="5">
+        <v>46196</v>
+      </c>
+      <c r="W320" s="9" t="s">
+        <v>670</v>
+      </c>
+      <c r="X320" s="6">
+        <v>1</v>
+      </c>
+      <c r="Y320" s="6"/>
+    </row>
+    <row r="321" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A321" s="10" t="s">
+        <v>676</v>
+      </c>
+      <c r="B321" s="11">
+        <v>46209.67539017361</v>
+      </c>
+      <c r="C321" s="11">
+        <v>46209.67538987269</v>
+      </c>
+      <c r="D321" s="11">
+        <v>46209.67580704861</v>
+      </c>
+      <c r="E321" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="F321" s="12" t="s">
+        <v>674</v>
+      </c>
+      <c r="G321" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="H321" s="12"/>
+      <c r="I321" s="12"/>
+      <c r="J321" s="12"/>
+      <c r="K321" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="L321" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="M321" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N321" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="O321" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="P321" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q321" s="7" t="s">
+        <v>332</v>
+      </c>
+      <c r="R321" s="7" t="s">
+        <v>332</v>
+      </c>
+      <c r="S321" s="12" t="s">
+        <v>669</v>
+      </c>
+      <c r="T321" s="12" t="s">
+        <v>670</v>
+      </c>
+      <c r="U321" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="V321" s="11">
+        <v>46196</v>
+      </c>
+      <c r="W321" s="9" t="s">
+        <v>670</v>
+      </c>
+      <c r="X321" s="12">
+        <v>1</v>
+      </c>
+      <c r="Y321" s="12"/>
+    </row>
+    <row r="322" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A322" s="4" t="s">
+        <v>677</v>
+      </c>
+      <c r="B322" s="5">
+        <v>46209.687911817135</v>
+      </c>
+      <c r="C322" s="5">
+        <v>46209.687911574074</v>
+      </c>
+      <c r="D322" s="5">
+        <v>46209.688580925926</v>
+      </c>
+      <c r="E322" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F322" s="6" t="s">
+        <v>678</v>
+      </c>
+      <c r="G322" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H322" s="6"/>
+      <c r="I322" s="6"/>
+      <c r="J322" s="5">
+        <v>46197</v>
+      </c>
+      <c r="K322" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="L322" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="M322" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N322" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="O322" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="P322" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q322" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="R322" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S322" s="6" t="s">
+        <v>679</v>
+      </c>
+      <c r="T322" s="6" t="s">
+        <v>680</v>
+      </c>
+      <c r="U322" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="V322" s="5">
+        <v>46198</v>
+      </c>
+      <c r="W322" s="9" t="s">
+        <v>670</v>
+      </c>
+      <c r="X322" s="6">
+        <v>1</v>
+      </c>
+      <c r="Y322" s="6"/>
+    </row>
+    <row r="323" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A323" s="10" t="s">
+        <v>681</v>
+      </c>
+      <c r="B323" s="11">
+        <v>46209.68791789352</v>
+      </c>
+      <c r="C323" s="11">
+        <v>46209.68791787037</v>
+      </c>
+      <c r="D323" s="11">
+        <v>46209.68859413195</v>
+      </c>
+      <c r="E323" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="F323" s="12" t="s">
+        <v>678</v>
+      </c>
+      <c r="G323" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="H323" s="12"/>
+      <c r="I323" s="12"/>
+      <c r="J323" s="11">
+        <v>46197</v>
+      </c>
+      <c r="K323" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="L323" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="M323" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N323" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="O323" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="P323" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q323" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="R323" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S323" s="12" t="s">
+        <v>679</v>
+      </c>
+      <c r="T323" s="12" t="s">
+        <v>680</v>
+      </c>
+      <c r="U323" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="V323" s="11">
+        <v>46198</v>
+      </c>
+      <c r="W323" s="9" t="s">
+        <v>670</v>
+      </c>
+      <c r="X323" s="12">
+        <v>1</v>
+      </c>
+      <c r="Y323" s="12"/>
+    </row>
+    <row r="324" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A324" s="4" t="s">
+        <v>682</v>
+      </c>
+      <c r="B324" s="5">
+        <v>46209.68793216435</v>
+      </c>
+      <c r="C324" s="5">
+        <v>46209.68793196759</v>
+      </c>
+      <c r="D324" s="5">
+        <v>46209.688607696764</v>
+      </c>
+      <c r="E324" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="F324" s="6" t="s">
+        <v>678</v>
+      </c>
+      <c r="G324" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H324" s="6"/>
+      <c r="I324" s="6"/>
+      <c r="J324" s="5">
+        <v>46197</v>
+      </c>
+      <c r="K324" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="L324" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="M324" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N324" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="O324" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="P324" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q324" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="R324" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S324" s="6" t="s">
+        <v>679</v>
+      </c>
+      <c r="T324" s="6" t="s">
+        <v>680</v>
+      </c>
+      <c r="U324" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="V324" s="5">
+        <v>46198</v>
+      </c>
+      <c r="W324" s="9" t="s">
+        <v>670</v>
+      </c>
+      <c r="X324" s="6">
+        <v>1</v>
+      </c>
+      <c r="Y324" s="6"/>
+    </row>
+    <row r="325" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A325" s="10" t="s">
+        <v>683</v>
+      </c>
+      <c r="B325" s="11">
+        <v>46209.69925508102</v>
+      </c>
+      <c r="C325" s="11">
+        <v>46209.69925484953</v>
+      </c>
+      <c r="D325" s="11">
+        <v>46209.69990349537</v>
+      </c>
+      <c r="E325" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="F325" s="12" t="s">
+        <v>684</v>
+      </c>
+      <c r="G325" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="H325" s="12"/>
+      <c r="I325" s="12"/>
+      <c r="J325" s="11">
+        <v>46197</v>
+      </c>
+      <c r="K325" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="L325" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="M325" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N325" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="O325" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="P325" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q325" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="R325" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S325" s="12" t="s">
+        <v>685</v>
+      </c>
+      <c r="T325" s="12" t="s">
+        <v>686</v>
+      </c>
+      <c r="U325" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="V325" s="11">
+        <v>46198</v>
+      </c>
+      <c r="W325" s="9" t="s">
+        <v>686</v>
+      </c>
+      <c r="X325" s="12">
+        <v>1</v>
+      </c>
+      <c r="Y325" s="12"/>
+    </row>
+    <row r="326" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A326" s="4" t="s">
+        <v>687</v>
+      </c>
+      <c r="B326" s="5">
+        <v>46209.69926057871</v>
+      </c>
+      <c r="C326" s="5">
+        <v>46209.69926055556</v>
+      </c>
+      <c r="D326" s="5">
+        <v>46209.69990407408</v>
+      </c>
+      <c r="E326" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="F326" s="6" t="s">
+        <v>684</v>
+      </c>
+      <c r="G326" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H326" s="6"/>
+      <c r="I326" s="6"/>
+      <c r="J326" s="5">
+        <v>46197</v>
+      </c>
+      <c r="K326" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="L326" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="M326" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N326" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="O326" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="P326" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q326" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="R326" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S326" s="6" t="s">
+        <v>685</v>
+      </c>
+      <c r="T326" s="6" t="s">
+        <v>686</v>
+      </c>
+      <c r="U326" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="V326" s="5">
+        <v>46198</v>
+      </c>
+      <c r="W326" s="9" t="s">
+        <v>686</v>
+      </c>
+      <c r="X326" s="6">
+        <v>1</v>
+      </c>
+      <c r="Y326" s="6"/>
+    </row>
+    <row r="327" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A327" s="10" t="s">
+        <v>688</v>
+      </c>
+      <c r="B327" s="11">
+        <v>46209.69927488426</v>
+      </c>
+      <c r="C327" s="11">
+        <v>46209.69927459491</v>
+      </c>
+      <c r="D327" s="11">
+        <v>46209.69990465278</v>
+      </c>
+      <c r="E327" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="F327" s="12" t="s">
+        <v>684</v>
+      </c>
+      <c r="G327" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="H327" s="12"/>
+      <c r="I327" s="12"/>
+      <c r="J327" s="11">
+        <v>46197</v>
+      </c>
+      <c r="K327" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="L327" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="M327" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N327" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="O327" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="P327" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q327" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="R327" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S327" s="12" t="s">
+        <v>685</v>
+      </c>
+      <c r="T327" s="12" t="s">
+        <v>686</v>
+      </c>
+      <c r="U327" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="V327" s="11">
+        <v>46198</v>
+      </c>
+      <c r="W327" s="9" t="s">
+        <v>686</v>
+      </c>
+      <c r="X327" s="12">
+        <v>1</v>
+      </c>
+      <c r="Y327" s="12"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Actualizar dashboard Oferta Zitron 2026 2026-07-09 20:41 UTC
</commit_message>
<xml_diff>
--- a/data_ofertas/Oferta Zitron 2026.xlsx
+++ b/data_ofertas/Oferta Zitron 2026.xlsx
@@ -24899,9 +24899,11 @@
       <c r="B316" s="5">
         <v>46209.59653997685</v>
       </c>
-      <c r="C316" s="6"/>
+      <c r="C316" s="5">
+        <v>46212.643280439814</v>
+      </c>
       <c r="D316" s="5">
-        <v>46209.86391932871</v>
+        <v>46212.643438125</v>
       </c>
       <c r="E316" s="6" t="s">
         <v>40</v>
@@ -24952,10 +24954,12 @@
       <c r="U316" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="V316" s="6"/>
+      <c r="V316" s="5">
+        <v>46211</v>
+      </c>
       <c r="W316" s="6"/>
       <c r="X316" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y316" s="6"/>
     </row>
@@ -24966,9 +24970,11 @@
       <c r="B317" s="11">
         <v>46209.596545925924</v>
       </c>
-      <c r="C317" s="12"/>
+      <c r="C317" s="11">
+        <v>46212.6433216088</v>
+      </c>
       <c r="D317" s="11">
-        <v>46209.863919490745</v>
+        <v>46212.64359856481</v>
       </c>
       <c r="E317" s="12" t="s">
         <v>83</v>
@@ -25019,10 +25025,12 @@
       <c r="U317" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="V317" s="12"/>
+      <c r="V317" s="11">
+        <v>46211</v>
+      </c>
       <c r="W317" s="12"/>
       <c r="X317" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y317" s="12"/>
     </row>
@@ -25033,9 +25041,11 @@
       <c r="B318" s="5">
         <v>46209.59655829861</v>
       </c>
-      <c r="C318" s="6"/>
+      <c r="C318" s="5">
+        <v>46212.64336990741</v>
+      </c>
       <c r="D318" s="5">
-        <v>46209.86391960648</v>
+        <v>46212.6436378588</v>
       </c>
       <c r="E318" s="6" t="s">
         <v>153</v>
@@ -25086,10 +25096,12 @@
       <c r="U318" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="V318" s="6"/>
+      <c r="V318" s="5">
+        <v>46211</v>
+      </c>
       <c r="W318" s="6"/>
       <c r="X318" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y318" s="6"/>
     </row>

</xml_diff>

<commit_message>
Actualizar dashboard Oferta Zitron 2026 2026-07-14 15:03 UTC
</commit_message>
<xml_diff>
--- a/data_ofertas/Oferta Zitron 2026.xlsx
+++ b/data_ofertas/Oferta Zitron 2026.xlsx
@@ -17311,9 +17311,11 @@
       <c r="B208" s="5">
         <v>46166.90221321759</v>
       </c>
-      <c r="C208" s="6"/>
+      <c r="C208" s="5">
+        <v>46217.59123023148</v>
+      </c>
       <c r="D208" s="5">
-        <v>46210.803671435184</v>
+        <v>46217.59128807871</v>
       </c>
       <c r="E208" s="6" t="s">
         <v>40</v>
@@ -17364,7 +17366,9 @@
       <c r="U208" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="V208" s="6"/>
+      <c r="V208" s="5">
+        <v>46217</v>
+      </c>
       <c r="W208" s="9" t="s">
         <v>460</v>
       </c>
@@ -17451,7 +17455,7 @@
       </c>
       <c r="C210" s="6"/>
       <c r="D210" s="5">
-        <v>46188.845834340274</v>
+        <v>46217.591239166664</v>
       </c>
       <c r="E210" s="6" t="s">
         <v>153</v>

</xml_diff>

<commit_message>
Actualizar dashboard Oferta Zitron 2026 2026-07-14 20:12 UTC
</commit_message>
<xml_diff>
--- a/data_ofertas/Oferta Zitron 2026.xlsx
+++ b/data_ofertas/Oferta Zitron 2026.xlsx
@@ -20704,9 +20704,11 @@
       <c r="B255" s="11">
         <v>46181.55896603009</v>
       </c>
-      <c r="C255" s="12"/>
+      <c r="C255" s="11">
+        <v>46217.78937728009</v>
+      </c>
       <c r="D255" s="11">
-        <v>46191.56176628472</v>
+        <v>46217.78948644676</v>
       </c>
       <c r="E255" s="12" t="s">
         <v>153</v>
@@ -20757,7 +20759,9 @@
       <c r="U255" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="V255" s="12"/>
+      <c r="V255" s="11">
+        <v>46217</v>
+      </c>
       <c r="W255" s="9" t="s">
         <v>553</v>
       </c>

</xml_diff>

<commit_message>
Actualizar dashboard Oferta Zitron 2026 2026-07-15 20:09 UTC
</commit_message>
<xml_diff>
--- a/data_ofertas/Oferta Zitron 2026.xlsx
+++ b/data_ofertas/Oferta Zitron 2026.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5392" uniqueCount="694">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5440" uniqueCount="701">
   <si>
     <t>Oferta Zitron 2026</t>
   </si>
@@ -2094,6 +2094,27 @@
   </si>
   <si>
     <t>1216309407658435</t>
+  </si>
+  <si>
+    <t>1216608715081803</t>
+  </si>
+  <si>
+    <t>26CL0071 - FRECIA COTIZACIÓN IC 3-5412</t>
+  </si>
+  <si>
+    <t>AVO02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26CL0071 </t>
+  </si>
+  <si>
+    <t>1216608989328665</t>
+  </si>
+  <si>
+    <t>1216608775865830</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26CL0071  </t>
   </si>
 </sst>
 </file>
@@ -2617,7 +2638,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Y330"/>
+  <dimension ref="A1:Y333"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10.4" customWidth="1"/>
@@ -14331,9 +14352,11 @@
       <c r="B166" s="5">
         <v>46209.86201597222</v>
       </c>
-      <c r="C166" s="6"/>
+      <c r="C166" s="5">
+        <v>46218.827997858796</v>
+      </c>
       <c r="D166" s="5">
-        <v>46209.862682129635</v>
+        <v>46218.82816923611</v>
       </c>
       <c r="E166" s="6" t="s">
         <v>40</v>
@@ -14373,7 +14396,7 @@
         <v>380</v>
       </c>
       <c r="R166" s="7" t="s">
-        <v>332</v>
+        <v>35</v>
       </c>
       <c r="S166" s="6" t="s">
         <v>369</v>
@@ -14384,12 +14407,14 @@
       <c r="U166" s="8" t="s">
         <v>291</v>
       </c>
-      <c r="V166" s="6"/>
+      <c r="V166" s="5">
+        <v>46216</v>
+      </c>
       <c r="W166" s="9" t="s">
         <v>375</v>
       </c>
       <c r="X166" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y166" s="6"/>
     </row>
@@ -14402,7 +14427,7 @@
       </c>
       <c r="C167" s="12"/>
       <c r="D167" s="11">
-        <v>46209.86268276621</v>
+        <v>46218.82818503473</v>
       </c>
       <c r="E167" s="12" t="s">
         <v>83</v>
@@ -14442,7 +14467,7 @@
         <v>380</v>
       </c>
       <c r="R167" s="7" t="s">
-        <v>332</v>
+        <v>35</v>
       </c>
       <c r="S167" s="12" t="s">
         <v>369</v>
@@ -14471,7 +14496,7 @@
       </c>
       <c r="C168" s="6"/>
       <c r="D168" s="5">
-        <v>46209.86268346065</v>
+        <v>46218.82819986111</v>
       </c>
       <c r="E168" s="6" t="s">
         <v>153</v>
@@ -14511,7 +14536,7 @@
         <v>380</v>
       </c>
       <c r="R168" s="7" t="s">
-        <v>332</v>
+        <v>35</v>
       </c>
       <c r="S168" s="6" t="s">
         <v>369</v>
@@ -21559,9 +21584,11 @@
       <c r="B268" s="5">
         <v>46185.56558032407</v>
       </c>
-      <c r="C268" s="6"/>
+      <c r="C268" s="5">
+        <v>46218.816941516205</v>
+      </c>
       <c r="D268" s="5">
-        <v>46188.70039008102</v>
+        <v>46218.81704105324</v>
       </c>
       <c r="E268" s="6" t="s">
         <v>40</v>
@@ -21612,12 +21639,14 @@
       <c r="U268" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="V268" s="6"/>
+      <c r="V268" s="5">
+        <v>46218</v>
+      </c>
       <c r="W268" s="9" t="s">
         <v>580</v>
       </c>
       <c r="X268" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y268" s="6"/>
     </row>
@@ -21701,9 +21730,11 @@
       <c r="B270" s="5">
         <v>46185.56559773148</v>
       </c>
-      <c r="C270" s="6"/>
+      <c r="C270" s="5">
+        <v>46218.817000462965</v>
+      </c>
       <c r="D270" s="5">
-        <v>46188.61571253472</v>
+        <v>46218.81706912037</v>
       </c>
       <c r="E270" s="6" t="s">
         <v>153</v>
@@ -21754,12 +21785,14 @@
       <c r="U270" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="V270" s="6"/>
+      <c r="V270" s="5">
+        <v>46218</v>
+      </c>
       <c r="W270" s="9" t="s">
         <v>580</v>
       </c>
       <c r="X270" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y270" s="6"/>
     </row>
@@ -25331,7 +25364,7 @@
         <v>46209.67579587963</v>
       </c>
       <c r="D322" s="5">
-        <v>46209.675797523145</v>
+        <v>46218.819764201384</v>
       </c>
       <c r="E322" s="6" t="s">
         <v>40</v>
@@ -25364,10 +25397,10 @@
         <v>153</v>
       </c>
       <c r="Q322" s="7" t="s">
-        <v>332</v>
+        <v>320</v>
       </c>
       <c r="R322" s="7" t="s">
-        <v>332</v>
+        <v>35</v>
       </c>
       <c r="S322" s="6" t="s">
         <v>674</v>
@@ -25400,7 +25433,7 @@
         <v>46209.67580091435</v>
       </c>
       <c r="D323" s="11">
-        <v>46209.675802453705</v>
+        <v>46218.81976479167</v>
       </c>
       <c r="E323" s="12" t="s">
         <v>83</v>
@@ -25433,10 +25466,10 @@
         <v>153</v>
       </c>
       <c r="Q323" s="7" t="s">
-        <v>332</v>
+        <v>320</v>
       </c>
       <c r="R323" s="7" t="s">
-        <v>332</v>
+        <v>35</v>
       </c>
       <c r="S323" s="12" t="s">
         <v>674</v>
@@ -25469,7 +25502,7 @@
         <v>46209.67538987269</v>
       </c>
       <c r="D324" s="5">
-        <v>46209.67580704861</v>
+        <v>46218.81976530093</v>
       </c>
       <c r="E324" s="6" t="s">
         <v>153</v>
@@ -25502,10 +25535,10 @@
         <v>32</v>
       </c>
       <c r="Q324" s="7" t="s">
-        <v>332</v>
+        <v>320</v>
       </c>
       <c r="R324" s="7" t="s">
-        <v>332</v>
+        <v>35</v>
       </c>
       <c r="S324" s="6" t="s">
         <v>674</v>
@@ -25952,6 +25985,213 @@
         <v>1</v>
       </c>
       <c r="Y330" s="6"/>
+    </row>
+    <row r="331" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A331" s="10" t="s">
+        <v>694</v>
+      </c>
+      <c r="B331" s="11">
+        <v>46218.81907759259</v>
+      </c>
+      <c r="C331" s="12"/>
+      <c r="D331" s="11">
+        <v>46218.82098853009</v>
+      </c>
+      <c r="E331" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="F331" s="12" t="s">
+        <v>695</v>
+      </c>
+      <c r="G331" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="H331" s="12"/>
+      <c r="I331" s="12"/>
+      <c r="J331" s="11">
+        <v>46217</v>
+      </c>
+      <c r="K331" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="L331" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="M331" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N331" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="O331" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="P331" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q331" s="7" t="s">
+        <v>380</v>
+      </c>
+      <c r="R331" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S331" s="12" t="s">
+        <v>696</v>
+      </c>
+      <c r="T331" s="12" t="s">
+        <v>697</v>
+      </c>
+      <c r="U331" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="V331" s="11">
+        <v>46198</v>
+      </c>
+      <c r="W331" s="9" t="s">
+        <v>697</v>
+      </c>
+      <c r="X331" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y331" s="12"/>
+    </row>
+    <row r="332" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A332" s="4" t="s">
+        <v>698</v>
+      </c>
+      <c r="B332" s="5">
+        <v>46218.81909099537</v>
+      </c>
+      <c r="C332" s="6"/>
+      <c r="D332" s="5">
+        <v>46218.82098917824</v>
+      </c>
+      <c r="E332" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="F332" s="6" t="s">
+        <v>695</v>
+      </c>
+      <c r="G332" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H332" s="6"/>
+      <c r="I332" s="6"/>
+      <c r="J332" s="5">
+        <v>46217</v>
+      </c>
+      <c r="K332" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="L332" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="M332" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N332" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="O332" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="P332" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q332" s="7" t="s">
+        <v>380</v>
+      </c>
+      <c r="R332" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S332" s="6" t="s">
+        <v>696</v>
+      </c>
+      <c r="T332" s="6" t="s">
+        <v>697</v>
+      </c>
+      <c r="U332" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="V332" s="5">
+        <v>46198</v>
+      </c>
+      <c r="W332" s="9" t="s">
+        <v>697</v>
+      </c>
+      <c r="X332" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y332" s="6"/>
+    </row>
+    <row r="333" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A333" s="10" t="s">
+        <v>699</v>
+      </c>
+      <c r="B333" s="11">
+        <v>46218.81909650463</v>
+      </c>
+      <c r="C333" s="12"/>
+      <c r="D333" s="11">
+        <v>46218.82098978009</v>
+      </c>
+      <c r="E333" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="F333" s="12" t="s">
+        <v>695</v>
+      </c>
+      <c r="G333" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="H333" s="12"/>
+      <c r="I333" s="12"/>
+      <c r="J333" s="11">
+        <v>46217</v>
+      </c>
+      <c r="K333" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="L333" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="M333" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N333" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="O333" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="P333" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q333" s="7" t="s">
+        <v>380</v>
+      </c>
+      <c r="R333" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S333" s="12" t="s">
+        <v>696</v>
+      </c>
+      <c r="T333" s="12" t="s">
+        <v>700</v>
+      </c>
+      <c r="U333" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="V333" s="11">
+        <v>46198</v>
+      </c>
+      <c r="W333" s="9" t="s">
+        <v>697</v>
+      </c>
+      <c r="X333" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y333" s="12"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Actualizar dashboard Oferta Zitron 2026 2026-07-15 20:49 UTC
</commit_message>
<xml_diff>
--- a/data_ofertas/Oferta Zitron 2026.xlsx
+++ b/data_ofertas/Oferta Zitron 2026.xlsx
@@ -21450,9 +21450,11 @@
       <c r="B266" s="5">
         <v>46185.55687354167</v>
       </c>
-      <c r="C266" s="6"/>
+      <c r="C266" s="5">
+        <v>46218.85385309027</v>
+      </c>
       <c r="D266" s="5">
-        <v>46203.54554041667</v>
+        <v>46218.8540481713</v>
       </c>
       <c r="E266" s="6" t="s">
         <v>83</v>
@@ -21501,12 +21503,14 @@
       <c r="U266" s="8" t="s">
         <v>291</v>
       </c>
-      <c r="V266" s="6"/>
+      <c r="V266" s="5">
+        <v>46216</v>
+      </c>
       <c r="W266" s="9" t="s">
         <v>574</v>
       </c>
       <c r="X266" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y266" s="6"/>
     </row>
@@ -21519,7 +21523,7 @@
       </c>
       <c r="C267" s="12"/>
       <c r="D267" s="11">
-        <v>46203.545551435185</v>
+        <v>46218.85385918981</v>
       </c>
       <c r="E267" s="12" t="s">
         <v>153</v>

</xml_diff>

<commit_message>
Actualizar dashboard Oferta Zitron 2026 2026-08-11 20:00 UTC
</commit_message>
<xml_diff>
--- a/data_ofertas/Oferta Zitron 2026.xlsx
+++ b/data_ofertas/Oferta Zitron 2026.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5488" uniqueCount="707">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5732" uniqueCount="740">
   <si>
     <t>Oferta Zitron 2026</t>
   </si>
@@ -2133,6 +2133,105 @@
   </si>
   <si>
     <t xml:space="preserve">26CL0071  </t>
+  </si>
+  <si>
+    <t>1217375038871328</t>
+  </si>
+  <si>
+    <t>26PE0024 - EQUIPO NUEVO CIA MINERA CHUNGAR_OC_4800001063.PDF</t>
+  </si>
+  <si>
+    <t>MINERA CHUNGAR</t>
+  </si>
+  <si>
+    <t>26PE0024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26PE0024 </t>
+  </si>
+  <si>
+    <t>1217375223871379</t>
+  </si>
+  <si>
+    <t>1217374997322161</t>
+  </si>
+  <si>
+    <t>1217375040992791</t>
+  </si>
+  <si>
+    <t>26CL0072 - URGENTE RFQ 6000152191 ZITRON</t>
+  </si>
+  <si>
+    <t>Lunding Mining</t>
+  </si>
+  <si>
+    <t>26CL0072</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26CL0072 </t>
+  </si>
+  <si>
+    <t>1217375313139452</t>
+  </si>
+  <si>
+    <t>1217375313062598</t>
+  </si>
+  <si>
+    <t>1217376604100336</t>
+  </si>
+  <si>
+    <t>26VE0005 - quipos de ventilación Zitron / Minerven</t>
+  </si>
+  <si>
+    <t>Minerven</t>
+  </si>
+  <si>
+    <t>26VE0005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26VE0005 </t>
+  </si>
+  <si>
+    <t>1217376840503494</t>
+  </si>
+  <si>
+    <t>1217376604430272</t>
+  </si>
+  <si>
+    <t>1217377064132073</t>
+  </si>
+  <si>
+    <t>26VE0005.b - quipos de ventilación Zitron / Minerven</t>
+  </si>
+  <si>
+    <t>26VE0005.b</t>
+  </si>
+  <si>
+    <t>26VE0005 .b</t>
+  </si>
+  <si>
+    <t>1217376996944695</t>
+  </si>
+  <si>
+    <t>1217376902114761</t>
+  </si>
+  <si>
+    <t>1217377135826160</t>
+  </si>
+  <si>
+    <t>26MX0067 - Sabinas Presupuesto 2027</t>
+  </si>
+  <si>
+    <t>26MX0067</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26MX0067 </t>
+  </si>
+  <si>
+    <t>1217377264867545</t>
+  </si>
+  <si>
+    <t>1217377264582215</t>
   </si>
 </sst>
 </file>
@@ -2656,7 +2755,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Y336"/>
+  <dimension ref="A1:Y351"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10.4" customWidth="1"/>
@@ -26416,6 +26515,1059 @@
       </c>
       <c r="Y336" s="6"/>
     </row>
+    <row r="337" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A337" s="10" t="s">
+        <v>707</v>
+      </c>
+      <c r="B337" s="11">
+        <v>46245.67044696759</v>
+      </c>
+      <c r="C337" s="12"/>
+      <c r="D337" s="11">
+        <v>46245.67186607639</v>
+      </c>
+      <c r="E337" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="F337" s="12" t="s">
+        <v>708</v>
+      </c>
+      <c r="G337" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H337" s="12"/>
+      <c r="I337" s="11">
+        <v>46217</v>
+      </c>
+      <c r="J337" s="11">
+        <v>46217</v>
+      </c>
+      <c r="K337" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="L337" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="M337" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N337" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="O337" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="P337" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q337" s="7" t="s">
+        <v>385</v>
+      </c>
+      <c r="R337" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="S337" s="12" t="s">
+        <v>709</v>
+      </c>
+      <c r="T337" s="12" t="s">
+        <v>710</v>
+      </c>
+      <c r="U337" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="V337" s="12"/>
+      <c r="W337" s="9" t="s">
+        <v>711</v>
+      </c>
+      <c r="X337" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y337" s="12"/>
+    </row>
+    <row r="338" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A338" s="4" t="s">
+        <v>712</v>
+      </c>
+      <c r="B338" s="5">
+        <v>46245.670453136576</v>
+      </c>
+      <c r="C338" s="6"/>
+      <c r="D338" s="5">
+        <v>46245.67186644676</v>
+      </c>
+      <c r="E338" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F338" s="6" t="s">
+        <v>708</v>
+      </c>
+      <c r="G338" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="H338" s="6"/>
+      <c r="I338" s="5">
+        <v>46217</v>
+      </c>
+      <c r="J338" s="5">
+        <v>46217</v>
+      </c>
+      <c r="K338" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="L338" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="M338" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N338" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="O338" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="P338" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q338" s="7" t="s">
+        <v>385</v>
+      </c>
+      <c r="R338" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="S338" s="6" t="s">
+        <v>709</v>
+      </c>
+      <c r="T338" s="6" t="s">
+        <v>710</v>
+      </c>
+      <c r="U338" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="V338" s="6"/>
+      <c r="W338" s="9" t="s">
+        <v>711</v>
+      </c>
+      <c r="X338" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y338" s="6"/>
+    </row>
+    <row r="339" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A339" s="10" t="s">
+        <v>713</v>
+      </c>
+      <c r="B339" s="11">
+        <v>46245.670467337965</v>
+      </c>
+      <c r="C339" s="12"/>
+      <c r="D339" s="11">
+        <v>46245.67186685185</v>
+      </c>
+      <c r="E339" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="F339" s="12" t="s">
+        <v>708</v>
+      </c>
+      <c r="G339" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H339" s="12"/>
+      <c r="I339" s="11">
+        <v>46217</v>
+      </c>
+      <c r="J339" s="11">
+        <v>46217</v>
+      </c>
+      <c r="K339" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="L339" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="M339" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N339" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="O339" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="P339" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q339" s="7" t="s">
+        <v>385</v>
+      </c>
+      <c r="R339" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="S339" s="12" t="s">
+        <v>709</v>
+      </c>
+      <c r="T339" s="12" t="s">
+        <v>710</v>
+      </c>
+      <c r="U339" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="V339" s="12"/>
+      <c r="W339" s="9" t="s">
+        <v>711</v>
+      </c>
+      <c r="X339" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y339" s="12"/>
+    </row>
+    <row r="340" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A340" s="4" t="s">
+        <v>714</v>
+      </c>
+      <c r="B340" s="5">
+        <v>46245.672699166666</v>
+      </c>
+      <c r="C340" s="5">
+        <v>46245.676609421294</v>
+      </c>
+      <c r="D340" s="5">
+        <v>46245.67681689815</v>
+      </c>
+      <c r="E340" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="F340" s="6" t="s">
+        <v>715</v>
+      </c>
+      <c r="G340" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H340" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="I340" s="5">
+        <v>46217</v>
+      </c>
+      <c r="J340" s="5">
+        <v>46217</v>
+      </c>
+      <c r="K340" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="L340" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="M340" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N340" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="O340" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="P340" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q340" s="7" t="s">
+        <v>385</v>
+      </c>
+      <c r="R340" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="S340" s="6" t="s">
+        <v>716</v>
+      </c>
+      <c r="T340" s="6" t="s">
+        <v>717</v>
+      </c>
+      <c r="U340" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="V340" s="5">
+        <v>46224</v>
+      </c>
+      <c r="W340" s="9" t="s">
+        <v>718</v>
+      </c>
+      <c r="X340" s="6">
+        <v>1</v>
+      </c>
+      <c r="Y340" s="6"/>
+    </row>
+    <row r="341" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A341" s="10" t="s">
+        <v>719</v>
+      </c>
+      <c r="B341" s="11">
+        <v>46245.67270501157</v>
+      </c>
+      <c r="C341" s="12"/>
+      <c r="D341" s="11">
+        <v>46245.67611371528</v>
+      </c>
+      <c r="E341" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="F341" s="12" t="s">
+        <v>715</v>
+      </c>
+      <c r="G341" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H341" s="12"/>
+      <c r="I341" s="11">
+        <v>46217</v>
+      </c>
+      <c r="J341" s="11">
+        <v>46217</v>
+      </c>
+      <c r="K341" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="L341" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="M341" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N341" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="O341" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="P341" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q341" s="7" t="s">
+        <v>385</v>
+      </c>
+      <c r="R341" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="S341" s="12" t="s">
+        <v>716</v>
+      </c>
+      <c r="T341" s="12" t="s">
+        <v>717</v>
+      </c>
+      <c r="U341" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="V341" s="12"/>
+      <c r="W341" s="9" t="s">
+        <v>718</v>
+      </c>
+      <c r="X341" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y341" s="12"/>
+    </row>
+    <row r="342" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A342" s="4" t="s">
+        <v>720</v>
+      </c>
+      <c r="B342" s="5">
+        <v>46245.67272284722</v>
+      </c>
+      <c r="C342" s="6"/>
+      <c r="D342" s="5">
+        <v>46245.67661574074</v>
+      </c>
+      <c r="E342" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F342" s="6" t="s">
+        <v>715</v>
+      </c>
+      <c r="G342" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="H342" s="6"/>
+      <c r="I342" s="5">
+        <v>46217</v>
+      </c>
+      <c r="J342" s="5">
+        <v>46217</v>
+      </c>
+      <c r="K342" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="L342" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="M342" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N342" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="O342" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P342" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q342" s="7" t="s">
+        <v>385</v>
+      </c>
+      <c r="R342" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="S342" s="6" t="s">
+        <v>716</v>
+      </c>
+      <c r="T342" s="6" t="s">
+        <v>717</v>
+      </c>
+      <c r="U342" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="V342" s="6"/>
+      <c r="W342" s="9" t="s">
+        <v>718</v>
+      </c>
+      <c r="X342" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y342" s="6"/>
+    </row>
+    <row r="343" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A343" s="10" t="s">
+        <v>721</v>
+      </c>
+      <c r="B343" s="11">
+        <v>46245.69379331019</v>
+      </c>
+      <c r="C343" s="12"/>
+      <c r="D343" s="11">
+        <v>46245.69473616898</v>
+      </c>
+      <c r="E343" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="F343" s="12" t="s">
+        <v>722</v>
+      </c>
+      <c r="G343" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H343" s="12"/>
+      <c r="I343" s="11">
+        <v>46220</v>
+      </c>
+      <c r="J343" s="11">
+        <v>46220</v>
+      </c>
+      <c r="K343" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="L343" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="M343" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N343" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="O343" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="P343" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q343" s="7" t="s">
+        <v>385</v>
+      </c>
+      <c r="R343" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="S343" s="12" t="s">
+        <v>723</v>
+      </c>
+      <c r="T343" s="12" t="s">
+        <v>724</v>
+      </c>
+      <c r="U343" s="8" t="s">
+        <v>515</v>
+      </c>
+      <c r="V343" s="12"/>
+      <c r="W343" s="9" t="s">
+        <v>725</v>
+      </c>
+      <c r="X343" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y343" s="12"/>
+    </row>
+    <row r="344" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A344" s="4" t="s">
+        <v>726</v>
+      </c>
+      <c r="B344" s="5">
+        <v>46245.6937994676</v>
+      </c>
+      <c r="C344" s="6"/>
+      <c r="D344" s="5">
+        <v>46245.694736516205</v>
+      </c>
+      <c r="E344" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F344" s="6" t="s">
+        <v>722</v>
+      </c>
+      <c r="G344" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="H344" s="6"/>
+      <c r="I344" s="5">
+        <v>46220</v>
+      </c>
+      <c r="J344" s="5">
+        <v>46220</v>
+      </c>
+      <c r="K344" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="L344" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="M344" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N344" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="O344" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="P344" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q344" s="7" t="s">
+        <v>385</v>
+      </c>
+      <c r="R344" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="S344" s="6" t="s">
+        <v>723</v>
+      </c>
+      <c r="T344" s="6" t="s">
+        <v>724</v>
+      </c>
+      <c r="U344" s="8" t="s">
+        <v>515</v>
+      </c>
+      <c r="V344" s="6"/>
+      <c r="W344" s="9" t="s">
+        <v>725</v>
+      </c>
+      <c r="X344" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y344" s="6"/>
+    </row>
+    <row r="345" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A345" s="10" t="s">
+        <v>727</v>
+      </c>
+      <c r="B345" s="11">
+        <v>46245.69381340277</v>
+      </c>
+      <c r="C345" s="12"/>
+      <c r="D345" s="11">
+        <v>46245.69473690972</v>
+      </c>
+      <c r="E345" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="F345" s="12" t="s">
+        <v>722</v>
+      </c>
+      <c r="G345" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H345" s="12"/>
+      <c r="I345" s="11">
+        <v>46220</v>
+      </c>
+      <c r="J345" s="11">
+        <v>46220</v>
+      </c>
+      <c r="K345" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="L345" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="M345" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N345" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="O345" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="P345" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q345" s="7" t="s">
+        <v>385</v>
+      </c>
+      <c r="R345" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="S345" s="12" t="s">
+        <v>723</v>
+      </c>
+      <c r="T345" s="12" t="s">
+        <v>724</v>
+      </c>
+      <c r="U345" s="8" t="s">
+        <v>515</v>
+      </c>
+      <c r="V345" s="12"/>
+      <c r="W345" s="9" t="s">
+        <v>725</v>
+      </c>
+      <c r="X345" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y345" s="12"/>
+    </row>
+    <row r="346" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A346" s="4" t="s">
+        <v>728</v>
+      </c>
+      <c r="B346" s="5">
+        <v>46245.69833460648</v>
+      </c>
+      <c r="C346" s="6"/>
+      <c r="D346" s="5">
+        <v>46245.69905877315</v>
+      </c>
+      <c r="E346" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="F346" s="6" t="s">
+        <v>729</v>
+      </c>
+      <c r="G346" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="H346" s="6"/>
+      <c r="I346" s="6"/>
+      <c r="J346" s="5">
+        <v>46220</v>
+      </c>
+      <c r="K346" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="L346" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="M346" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N346" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="O346" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="P346" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q346" s="7" t="s">
+        <v>385</v>
+      </c>
+      <c r="R346" s="7" t="s">
+        <v>337</v>
+      </c>
+      <c r="S346" s="6" t="s">
+        <v>723</v>
+      </c>
+      <c r="T346" s="6" t="s">
+        <v>730</v>
+      </c>
+      <c r="U346" s="8" t="s">
+        <v>515</v>
+      </c>
+      <c r="V346" s="6"/>
+      <c r="W346" s="9" t="s">
+        <v>731</v>
+      </c>
+      <c r="X346" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y346" s="6"/>
+    </row>
+    <row r="347" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A347" s="10" t="s">
+        <v>732</v>
+      </c>
+      <c r="B347" s="11">
+        <v>46245.69833921296</v>
+      </c>
+      <c r="C347" s="12"/>
+      <c r="D347" s="11">
+        <v>46245.69905914352</v>
+      </c>
+      <c r="E347" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="F347" s="12" t="s">
+        <v>729</v>
+      </c>
+      <c r="G347" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H347" s="12"/>
+      <c r="I347" s="12"/>
+      <c r="J347" s="11">
+        <v>46220</v>
+      </c>
+      <c r="K347" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="L347" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="M347" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N347" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="O347" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="P347" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q347" s="7" t="s">
+        <v>385</v>
+      </c>
+      <c r="R347" s="7" t="s">
+        <v>337</v>
+      </c>
+      <c r="S347" s="12" t="s">
+        <v>723</v>
+      </c>
+      <c r="T347" s="12" t="s">
+        <v>730</v>
+      </c>
+      <c r="U347" s="8" t="s">
+        <v>515</v>
+      </c>
+      <c r="V347" s="12"/>
+      <c r="W347" s="9" t="s">
+        <v>731</v>
+      </c>
+      <c r="X347" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y347" s="12"/>
+    </row>
+    <row r="348" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A348" s="4" t="s">
+        <v>733</v>
+      </c>
+      <c r="B348" s="5">
+        <v>46245.69835390046</v>
+      </c>
+      <c r="C348" s="6"/>
+      <c r="D348" s="5">
+        <v>46245.69905947917</v>
+      </c>
+      <c r="E348" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F348" s="6" t="s">
+        <v>729</v>
+      </c>
+      <c r="G348" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="H348" s="6"/>
+      <c r="I348" s="6"/>
+      <c r="J348" s="5">
+        <v>46220</v>
+      </c>
+      <c r="K348" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="L348" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="M348" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N348" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="O348" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P348" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q348" s="7" t="s">
+        <v>385</v>
+      </c>
+      <c r="R348" s="7" t="s">
+        <v>337</v>
+      </c>
+      <c r="S348" s="6" t="s">
+        <v>723</v>
+      </c>
+      <c r="T348" s="6" t="s">
+        <v>730</v>
+      </c>
+      <c r="U348" s="8" t="s">
+        <v>515</v>
+      </c>
+      <c r="V348" s="6"/>
+      <c r="W348" s="9" t="s">
+        <v>731</v>
+      </c>
+      <c r="X348" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y348" s="6"/>
+    </row>
+    <row r="349" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A349" s="10" t="s">
+        <v>734</v>
+      </c>
+      <c r="B349" s="11">
+        <v>46245.70305795139</v>
+      </c>
+      <c r="C349" s="11">
+        <v>46245.70368289352</v>
+      </c>
+      <c r="D349" s="11">
+        <v>46245.70419758101</v>
+      </c>
+      <c r="E349" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="F349" s="12" t="s">
+        <v>735</v>
+      </c>
+      <c r="G349" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="H349" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="I349" s="11">
+        <v>46188</v>
+      </c>
+      <c r="J349" s="11">
+        <v>46188</v>
+      </c>
+      <c r="K349" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="L349" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="M349" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N349" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="O349" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="P349" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q349" s="7" t="s">
+        <v>385</v>
+      </c>
+      <c r="R349" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="S349" s="12" t="s">
+        <v>551</v>
+      </c>
+      <c r="T349" s="12" t="s">
+        <v>736</v>
+      </c>
+      <c r="U349" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="V349" s="11">
+        <v>46218</v>
+      </c>
+      <c r="W349" s="9" t="s">
+        <v>737</v>
+      </c>
+      <c r="X349" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y349" s="12"/>
+    </row>
+    <row r="350" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A350" s="4" t="s">
+        <v>738</v>
+      </c>
+      <c r="B350" s="5">
+        <v>46245.703064375004</v>
+      </c>
+      <c r="C350" s="5">
+        <v>46245.70368362268</v>
+      </c>
+      <c r="D350" s="5">
+        <v>46245.704197997686</v>
+      </c>
+      <c r="E350" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F350" s="6" t="s">
+        <v>735</v>
+      </c>
+      <c r="G350" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H350" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="I350" s="5">
+        <v>46188</v>
+      </c>
+      <c r="J350" s="5">
+        <v>46188</v>
+      </c>
+      <c r="K350" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="L350" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="M350" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N350" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="O350" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="P350" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q350" s="7" t="s">
+        <v>385</v>
+      </c>
+      <c r="R350" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="S350" s="6" t="s">
+        <v>551</v>
+      </c>
+      <c r="T350" s="6" t="s">
+        <v>736</v>
+      </c>
+      <c r="U350" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="V350" s="5">
+        <v>46218</v>
+      </c>
+      <c r="W350" s="9" t="s">
+        <v>737</v>
+      </c>
+      <c r="X350" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y350" s="6"/>
+    </row>
+    <row r="351" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A351" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B351" s="11">
+        <v>46245.703077847225</v>
+      </c>
+      <c r="C351" s="11">
+        <v>46245.70368424768</v>
+      </c>
+      <c r="D351" s="11">
+        <v>46245.704198391206</v>
+      </c>
+      <c r="E351" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="F351" s="12" t="s">
+        <v>735</v>
+      </c>
+      <c r="G351" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="H351" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="I351" s="11">
+        <v>46188</v>
+      </c>
+      <c r="J351" s="11">
+        <v>46188</v>
+      </c>
+      <c r="K351" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="L351" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="M351" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="N351" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="O351" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="P351" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q351" s="7" t="s">
+        <v>385</v>
+      </c>
+      <c r="R351" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="S351" s="12" t="s">
+        <v>551</v>
+      </c>
+      <c r="T351" s="12" t="s">
+        <v>736</v>
+      </c>
+      <c r="U351" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="V351" s="11">
+        <v>46218</v>
+      </c>
+      <c r="W351" s="9" t="s">
+        <v>737</v>
+      </c>
+      <c r="X351" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y351" s="12"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>